<commit_message>
Deployed 37a1cccc6 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -6221,12 +6221,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6236,7 +6236,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6292,17 +6292,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6312,7 +6312,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6331,12 +6331,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6402,17 +6402,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -11715,12 +11715,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11730,7 +11730,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping Project - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11772,16 +11772,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.6286, 48.1332], [-122.8941, 48.1332], [-122.8941, 51.9689], [-128.6286, 51.9689], [-128.6286, 48.1332]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11791,12 +11791,12 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11806,7 +11806,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11817,9 +11817,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X104" t="n">
-        <v>3</v>
-      </c>
+      <c r="X104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11827,12 +11825,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11842,7 +11840,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping Project - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11860,7 +11858,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -11884,16 +11882,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.6286, 48.1332], [-122.8941, 48.1332], [-122.8941, 51.9689], [-128.6286, 51.9689], [-128.6286, 48.1332]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11903,12 +11901,12 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11918,7 +11916,7 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="V105" t="n">
@@ -11929,7 +11927,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X105" t="inlineStr"/>
+      <c r="X105" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -13147,12 +13147,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13162,7 +13162,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13185,7 +13185,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13204,11 +13204,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13223,12 +13223,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13238,7 +13238,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13246,7 +13246,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13257,12 +13257,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13272,7 +13272,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13295,7 +13295,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13314,11 +13314,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13333,12 +13333,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13348,7 +13348,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13356,7 +13356,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -15229,7 +15229,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X135" t="inlineStr"/>
+      <c r="X135" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -16111,7 +16113,9 @@
           <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X143" t="inlineStr"/>
+      <c r="X143" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -16779,12 +16783,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>ca-cioos_cec3dcef-8dba-4d91-aee6-b60ce416497c</t>
+          <t>ca-cioos_c89e35df-8a16-4efc-ae29-15f4e3da8a55</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -16794,7 +16798,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Mussel Dynamics - Point Intercepts - BC Central Coast</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -16850,17 +16854,17 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
         <is>
-          <t>10.21966/ns9h-1126</t>
+          <t>10.21966/0yk3-9b74</t>
         </is>
       </c>
       <c r="S150" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-MotaGdFmX3xEvWjXQA5</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-Motctf2E7ids9V-6Cfb</t>
         </is>
       </c>
       <c r="T150" t="inlineStr">
@@ -16870,7 +16874,7 @@
       </c>
       <c r="U150" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="V150" t="n">
@@ -16889,12 +16893,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>ca-cioos_c89e35df-8a16-4efc-ae29-15f4e3da8a55</t>
+          <t>ca-cioos_cec3dcef-8dba-4d91-aee6-b60ce416497c</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -16904,7 +16908,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast</t>
+          <t>Mussel Dynamics - Point Intercepts - BC Central Coast</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -16960,17 +16964,17 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
         <is>
-          <t>10.21966/0yk3-9b74</t>
+          <t>10.21966/ns9h-1126</t>
         </is>
       </c>
       <c r="S151" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-Motctf2E7ids9V-6Cfb</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-MotaGdFmX3xEvWjXQA5</t>
         </is>
       </c>
       <c r="T151" t="inlineStr">
@@ -16980,7 +16984,7 @@
       </c>
       <c r="U151" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V151" t="n">
@@ -18979,12 +18983,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>75b60436-da51-4ccf-b14a-27f45f782b2b</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>ca-cioos_476204a7-0714-4755-953d-61fa3c5df497</t>
+          <t>ca-cioos_24f1c230-6c37-470c-907d-25b9b022f5c2</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -18994,7 +18998,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Hakai Institute Nutrients (Dosser et al., 2021)</t>
+          <t>Differential infestation of juvenile Pacific salmon by parasitic sea lice in British Columbia, Canada</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -19012,7 +19016,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -19040,27 +19044,27 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.6, 50.69], [-126.3, 50.8], [-124.8, 50.44], [-123.9, 49.65], [-125.1, 49.65], [-127.6, 50.69]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.87477074, 49.80151064], [-124.30109865, 49.80151064], [-124.30109865, 50.66883255], [-126.87477074, 50.66883255], [-126.87477074, 49.80151064]]]}</t>
         </is>
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '9.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>nutrients</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
         <is>
-          <t>10.21966/j3j5-wt70</t>
+          <t>10.21966/54tw-kh93</t>
         </is>
       </c>
       <c r="S170" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/oOseiEWez6TzqPUIisEXczg6G8y2/-MoZtzH-n9LBy9Bn29Hl</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZDeElXT3dpUFNlOGQ</t>
         </is>
       </c>
       <c r="T170" t="inlineStr">
@@ -19070,7 +19074,7 @@
       </c>
       <c r="U170" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V170" t="n">
@@ -19089,12 +19093,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>75b60436-da51-4ccf-b14a-27f45f782b2b</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>ca-cioos_24f1c230-6c37-470c-907d-25b9b022f5c2</t>
+          <t>ca-cioos_476204a7-0714-4755-953d-61fa3c5df497</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -19104,7 +19108,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Differential infestation of juvenile Pacific salmon by parasitic sea lice in British Columbia, Canada</t>
+          <t>Hakai Institute Nutrients (Dosser et al., 2021)</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
@@ -19122,7 +19126,7 @@
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>Juvenile Salmon Program</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -19150,27 +19154,27 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.87477074, 49.80151064], [-124.30109865, 49.80151064], [-124.30109865, 50.66883255], [-126.87477074, 50.66883255], [-126.87477074, 49.80151064]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.6, 50.69], [-126.3, 50.8], [-124.8, 50.44], [-123.9, 49.65], [-125.1, 49.65], [-127.6, 50.69]]]}</t>
         </is>
       </c>
       <c r="P171" t="inlineStr">
         <is>
-          <t>[{'max': '9.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>nutrients</t>
         </is>
       </c>
       <c r="R171" t="inlineStr">
         <is>
-          <t>10.21966/54tw-kh93</t>
+          <t>10.21966/j3j5-wt70</t>
         </is>
       </c>
       <c r="S171" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZDeElXT3dpUFNlOGQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/oOseiEWez6TzqPUIisEXczg6G8y2/-MoZtzH-n9LBy9Bn29Hl</t>
         </is>
       </c>
       <c r="T171" t="inlineStr">
@@ -19180,7 +19184,7 @@
       </c>
       <c r="U171" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="V171" t="n">
@@ -19191,9 +19195,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X171" t="n">
-        <v>1</v>
-      </c>
+      <c r="X171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -24471,9 +24473,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X219" t="n">
-        <v>1</v>
-      </c>
+      <c r="X219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -27874,7 +27874,7 @@
       </c>
       <c r="U250" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="V250" t="n">
@@ -30968,7 +30968,7 @@
         </is>
       </c>
       <c r="X278" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="279">

</xml_diff>

<commit_message>
Deployed ee63adcb9 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X284"/>
+  <dimension ref="A1:X300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6221,12 +6221,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6236,7 +6236,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6292,17 +6292,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6312,7 +6312,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6331,12 +6331,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6402,17 +6402,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -13147,12 +13147,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13162,7 +13162,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13185,7 +13185,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13204,11 +13204,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13223,12 +13223,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13238,7 +13238,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13246,7 +13246,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13257,12 +13257,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -13272,7 +13272,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -13295,7 +13295,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -13314,11 +13314,11 @@
         </is>
       </c>
       <c r="N118" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P118" t="inlineStr">
@@ -13333,12 +13333,12 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S118" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T118" t="inlineStr">
@@ -13348,7 +13348,7 @@
       </c>
       <c r="U118" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V118" t="n">
@@ -13356,7 +13356,7 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
@@ -13477,12 +13477,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13492,7 +13492,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13510,12 +13510,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13534,16 +13534,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13553,12 +13553,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -13587,12 +13587,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -13602,7 +13602,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -13620,12 +13620,12 @@
       </c>
       <c r="I121" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -13644,16 +13644,16 @@
         </is>
       </c>
       <c r="N121" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr">
@@ -13663,12 +13663,12 @@
       </c>
       <c r="R121" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S121" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T121" t="inlineStr">
@@ -15229,9 +15229,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X135" t="n">
-        <v>1</v>
-      </c>
+      <c r="X135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -16113,9 +16111,7 @@
           <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X143" t="n">
-        <v>1</v>
-      </c>
+      <c r="X143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -16783,12 +16779,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>ca-cioos_c89e35df-8a16-4efc-ae29-15f4e3da8a55</t>
+          <t>ca-cioos_cec3dcef-8dba-4d91-aee6-b60ce416497c</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -16798,7 +16794,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast</t>
+          <t>Mussel Dynamics - Point Intercepts - BC Central Coast</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -16854,17 +16850,17 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
         <is>
-          <t>10.21966/0yk3-9b74</t>
+          <t>10.21966/ns9h-1126</t>
         </is>
       </c>
       <c r="S150" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-Motctf2E7ids9V-6Cfb</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-MotaGdFmX3xEvWjXQA5</t>
         </is>
       </c>
       <c r="T150" t="inlineStr">
@@ -16874,7 +16870,7 @@
       </c>
       <c r="U150" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V150" t="n">
@@ -16893,12 +16889,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>ca-cioos_cec3dcef-8dba-4d91-aee6-b60ce416497c</t>
+          <t>ca-cioos_c89e35df-8a16-4efc-ae29-15f4e3da8a55</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -16908,7 +16904,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Mussel Dynamics - Point Intercepts - BC Central Coast</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -16964,17 +16960,17 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
         <is>
-          <t>10.21966/ns9h-1126</t>
+          <t>10.21966/0yk3-9b74</t>
         </is>
       </c>
       <c r="S151" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-MotaGdFmX3xEvWjXQA5</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-Motctf2E7ids9V-6Cfb</t>
         </is>
       </c>
       <c r="T151" t="inlineStr">
@@ -16984,7 +16980,7 @@
       </c>
       <c r="U151" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="V151" t="n">
@@ -30968,7 +30964,7 @@
         </is>
       </c>
       <c r="X278" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="279">
@@ -31411,12 +31407,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
+          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
+          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -31426,7 +31422,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -31472,7 +31468,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
         </is>
       </c>
       <c r="P283" t="inlineStr">
@@ -31487,12 +31483,12 @@
       </c>
       <c r="R283" t="inlineStr">
         <is>
-          <t>10.21966/q2e0-j004</t>
+          <t>10.21966/r9zr-xz33</t>
         </is>
       </c>
       <c r="S283" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
         </is>
       </c>
       <c r="T283" t="inlineStr">
@@ -31502,7 +31498,7 @@
       </c>
       <c r="U283" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="V283" t="n">
@@ -31514,7 +31510,7 @@
         </is>
       </c>
       <c r="X283" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="284">
@@ -31523,12 +31519,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -31538,7 +31534,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -31556,12 +31552,12 @@
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Estuary Resilience</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K284" t="inlineStr">
@@ -31576,7 +31572,7 @@
       </c>
       <c r="M284" t="inlineStr">
         <is>
-          <t>Tula Foundation</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N284" t="n">
@@ -31584,44 +31580,1836 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R284" t="inlineStr">
+        <is>
+          <t>10.21966/9dbb-5d54</t>
+        </is>
+      </c>
+      <c r="S284" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
+        </is>
+      </c>
+      <c r="T284" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U284" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V284" t="n">
+        <v>0</v>
+      </c>
+      <c r="W284" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X284" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>283</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H285" t="b">
+        <v>0</v>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N285" t="n">
+        <v>1</v>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R285" t="inlineStr">
+        <is>
+          <t>10.21966/vpz7-mm73</t>
+        </is>
+      </c>
+      <c r="S285" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
+        </is>
+      </c>
+      <c r="T285" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U285" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V285" t="n">
+        <v>0</v>
+      </c>
+      <c r="W285" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X285" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>284</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>0ce3ee5b-425b-4eb0-a201-96bdfb795a3f</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>ca-cioos_354b5b83-e752-4ffb-a740-d1cdc02ac8c6</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Dtlaxsiwè River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H286" t="b">
+        <v>0</v>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N286" t="n">
+        <v>1</v>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.1721, 50.61011], [-127.17933, 50.612], [-127.1873, 50.6098], [-127.19703, 50.61072], [-127.20524, 50.61585], [-127.19007, 50.61844], [-127.18675, 50.61393], [-127.17744, 50.61359], [-127.17161, 50.61118], [-127.17203, 50.61011], [-127.1721, 50.61011]]]}</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R286" t="inlineStr">
+        <is>
+          <t>10.21966/ydm2-m238</t>
+        </is>
+      </c>
+      <c r="S286" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7Dng-ZtRd05hnZCq1</t>
+        </is>
+      </c>
+      <c r="T286" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U286" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V286" t="n">
+        <v>0</v>
+      </c>
+      <c r="W286" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X286" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>285</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>1a2aa5c8-9a83-46f7-967d-1127436c2084</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>ca-cioos_58a5140a-0b2c-4186-a648-53d9f58e5226</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Kvai River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H287" t="b">
+        <v>0</v>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N287" t="n">
+        <v>1</v>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.81882, 51.77547], [-127.83122, 51.77986], [-127.85192, 51.781], [-127.86785, 51.78358], [-127.8958, 51.77366], [-127.89418, 51.77118], [-127.87834, 51.77309], [-127.86508, 51.77748], [-127.84009, 51.77519], [-127.82731, 51.77452], [-127.82025, 51.77309], [-127.81853, 51.77566], [-127.81882, 51.77547]]]}</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R287" t="inlineStr">
+        <is>
+          <t>10.21966/pm9m-h431</t>
+        </is>
+      </c>
+      <c r="S287" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7QQE3ifLCAPcu3Jih</t>
+        </is>
+      </c>
+      <c r="T287" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U287" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V287" t="n">
+        <v>0</v>
+      </c>
+      <c r="W287" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X287" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>286</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>c035b81c-0fc3-446e-bec5-8b8933ae874b</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>ca-cioos_7fbc28f7-ee87-4361-bbee-0ed8ce24522d</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Gwa'dzi River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H288" t="b">
+        <v>0</v>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N288" t="n">
+        <v>1</v>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.46176, 50.74217], [-127.49022, 50.72165], [-127.49167, 50.71188], [-127.4832, 50.70356], [-127.4874, 50.69181], [-127.46443, 50.6928], [-127.47282, 50.70776], [-127.47992, 50.71424], [-127.48305, 50.72058], [-127.45901, 50.74011], [-127.46153, 50.74217], [-127.46176, 50.74217]]]}</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R288" t="inlineStr">
+        <is>
+          <t>10.21966/xq99-x273</t>
+        </is>
+      </c>
+      <c r="S288" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7BCRnF2C30YPkxIyd</t>
+        </is>
+      </c>
+      <c r="T288" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U288" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V288" t="n">
+        <v>0</v>
+      </c>
+      <c r="W288" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X288" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>287</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H289" t="b">
+        <v>0</v>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N289" t="n">
+        <v>1</v>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>10.21966/kde9-8g12</t>
+        </is>
+      </c>
+      <c r="S289" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
+        </is>
+      </c>
+      <c r="T289" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U289" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V289" t="n">
+        <v>0</v>
+      </c>
+      <c r="W289" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X289" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>288</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H290" t="b">
+        <v>0</v>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N290" t="n">
+        <v>1</v>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>10.21966/9a97-2j48</t>
+        </is>
+      </c>
+      <c r="S290" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
+        </is>
+      </c>
+      <c r="T290" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U290" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V290" t="n">
+        <v>0</v>
+      </c>
+      <c r="W290" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X290" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>289</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H291" t="b">
+        <v>0</v>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N291" t="n">
+        <v>1</v>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R291" t="inlineStr">
+        <is>
+          <t>10.21966/ed9w-2653</t>
+        </is>
+      </c>
+      <c r="S291" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
+        </is>
+      </c>
+      <c r="T291" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U291" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V291" t="n">
+        <v>0</v>
+      </c>
+      <c r="W291" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X291" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>290</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>1af6a43a-e73b-4774-8e10-b9f2928ab133</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>ca-cioos_ae7e017c-9211-4f98-b56e-90a4bbac161c</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Snuneymuxw River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H292" t="b">
+        <v>0</v>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N292" t="n">
+        <v>1</v>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.88685, 49.19332], [-123.92494, 49.1612], [-123.92581, 49.13841], [-123.91159, 49.123], [-123.88023, 49.11117], [-123.85971, 49.12766], [-123.89792, 49.16196], [-123.88099, 49.18866], [-123.88685, 49.19332]]]}</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R292" t="inlineStr">
+        <is>
+          <t>10.21966/k01q-wb27</t>
+        </is>
+      </c>
+      <c r="S292" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt459vxCIH7YPRN9fp</t>
+        </is>
+      </c>
+      <c r="T292" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U292" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V292" t="n">
+        <v>0</v>
+      </c>
+      <c r="W292" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X292" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>291</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>ca-cioos_b922699f-69b6-4d63-b538-7c290086a408</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Quw'utsun/Xwulqw'selu River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H293" t="b">
+        <v>0</v>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N293" t="n">
+        <v>1</v>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.56201, 48.73508], [-123.59772, 48.75559], [-123.62127, 48.76514], [-123.63885, 48.77426], [-123.66935, 48.78033], [-123.67901, 48.75472], [-123.65155, 48.74322], [-123.63017, 48.7405], [-123.60792, 48.74289], [-123.56494, 48.72987], [-123.56179, 48.73529], [-123.56201, 48.73508]]]}</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R293" t="inlineStr">
+        <is>
+          <t>10.21966/2ha7-9p26</t>
+        </is>
+      </c>
+      <c r="S293" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpsCA3ycwZ7bFTDIQxh</t>
+        </is>
+      </c>
+      <c r="T293" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U293" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V293" t="n">
+        <v>0</v>
+      </c>
+      <c r="W293" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X293" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>292</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H294" t="b">
+        <v>0</v>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N294" t="n">
+        <v>1</v>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635], [-123.66843, 48.91641]]]}</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R294" t="inlineStr">
+        <is>
+          <t>10.21966/q2e0-j004</t>
+        </is>
+      </c>
+      <c r="S294" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
+        </is>
+      </c>
+      <c r="T294" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U294" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V294" t="n">
+        <v>0</v>
+      </c>
+      <c r="W294" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X294" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>293</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H295" t="b">
+        <v>0</v>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N295" t="n">
+        <v>1</v>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R295" t="inlineStr">
+        <is>
+          <t>10.21966/hjkj-6611</t>
+        </is>
+      </c>
+      <c r="S295" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
+        </is>
+      </c>
+      <c r="T295" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U295" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V295" t="n">
+        <v>0</v>
+      </c>
+      <c r="W295" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X295" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>294</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>ca-cioos_dce15b7b-3772-4106-ab20-c3979c4c3f57</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Fulmore River - Shoal Creek Estuary Complex (Provisional)</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H296" t="b">
+        <v>0</v>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N296" t="n">
+        <v>1</v>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.08798, 50.4777], [-126.09599, 50.48418], [-126.09046, 50.50918], [-126.0647, 50.52425], [-125.99698, 50.53569], [-125.93459, 50.56717], [-125.93173, 50.56202], [-125.93764, 50.55458], [-125.91055, 50.55134], [-125.89853, 50.54943], [-125.90063, 50.54466], [-125.96416, 50.53989], [-125.98973, 50.52043], [-126.06566, 50.5067], [-126.08779, 50.47789], [-126.08798, 50.4777]]]}</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R296" t="inlineStr">
+        <is>
+          <t>10.21966/g1cn-xs92</t>
+        </is>
+      </c>
+      <c r="S296" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptdJ8iUmLeOrdmqzrQ</t>
+        </is>
+      </c>
+      <c r="T296" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U296" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V296" t="n">
+        <v>0</v>
+      </c>
+      <c r="W296" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X296" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>295</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H297" t="b">
+        <v>0</v>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N297" t="n">
+        <v>1</v>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R297" t="inlineStr">
+        <is>
+          <t>10.21966/npe4-3036</t>
+        </is>
+      </c>
+      <c r="S297" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
+        </is>
+      </c>
+      <c r="T297" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U297" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V297" t="n">
+        <v>0</v>
+      </c>
+      <c r="W297" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X297" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>296</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>ca-cioos_e9b72149-8cf1-4000-ae3e-6b29ad60b078</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Malksope River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H298" t="b">
+        <v>0</v>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N298" t="n">
+        <v>1</v>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.46569, 50.12556], [-127.45723, 50.13142], [-127.43281, 50.13338], [-127.42845, 50.13765], [-127.41181, 50.14408], [-127.40973, 50.14233], [-127.41999, 50.13627], [-127.41803, 50.13195], [-127.43106, 50.12796], [-127.46545, 50.12446], [-127.46569, 50.12548], [-127.46569, 50.12556]]]}</t>
+        </is>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R298" t="inlineStr">
+        <is>
+          <t>10.21966/21sf-ey03</t>
+        </is>
+      </c>
+      <c r="S298" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq77iyWJfPg4z-FvOSb</t>
+        </is>
+      </c>
+      <c r="T298" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U298" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V298" t="n">
+        <v>0</v>
+      </c>
+      <c r="W298" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X298" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>297</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>5177d019-598e-4415-b778-9688403652c8</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>ca-cioos_ed84df74-5a2d-4a7d-87c8-a7b93f11088e</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>BC Estuary Water Quality Monitoring Data - Nalaxdlala River Estuary (Provisional)</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H299" t="b">
+        <v>0</v>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>Estuary Resilience</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>tentative</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N299" t="n">
+        <v>1</v>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.9489, 50.70902], [-125.9696, 50.70291], [-126.00938, 50.69118], [-126.00108, 50.66848], [-125.98257, 50.68374], [-125.98152, 50.69271], [-125.95462, 50.70263], [-125.94785, 50.70768], [-125.9489, 50.70911], [-125.9489, 50.70902]]]}</t>
+        </is>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+        </is>
+      </c>
+      <c r="Q299" t="inlineStr">
+        <is>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R299" t="inlineStr">
+        <is>
+          <t>10.21966/4krv-aw23</t>
+        </is>
+      </c>
+      <c r="S299" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptbxmpkBsfyWWfSxOJ</t>
+        </is>
+      </c>
+      <c r="T299" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="U299" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="V299" t="n">
+        <v>0</v>
+      </c>
+      <c r="W299" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X299" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>298</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H300" t="b">
+        <v>0</v>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory, Geospatial</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>Tula Foundation</t>
+        </is>
+      </c>
+      <c r="N300" t="n">
+        <v>1</v>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
           <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
-      <c r="P284" t="inlineStr">
+      <c r="P300" t="inlineStr">
         <is>
           <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
-      <c r="Q284" t="inlineStr">
+      <c r="Q300" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="R284" t="inlineStr">
+      <c r="R300" t="inlineStr">
         <is>
           <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
-      <c r="S284" t="inlineStr">
+      <c r="S300" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
         </is>
       </c>
-      <c r="T284" t="inlineStr"/>
-      <c r="U284" t="inlineStr">
+      <c r="T300" t="inlineStr"/>
+      <c r="U300" t="inlineStr">
         <is>
           <t>2025-04-02</t>
         </is>
       </c>
-      <c r="V284" t="n">
-        <v>0</v>
-      </c>
-      <c r="W284" t="inlineStr">
+      <c r="V300" t="n">
+        <v>0</v>
+      </c>
+      <c r="W300" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="X284" t="inlineStr"/>
+      <c r="X300" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deployed 46f7daed9 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5561,12 +5561,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5576,7 +5576,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5622,7 +5622,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5632,17 +5632,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5671,12 +5671,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5747,12 +5747,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5781,12 +5781,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5852,17 +5852,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/1.715740</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -5891,12 +5891,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5962,17 +5962,17 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>10.21966/1.715740</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V51" t="n">
@@ -8523,12 +8523,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8538,7 +8538,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8580,16 +8580,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8599,12 +8599,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8633,12 +8633,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8648,7 +8648,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8690,16 +8690,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8709,12 +8709,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -14577,12 +14577,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14592,7 +14592,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14610,7 +14610,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14630,7 +14630,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14638,27 +14638,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14668,7 +14668,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14687,12 +14687,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14702,7 +14702,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14740,7 +14740,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14748,27 +14748,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -16779,12 +16779,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>ca-cioos_cec3dcef-8dba-4d91-aee6-b60ce416497c</t>
+          <t>ca-cioos_c89e35df-8a16-4efc-ae29-15f4e3da8a55</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -16794,7 +16794,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Mussel Dynamics - Point Intercepts - BC Central Coast</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -16850,17 +16850,17 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
         <is>
-          <t>10.21966/ns9h-1126</t>
+          <t>10.21966/0yk3-9b74</t>
         </is>
       </c>
       <c r="S150" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-MotaGdFmX3xEvWjXQA5</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-Motctf2E7ids9V-6Cfb</t>
         </is>
       </c>
       <c r="T150" t="inlineStr">
@@ -16870,7 +16870,7 @@
       </c>
       <c r="U150" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="V150" t="n">
@@ -16889,12 +16889,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>ca-cioos_c89e35df-8a16-4efc-ae29-15f4e3da8a55</t>
+          <t>ca-cioos_cec3dcef-8dba-4d91-aee6-b60ce416497c</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -16904,7 +16904,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast</t>
+          <t>Mussel Dynamics - Point Intercepts - BC Central Coast</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -16960,17 +16960,17 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R151" t="inlineStr">
         <is>
-          <t>10.21966/0yk3-9b74</t>
+          <t>10.21966/ns9h-1126</t>
         </is>
       </c>
       <c r="S151" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-Motctf2E7ids9V-6Cfb</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-MotaGdFmX3xEvWjXQA5</t>
         </is>
       </c>
       <c r="T151" t="inlineStr">
@@ -16980,7 +16980,7 @@
       </c>
       <c r="U151" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V151" t="n">
@@ -21623,12 +21623,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>ca-cioos_33a367c1-2706-4301-af99-4455fbe189a0</t>
+          <t>ca-cioos_3efdccb0-08ef-4e90-ac91-72969f94a99a</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -21638,7 +21638,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Cryosphere Snow Surveys Southwest British Columbia - Airborne Coastal Observatory</t>
+          <t>Bute Inlet Geohazard - Topography Surveys - 2023 - Hakai Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -21680,16 +21680,16 @@
         </is>
       </c>
       <c r="N194" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.9, 48.62], [-122.1, 48.62], [-122.1, 50.82], [-126.9, 50.82], [-126.9, 48.62]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.9, 50.53], [-124.2, 50.53], [-124.2, 50.99], [-124.9, 50.99], [-124.9, 50.53]]]}</t>
         </is>
       </c>
       <c r="P194" t="inlineStr">
         <is>
-          <t>[{'max': '2300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2600.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q194" t="inlineStr">
@@ -21699,12 +21699,12 @@
       </c>
       <c r="R194" t="inlineStr">
         <is>
-          <t>10.21966/thq7-0g08</t>
+          <t>10.21966/e4b8-vp48</t>
         </is>
       </c>
       <c r="S194" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRfMcU9I8mMcBH6qiv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRG7xQ84LQrgS4jhie</t>
         </is>
       </c>
       <c r="T194" t="inlineStr">
@@ -21714,15 +21714,15 @@
       </c>
       <c r="U194" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V194" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W194" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
       <c r="X194" t="inlineStr"/>
@@ -21733,12 +21733,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>ca-cioos_3efdccb0-08ef-4e90-ac91-72969f94a99a</t>
+          <t>ca-cioos_43422dc8-2573-4f60-bf87-df447d57ab7a</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -21748,7 +21748,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Bute Inlet Geohazard - Topography Surveys - 2023 - Hakai Airborne Coastal Observatory</t>
+          <t>USGS Glacier Mapping - 2023 - Hakai Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -21790,16 +21790,16 @@
         </is>
       </c>
       <c r="N195" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.9, 50.53], [-124.2, 50.53], [-124.2, 50.99], [-124.9, 50.99], [-124.9, 50.53]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.4, 47.68], [-113.0, 47.68], [-113.0, 49.08], [-121.4, 49.08], [-121.4, 47.68]]]}</t>
         </is>
       </c>
       <c r="P195" t="inlineStr">
         <is>
-          <t>[{'max': '2600.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2800.0', 'min': '100.0'}]</t>
         </is>
       </c>
       <c r="Q195" t="inlineStr">
@@ -21809,12 +21809,12 @@
       </c>
       <c r="R195" t="inlineStr">
         <is>
-          <t>10.21966/e4b8-vp48</t>
+          <t>10.21966/bzr6-er66</t>
         </is>
       </c>
       <c r="S195" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRG7xQ84LQrgS4jhie</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRKhzLRiCcp6ENuX2r</t>
         </is>
       </c>
       <c r="T195" t="inlineStr">
@@ -21824,15 +21824,15 @@
       </c>
       <c r="U195" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V195" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W195" t="inlineStr">
         <is>
-          <t>[{'year': '2026', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X195" t="inlineStr"/>
@@ -21843,12 +21843,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>ca-cioos_43422dc8-2573-4f60-bf87-df447d57ab7a</t>
+          <t>ca-cioos_33a367c1-2706-4301-af99-4455fbe189a0</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -21858,7 +21858,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>USGS Glacier Mapping - 2023 - Hakai Airborne Coastal Observatory</t>
+          <t>Cryosphere Snow Surveys Southwest British Columbia - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -21904,12 +21904,12 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.4, 47.68], [-113.0, 47.68], [-113.0, 49.08], [-121.4, 49.08], [-121.4, 47.68]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.9, 48.62], [-122.1, 48.62], [-122.1, 50.82], [-126.9, 50.82], [-126.9, 48.62]]]}</t>
         </is>
       </c>
       <c r="P196" t="inlineStr">
         <is>
-          <t>[{'max': '2800.0', 'min': '100.0'}]</t>
+          <t>[{'max': '2300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q196" t="inlineStr">
@@ -21919,12 +21919,12 @@
       </c>
       <c r="R196" t="inlineStr">
         <is>
-          <t>10.21966/bzr6-er66</t>
+          <t>10.21966/thq7-0g08</t>
         </is>
       </c>
       <c r="S196" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRKhzLRiCcp6ENuX2r</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRfMcU9I8mMcBH6qiv</t>
         </is>
       </c>
       <c r="T196" t="inlineStr">
@@ -21934,7 +21934,7 @@
       </c>
       <c r="U196" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V196" t="n">
@@ -21945,7 +21945,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X196" t="inlineStr"/>
+      <c r="X196" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -31195,12 +31197,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
+          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -31210,17 +31212,17 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
+          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>collection</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H281" t="b">
@@ -31233,7 +31235,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -31256,27 +31258,23 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
         </is>
       </c>
       <c r="P281" t="inlineStr">
         <is>
-          <t>[{'max': '2.5', 'min': '2.5'}]</t>
+          <t>[{'max': '0.0', 'min': '600.0'}]</t>
         </is>
       </c>
       <c r="Q281" t="inlineStr">
         <is>
-          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R281" t="inlineStr">
-        <is>
-          <t>10.21966/rrzq-yw32</t>
-        </is>
-      </c>
+          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr"/>
       <c r="S281" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
         </is>
       </c>
       <c r="T281" t="inlineStr">
@@ -31289,15 +31287,11 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="V281" t="n">
-        <v>0</v>
-      </c>
-      <c r="W281" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X281" t="inlineStr"/>
+      <c r="V281" t="inlineStr"/>
+      <c r="W281" t="inlineStr"/>
+      <c r="X281" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -31305,12 +31299,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
+          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -31320,17 +31314,17 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
+          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>collection</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H282" t="b">
@@ -31343,7 +31337,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -31366,23 +31360,27 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
         </is>
       </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '600.0'}]</t>
+          <t>[{'max': '2.5', 'min': '2.5'}]</t>
         </is>
       </c>
       <c r="Q282" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R282" t="inlineStr"/>
+          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>10.21966/rrzq-yw32</t>
+        </is>
+      </c>
       <c r="S282" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
         </is>
       </c>
       <c r="T282" t="inlineStr">
@@ -31395,10 +31393,16 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="V282" t="inlineStr"/>
-      <c r="W282" t="inlineStr"/>
+      <c r="V282" t="n">
+        <v>0</v>
+      </c>
+      <c r="W282" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="X282" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="283">
@@ -32294,7 +32298,7 @@
         </is>
       </c>
       <c r="X290" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="291">

</xml_diff>

<commit_message>
Deployed 47d7d4fe5 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X300"/>
+  <dimension ref="A1:X301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5561,12 +5561,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5576,7 +5576,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5622,7 +5622,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5632,17 +5632,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5671,12 +5671,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5747,12 +5747,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5781,12 +5781,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5852,17 +5852,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/1.715740</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -5891,12 +5891,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5962,17 +5962,17 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/1.715740</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V51" t="n">
@@ -6221,12 +6221,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6236,7 +6236,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6292,17 +6292,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6312,7 +6312,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6331,12 +6331,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6402,17 +6402,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -11715,12 +11715,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11730,7 +11730,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping Project - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11772,16 +11772,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.6286, 48.1332], [-122.8941, 48.1332], [-122.8941, 51.9689], [-128.6286, 51.9689], [-128.6286, 48.1332]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11791,12 +11791,12 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11806,7 +11806,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -11817,7 +11817,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X104" t="inlineStr"/>
+      <c r="X104" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -11825,12 +11827,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11840,7 +11842,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping Project - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -11858,7 +11860,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -11882,16 +11884,16 @@
         </is>
       </c>
       <c r="N105" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.6286, 48.1332], [-122.8941, 48.1332], [-122.8941, 51.9689], [-128.6286, 51.9689], [-128.6286, 48.1332]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -11901,12 +11903,12 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S105" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T105" t="inlineStr">
@@ -11916,7 +11918,7 @@
       </c>
       <c r="U105" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V105" t="n">
@@ -11927,9 +11929,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X105" t="n">
-        <v>3</v>
-      </c>
+      <c r="X105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -14577,12 +14577,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14592,7 +14592,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14610,7 +14610,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14630,7 +14630,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14638,27 +14638,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14668,7 +14668,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14687,12 +14687,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14702,7 +14702,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14740,7 +14740,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14748,27 +14748,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -21623,12 +21623,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
+          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>ca-cioos_3efdccb0-08ef-4e90-ac91-72969f94a99a</t>
+          <t>ca-cioos_33a367c1-2706-4301-af99-4455fbe189a0</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -21638,7 +21638,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Bute Inlet Geohazard - Topography Surveys - 2023 - Hakai Airborne Coastal Observatory</t>
+          <t>Cryosphere Snow Surveys Southwest British Columbia - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
@@ -21680,16 +21680,16 @@
         </is>
       </c>
       <c r="N194" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.9, 50.53], [-124.2, 50.53], [-124.2, 50.99], [-124.9, 50.99], [-124.9, 50.53]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.9, 48.62], [-122.1, 48.62], [-122.1, 50.82], [-126.9, 50.82], [-126.9, 48.62]]]}</t>
         </is>
       </c>
       <c r="P194" t="inlineStr">
         <is>
-          <t>[{'max': '2600.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q194" t="inlineStr">
@@ -21699,12 +21699,12 @@
       </c>
       <c r="R194" t="inlineStr">
         <is>
-          <t>10.21966/e4b8-vp48</t>
+          <t>10.21966/thq7-0g08</t>
         </is>
       </c>
       <c r="S194" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRG7xQ84LQrgS4jhie</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRfMcU9I8mMcBH6qiv</t>
         </is>
       </c>
       <c r="T194" t="inlineStr">
@@ -21714,15 +21714,15 @@
       </c>
       <c r="U194" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="V194" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W194" t="inlineStr">
         <is>
-          <t>[{'year': '2026', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X194" t="inlineStr"/>
@@ -21733,12 +21733,12 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
+          <t>f1aee211-bfab-46fd-b650-c5cacb782f40</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>ca-cioos_43422dc8-2573-4f60-bf87-df447d57ab7a</t>
+          <t>ca-cioos_3efdccb0-08ef-4e90-ac91-72969f94a99a</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -21748,7 +21748,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>USGS Glacier Mapping - 2023 - Hakai Airborne Coastal Observatory</t>
+          <t>Bute Inlet Geohazard - Topography Surveys - 2023 - Hakai Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
@@ -21790,16 +21790,16 @@
         </is>
       </c>
       <c r="N195" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.4, 47.68], [-113.0, 47.68], [-113.0, 49.08], [-121.4, 49.08], [-121.4, 47.68]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.9, 50.53], [-124.2, 50.53], [-124.2, 50.99], [-124.9, 50.99], [-124.9, 50.53]]]}</t>
         </is>
       </c>
       <c r="P195" t="inlineStr">
         <is>
-          <t>[{'max': '2800.0', 'min': '100.0'}]</t>
+          <t>[{'max': '2600.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q195" t="inlineStr">
@@ -21809,12 +21809,12 @@
       </c>
       <c r="R195" t="inlineStr">
         <is>
-          <t>10.21966/bzr6-er66</t>
+          <t>10.21966/e4b8-vp48</t>
         </is>
       </c>
       <c r="S195" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRKhzLRiCcp6ENuX2r</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRG7xQ84LQrgS4jhie</t>
         </is>
       </c>
       <c r="T195" t="inlineStr">
@@ -21824,15 +21824,15 @@
       </c>
       <c r="U195" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V195" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W195" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
       <c r="X195" t="inlineStr"/>
@@ -21843,12 +21843,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>6a28454e-107a-4059-9b7d-e43bf8ee693b</t>
+          <t>78efda1b-9688-4bcf-b16e-7167c17c0bcb</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>ca-cioos_33a367c1-2706-4301-af99-4455fbe189a0</t>
+          <t>ca-cioos_43422dc8-2573-4f60-bf87-df447d57ab7a</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -21858,7 +21858,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Cryosphere Snow Surveys Southwest British Columbia - Airborne Coastal Observatory</t>
+          <t>USGS Glacier Mapping - 2023 - Hakai Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -21904,12 +21904,12 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.9, 48.62], [-122.1, 48.62], [-122.1, 50.82], [-126.9, 50.82], [-126.9, 48.62]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.4, 47.68], [-113.0, 47.68], [-113.0, 49.08], [-121.4, 49.08], [-121.4, 47.68]]]}</t>
         </is>
       </c>
       <c r="P196" t="inlineStr">
         <is>
-          <t>[{'max': '2300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2800.0', 'min': '100.0'}]</t>
         </is>
       </c>
       <c r="Q196" t="inlineStr">
@@ -21919,12 +21919,12 @@
       </c>
       <c r="R196" t="inlineStr">
         <is>
-          <t>10.21966/thq7-0g08</t>
+          <t>10.21966/bzr6-er66</t>
         </is>
       </c>
       <c r="S196" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRfMcU9I8mMcBH6qiv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-NpRKhzLRiCcp6ENuX2r</t>
         </is>
       </c>
       <c r="T196" t="inlineStr">
@@ -21934,7 +21934,7 @@
       </c>
       <c r="U196" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V196" t="n">
@@ -21945,9 +21945,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X196" t="n">
-        <v>1</v>
-      </c>
+      <c r="X196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -22596,7 +22594,7 @@
       </c>
       <c r="U202" t="inlineStr">
         <is>
-          <t>2025-05-12</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="V202" t="n">
@@ -23047,7 +23045,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X206" t="inlineStr"/>
+      <c r="X206" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -31146,7 +31146,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.343, 51.8489], [-126.3333, 51.815], [-122.6652, 49.5126], [-123.9831, 49.2554], [-128.343, 51.8489]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.0471, 52.2577], [-128.9141, 51.7033], [-127.6841, 50.7687], [-123.7744, 48.9864], [-122.764, 49.331], [-122.8299, 49.9706], [-127.0471, 52.2577]]]}</t>
         </is>
       </c>
       <c r="P280" t="inlineStr">
@@ -31176,7 +31176,7 @@
       </c>
       <c r="U280" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="V280" t="n">
@@ -31197,12 +31197,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
+          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -31212,17 +31212,17 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
+          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>collection</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H281" t="b">
@@ -31235,7 +31235,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -31258,23 +31258,27 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
         </is>
       </c>
       <c r="P281" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '600.0'}]</t>
+          <t>[{'max': '2.5', 'min': '2.5'}]</t>
         </is>
       </c>
       <c r="Q281" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R281" t="inlineStr"/>
+          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr">
+        <is>
+          <t>10.21966/rrzq-yw32</t>
+        </is>
+      </c>
       <c r="S281" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
         </is>
       </c>
       <c r="T281" t="inlineStr">
@@ -31287,11 +31291,15 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="V281" t="inlineStr"/>
-      <c r="W281" t="inlineStr"/>
-      <c r="X281" t="n">
-        <v>2</v>
-      </c>
+      <c r="V281" t="n">
+        <v>0</v>
+      </c>
+      <c r="W281" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -31299,12 +31307,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
+          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -31314,17 +31322,17 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
+          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>collection</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H282" t="b">
@@ -31337,7 +31345,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -31360,27 +31368,23 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
         </is>
       </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>[{'max': '2.5', 'min': '2.5'}]</t>
+          <t>[{'max': '0.0', 'min': '600.0'}]</t>
         </is>
       </c>
       <c r="Q282" t="inlineStr">
         <is>
-          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R282" t="inlineStr">
-        <is>
-          <t>10.21966/rrzq-yw32</t>
-        </is>
-      </c>
+          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr"/>
       <c r="S282" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
         </is>
       </c>
       <c r="T282" t="inlineStr">
@@ -31393,16 +31397,10 @@
           <t>2026-09-10</t>
         </is>
       </c>
-      <c r="V282" t="n">
-        <v>0</v>
-      </c>
-      <c r="W282" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="V282" t="inlineStr"/>
+      <c r="W282" t="inlineStr"/>
       <c r="X282" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="283">
@@ -32298,7 +32296,7 @@
         </is>
       </c>
       <c r="X290" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="291">
@@ -33315,105 +33313,215 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
+          <t>dd471e82-a6b8-4f32-891c-bbea26e9998e</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>ca-cioos_aeb30028-a7eb-462e-ac0f-6c5fe101d4a2</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>DNA Metabarcoding Captures Temporal and Vertical Dynamics of Mesozooplankton Communities</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H300" t="b">
+        <v>0</v>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>Genomics, Oceanography</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
+      <c r="N300" t="n">
+        <v>2</v>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>{'type': 'Point', 'coordinates': [-125.0992, 50.0307]}</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>[{'max': '260.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>zooplanktonBiomassAndDiversity</t>
+        </is>
+      </c>
+      <c r="R300" t="inlineStr">
+        <is>
+          <t>10.21966/6b20-7r76</t>
+        </is>
+      </c>
+      <c r="S300" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OvzbmseH_syBXg1RXKd</t>
+        </is>
+      </c>
+      <c r="T300" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="U300" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="V300" t="n">
+        <v>0</v>
+      </c>
+      <c r="W300" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>299</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
           <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
         </is>
       </c>
-      <c r="C300" t="inlineStr">
+      <c r="C301" t="inlineStr">
         <is>
           <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
         </is>
       </c>
-      <c r="D300" t="inlineStr">
-        <is>
-          <t>Hakai Institute</t>
-        </is>
-      </c>
-      <c r="E300" t="inlineStr">
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
         <is>
           <t>Mount Robson Aerial Photo and LiDAR Survey</t>
         </is>
       </c>
-      <c r="F300" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="G300" t="inlineStr">
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
         <is>
           <t>CC-BY-4.0</t>
         </is>
       </c>
-      <c r="H300" t="b">
-        <v>0</v>
-      </c>
-      <c r="I300" t="inlineStr">
+      <c r="H301" t="b">
+        <v>0</v>
+      </c>
+      <c r="I301" t="inlineStr">
         <is>
           <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
-      <c r="J300" t="inlineStr">
+      <c r="J301" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="K300" t="inlineStr">
+      <c r="K301" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="L300" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="M300" t="inlineStr">
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M301" t="inlineStr">
         <is>
           <t>Tula Foundation</t>
         </is>
       </c>
-      <c r="N300" t="n">
+      <c r="N301" t="n">
         <v>1</v>
       </c>
-      <c r="O300" t="inlineStr">
+      <c r="O301" t="inlineStr">
         <is>
           <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
-      <c r="P300" t="inlineStr">
+      <c r="P301" t="inlineStr">
         <is>
           <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
-      <c r="Q300" t="inlineStr">
+      <c r="Q301" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="R300" t="inlineStr">
+      <c r="R301" t="inlineStr">
         <is>
           <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
-      <c r="S300" t="inlineStr">
+      <c r="S301" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
         </is>
       </c>
-      <c r="T300" t="inlineStr"/>
-      <c r="U300" t="inlineStr">
+      <c r="T301" t="inlineStr"/>
+      <c r="U301" t="inlineStr">
         <is>
           <t>2025-04-02</t>
         </is>
       </c>
-      <c r="V300" t="n">
-        <v>0</v>
-      </c>
-      <c r="W300" t="inlineStr">
+      <c r="V301" t="n">
+        <v>0</v>
+      </c>
+      <c r="W301" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="X300" t="inlineStr"/>
+      <c r="X301" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deployed fa7e2a091 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5561,12 +5561,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5576,7 +5576,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5622,7 +5622,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5632,17 +5632,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5671,12 +5671,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5747,12 +5747,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5781,12 +5781,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5852,17 +5852,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/1.715740</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -5891,12 +5891,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5962,17 +5962,17 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>10.21966/1.715740</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V51" t="n">
@@ -6221,12 +6221,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6236,7 +6236,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6292,17 +6292,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6312,7 +6312,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6331,12 +6331,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6402,17 +6402,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -8523,12 +8523,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8538,7 +8538,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8580,16 +8580,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8599,12 +8599,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8633,12 +8633,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8648,7 +8648,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8690,16 +8690,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8709,12 +8709,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -15127,12 +15127,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15142,7 +15142,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15160,7 +15160,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15180,20 +15180,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15203,12 +15203,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15218,7 +15218,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -15237,12 +15237,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -15252,7 +15252,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -15270,7 +15270,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -15290,20 +15290,20 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N136" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -15313,12 +15313,12 @@
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T136" t="inlineStr">
@@ -15328,7 +15328,7 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V136" t="n">
@@ -21494,7 +21494,7 @@
       </c>
       <c r="U192" t="inlineStr">
         <is>
-          <t>2025-04-23</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="V192" t="n">
@@ -21505,7 +21505,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X192" t="inlineStr"/>
+      <c r="X192" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -23045,9 +23047,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X206" t="n">
-        <v>1</v>
-      </c>
+      <c r="X206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="n">

</xml_diff>

<commit_message>
Deployed 8f7b419e0 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -8523,12 +8523,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8538,7 +8538,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8580,16 +8580,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8599,12 +8599,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8633,12 +8633,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8648,7 +8648,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8690,16 +8690,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8709,12 +8709,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -14577,12 +14577,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14592,7 +14592,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14610,7 +14610,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14630,7 +14630,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14638,27 +14638,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14668,7 +14668,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14687,12 +14687,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14702,7 +14702,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14740,7 +14740,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14748,27 +14748,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V131" t="n">
@@ -15127,12 +15127,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15142,7 +15142,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15160,7 +15160,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15180,20 +15180,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15203,12 +15203,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15218,7 +15218,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -15237,12 +15237,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -15252,7 +15252,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -15270,7 +15270,7 @@
       </c>
       <c r="I136" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J136" t="inlineStr">
@@ -15290,20 +15290,20 @@
       </c>
       <c r="M136" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N136" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">
@@ -15313,12 +15313,12 @@
       </c>
       <c r="R136" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S136" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T136" t="inlineStr">
@@ -15328,7 +15328,7 @@
       </c>
       <c r="U136" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V136" t="n">
@@ -27333,7 +27333,9 @@
           <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X245" t="inlineStr"/>
+      <c r="X245" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="n">

</xml_diff>

<commit_message>
Deployed 46332e004 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -4569,12 +4569,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
+          <t>b1d18883-a622-4f3c-9892-57564271e009</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ca-cioos_26a09a27-7f16-4944-b88d-8c3bf2d36f03</t>
+          <t>ca-cioos_33c870b8-3b4c-429d-bc10-99dd4c7f4c7d</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -4584,7 +4584,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Wind Fetch - BC Central Coast - Canada</t>
+          <t>Nearshore elevation and imagery models - Quadra Island Hakai Institute Facility Shoreline - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -4626,16 +4626,16 @@
         </is>
       </c>
       <c r="N39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.7578125, 50.16193379], [-126.22070312, 50.16193379], [-126.22070312, 52.84175491], [-131.7578125, 52.84175491], [-131.7578125, 50.16193379]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.2229327, 50.11245881], [-125.21821201, 50.11245881], [-125.21821201, 50.1172472], [-125.2229327, 50.1172472], [-125.2229327, 50.11245881]]]}</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -4645,12 +4645,12 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>10.21966/845b-yn81</t>
+          <t>10.21966/ebd6-yd93</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXNDOU8zYXhRdDA3RWM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXN1MUhmRE9GRndsSko</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
@@ -4660,7 +4660,7 @@
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="V39" t="n">
@@ -4679,12 +4679,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>b1d18883-a622-4f3c-9892-57564271e009</t>
+          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ca-cioos_33c870b8-3b4c-429d-bc10-99dd4c7f4c7d</t>
+          <t>ca-cioos_3f40326a-23f9-4e30-a16a-f332ace14e2f</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -4694,7 +4694,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Nearshore elevation and imagery models - Quadra Island Hakai Institute Facility Shoreline - British Columbia - Canada</t>
+          <t>Nereocystis kelp canopy productivity data from BC Central Coast</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -4712,12 +4712,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -4736,31 +4736,31 @@
         </is>
       </c>
       <c r="N40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.2229327, 50.11245881], [-125.21821201, 50.11245881], [-125.21821201, 50.1172472], [-125.2229327, 50.1172472], [-125.2229327, 50.11245881]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.6, 51.19], [-127.1, 51.19], [-127.1, 52.28], [-128.6, 52.28], [-128.6, 51.19]]]}</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>10.21966/ebd6-yd93</t>
+          <t>10.21966/d1s2-s530</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXN1MUhmRE9GRndsSko</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/df5J7W5Hk4e0p4yvlOAI0qcU9Gs2/-MtG8b48aDAEdJoqNT6N</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
@@ -4770,18 +4770,20 @@
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="V40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X40" t="inlineStr"/>
+          <t>[{'year': '2024', 'total': 1}]</t>
+        </is>
+      </c>
+      <c r="X40" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -4789,12 +4791,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>8275a332-8870-4300-8ca8-48b854e7dccf</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ca-cioos_3f40326a-23f9-4e30-a16a-f332ace14e2f</t>
+          <t>ca-cioos_26a09a27-7f16-4944-b88d-8c3bf2d36f03</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -4804,7 +4806,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Nereocystis kelp canopy productivity data from BC Central Coast</t>
+          <t>Wind Fetch - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -4822,12 +4824,12 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -4850,27 +4852,27 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.6, 51.19], [-127.1, 51.19], [-127.1, 52.28], [-128.6, 52.28], [-128.6, 51.19]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.7578125, 50.16193379], [-126.22070312, 50.16193379], [-126.22070312, 52.84175491], [-131.7578125, 52.84175491], [-131.7578125, 50.16193379]]]}</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>[{'max': '30.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>macroalgalCanopyCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>10.21966/d1s2-s530</t>
+          <t>10.21966/845b-yn81</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/df5J7W5Hk4e0p4yvlOAI0qcU9Gs2/-MtG8b48aDAEdJoqNT6N</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXNDOU8zYXhRdDA3RWM</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
@@ -4880,20 +4882,18 @@
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W41" t="inlineStr">
         <is>
-          <t>[{'year': '2024', 'total': 1}]</t>
-        </is>
-      </c>
-      <c r="X41" t="n">
-        <v>3</v>
-      </c>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -5561,12 +5561,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5576,7 +5576,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5622,7 +5622,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5632,17 +5632,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5671,12 +5671,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5732,7 +5732,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5747,12 +5747,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5781,12 +5781,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5814,7 +5814,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5852,17 +5852,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/1.715740</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5872,7 +5872,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -5891,12 +5891,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5906,7 +5906,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5952,7 +5952,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5962,17 +5962,17 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/1.715740</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -5982,7 +5982,7 @@
       </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V51" t="n">
@@ -6221,12 +6221,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6236,7 +6236,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6292,17 +6292,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6312,7 +6312,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -6331,12 +6331,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6346,7 +6346,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P55" t="inlineStr">
@@ -6402,17 +6402,17 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T55" t="inlineStr">
@@ -6422,7 +6422,7 @@
       </c>
       <c r="U55" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V55" t="n">
@@ -8523,12 +8523,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8538,7 +8538,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8580,16 +8580,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8599,12 +8599,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -8633,12 +8633,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8648,7 +8648,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -8690,16 +8690,16 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -8709,12 +8709,12 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T76" t="inlineStr">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="U76" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V76" t="n">
@@ -14577,12 +14577,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14592,7 +14592,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14610,7 +14610,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14630,7 +14630,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14638,27 +14638,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14668,7 +14668,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -14687,12 +14687,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -14702,7 +14702,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -14720,7 +14720,7 @@
       </c>
       <c r="I131" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J131" t="inlineStr">
@@ -14740,7 +14740,7 @@
       </c>
       <c r="M131" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N131" t="n">
@@ -14748,27 +14748,27 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R131" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S131" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T131" t="inlineStr">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="U131" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V131" t="n">

</xml_diff>

<commit_message>
Deployed f5a05c4f6 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5447,12 +5447,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5462,7 +5462,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -5518,17 +5518,17 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
@@ -5538,7 +5538,7 @@
       </c>
       <c r="U47" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V47" t="n">
@@ -5557,12 +5557,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5618,7 +5618,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5633,12 +5633,12 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5667,12 +5667,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5700,7 +5700,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -5728,7 +5728,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5738,17 +5738,17 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/1.715740</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5758,7 +5758,7 @@
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V49" t="n">
@@ -5777,12 +5777,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
+          <t>ca-cioos_4624baf9-ec39-4538-83fe-1563511b722c</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5792,7 +5792,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
+          <t>High-resolution record of surface seawater CO2 content from June 2017 to April 2019 collected in Sitka Harbor, Alaska, USA</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5838,7 +5838,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-135.62915433, 56.79541908], [-135.02059329, 56.79541908], [-135.02059329, 57.22157626], [-135.62915433, 57.22157626], [-135.62915433, 56.79541908]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5848,17 +5848,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/1.715740</t>
+          <t>10.21966/fwk1-a364</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXFtYXJjVDZ5V3UxcTk</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5868,7 +5868,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -5887,12 +5887,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>cb9c0488-666b-4869-9ca4-04d7125fdf8a</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ca-cioos_4624baf9-ec39-4538-83fe-1563511b722c</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>High-resolution record of surface seawater CO2 content from June 2017 to April 2019 collected in Sitka Harbor, Alaska, USA</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-135.62915433, 56.79541908], [-135.02059329, 56.79541908], [-135.02059329, 57.22157626], [-135.62915433, 57.22157626], [-135.62915433, 56.79541908]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
@@ -5963,12 +5963,12 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>10.21966/fwk1-a364</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXFtYXJjVDZ5V3UxcTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -13359,12 +13359,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -13374,7 +13374,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -13392,12 +13392,12 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -13416,16 +13416,16 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr">
@@ -13435,12 +13435,12 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T119" t="inlineStr">
@@ -13469,12 +13469,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13484,7 +13484,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13502,12 +13502,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13526,16 +13526,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13545,12 +13545,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -14459,12 +14459,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -14474,7 +14474,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -14492,7 +14492,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -14512,7 +14512,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N129" t="n">
@@ -14520,27 +14520,27 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T129" t="inlineStr">
@@ -14550,7 +14550,7 @@
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V129" t="n">
@@ -14569,12 +14569,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14584,7 +14584,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14602,7 +14602,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14622,7 +14622,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14630,27 +14630,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14660,7 +14660,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V130" t="n">

</xml_diff>

<commit_message>
Deployed 6138ef405 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5989,7 +5989,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X51" t="inlineStr"/>
+      <c r="X51" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -6107,12 +6109,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6122,7 +6124,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6168,7 +6170,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6178,17 +6180,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6198,7 +6200,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -6217,12 +6219,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6232,7 +6234,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6278,7 +6280,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6288,17 +6290,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6308,7 +6310,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -8407,12 +8409,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8422,7 +8424,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -8464,16 +8466,16 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -8483,12 +8485,12 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T74" t="inlineStr">
@@ -8498,7 +8500,7 @@
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V74" t="n">
@@ -8517,12 +8519,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8532,7 +8534,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8574,16 +8576,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8593,12 +8595,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8608,7 +8610,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -13359,12 +13361,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -13374,7 +13376,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -13392,12 +13394,12 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -13416,16 +13418,16 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr">
@@ -13435,12 +13437,12 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T119" t="inlineStr">
@@ -13469,12 +13471,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13484,7 +13486,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13502,12 +13504,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13526,16 +13528,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13545,12 +13547,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -15009,12 +15011,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -15024,7 +15026,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -15042,7 +15044,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -15062,20 +15064,20 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N134" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -15085,12 +15087,12 @@
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -15100,7 +15102,7 @@
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V134" t="n">
@@ -15119,12 +15121,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15134,7 +15136,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15152,7 +15154,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15172,20 +15174,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15195,12 +15197,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15210,7 +15212,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -16661,12 +16663,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
+          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>ca-cioos_cec3dcef-8dba-4d91-aee6-b60ce416497c</t>
+          <t>ca-cioos_c89e35df-8a16-4efc-ae29-15f4e3da8a55</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -16676,7 +16678,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Mussel Dynamics - Point Intercepts - BC Central Coast</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -16732,17 +16734,17 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R149" t="inlineStr">
         <is>
-          <t>10.21966/ns9h-1126</t>
+          <t>10.21966/0yk3-9b74</t>
         </is>
       </c>
       <c r="S149" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-MotaGdFmX3xEvWjXQA5</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-Motctf2E7ids9V-6Cfb</t>
         </is>
       </c>
       <c r="T149" t="inlineStr">
@@ -16752,7 +16754,7 @@
       </c>
       <c r="U149" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="V149" t="n">
@@ -16771,12 +16773,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>6ce6e697-d539-41b1-9771-b5e859a6ff50</t>
+          <t>46377bf0-06d5-4612-970d-29cd972e4870</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>ca-cioos_c89e35df-8a16-4efc-ae29-15f4e3da8a55</t>
+          <t>ca-cioos_cec3dcef-8dba-4d91-aee6-b60ce416497c</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -16786,7 +16788,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast</t>
+          <t>Mussel Dynamics - Point Intercepts - BC Central Coast</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -16842,17 +16844,17 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R150" t="inlineStr">
         <is>
-          <t>10.21966/0yk3-9b74</t>
+          <t>10.21966/ns9h-1126</t>
         </is>
       </c>
       <c r="S150" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-Motctf2E7ids9V-6Cfb</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-MotaGdFmX3xEvWjXQA5</t>
         </is>
       </c>
       <c r="T150" t="inlineStr">
@@ -16862,7 +16864,7 @@
       </c>
       <c r="U150" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V150" t="n">
@@ -21717,7 +21719,9 @@
           <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X194" t="inlineStr"/>
+      <c r="X194" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -31490,7 +31494,7 @@
       </c>
       <c r="U283" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V283" t="n">
@@ -31501,9 +31505,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X283" t="n">
-        <v>1</v>
-      </c>
+      <c r="X283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="n">
@@ -31602,7 +31604,7 @@
       </c>
       <c r="U284" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V284" t="n">
@@ -31613,9 +31615,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X284" t="n">
-        <v>1</v>
-      </c>
+      <c r="X284" t="inlineStr"/>
     </row>
     <row r="285">
       <c r="A285" t="n">
@@ -31714,7 +31714,7 @@
       </c>
       <c r="U285" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V285" t="n">
@@ -31725,9 +31725,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X285" t="n">
-        <v>1</v>
-      </c>
+      <c r="X285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="n">
@@ -31826,7 +31824,7 @@
       </c>
       <c r="U286" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V286" t="n">
@@ -31837,9 +31835,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X286" t="n">
-        <v>1</v>
-      </c>
+      <c r="X286" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" t="n">
@@ -31938,7 +31934,7 @@
       </c>
       <c r="U287" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V287" t="n">
@@ -31949,9 +31945,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X287" t="n">
-        <v>1</v>
-      </c>
+      <c r="X287" t="inlineStr"/>
     </row>
     <row r="288">
       <c r="A288" t="n">
@@ -32050,7 +32044,7 @@
       </c>
       <c r="U288" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V288" t="n">
@@ -32061,9 +32055,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X288" t="n">
-        <v>1</v>
-      </c>
+      <c r="X288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="n">
@@ -32162,7 +32154,7 @@
       </c>
       <c r="U289" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V289" t="n">
@@ -32173,9 +32165,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X289" t="n">
-        <v>1</v>
-      </c>
+      <c r="X289" t="inlineStr"/>
     </row>
     <row r="290">
       <c r="A290" t="n">
@@ -32274,7 +32264,7 @@
       </c>
       <c r="U290" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V290" t="n">
@@ -32285,9 +32275,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X290" t="n">
-        <v>1</v>
-      </c>
+      <c r="X290" t="inlineStr"/>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -32386,7 +32374,7 @@
       </c>
       <c r="U291" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V291" t="n">
@@ -32397,9 +32385,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X291" t="n">
-        <v>1</v>
-      </c>
+      <c r="X291" t="inlineStr"/>
     </row>
     <row r="292">
       <c r="A292" t="n">
@@ -32498,7 +32484,7 @@
       </c>
       <c r="U292" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V292" t="n">
@@ -32509,9 +32495,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X292" t="n">
-        <v>1</v>
-      </c>
+      <c r="X292" t="inlineStr"/>
     </row>
     <row r="293">
       <c r="A293" t="n">
@@ -32519,12 +32503,12 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
+          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>ca-cioos_b922699f-69b6-4d63-b538-7c290086a408</t>
+          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -32534,7 +32518,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Quw'utsun/Xwulqw'selu River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
@@ -32580,7 +32564,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.56201, 48.73508], [-123.59772, 48.75559], [-123.62127, 48.76514], [-123.63885, 48.77426], [-123.66935, 48.78033], [-123.67901, 48.75472], [-123.65155, 48.74322], [-123.63017, 48.7405], [-123.60792, 48.74289], [-123.56494, 48.72987], [-123.56179, 48.73529], [-123.56201, 48.73508]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635], [-123.66843, 48.91641]]]}</t>
         </is>
       </c>
       <c r="P293" t="inlineStr">
@@ -32595,12 +32579,12 @@
       </c>
       <c r="R293" t="inlineStr">
         <is>
-          <t>10.21966/2ha7-9p26</t>
+          <t>10.21966/q2e0-j004</t>
         </is>
       </c>
       <c r="S293" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpsCA3ycwZ7bFTDIQxh</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
         </is>
       </c>
       <c r="T293" t="inlineStr">
@@ -32610,7 +32594,7 @@
       </c>
       <c r="U293" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V293" t="n">
@@ -32621,9 +32605,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X293" t="n">
-        <v>1</v>
-      </c>
+      <c r="X293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -32631,12 +32613,12 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
+          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
+          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -32646,7 +32628,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -32692,7 +32674,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635], [-123.66843, 48.91641]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
         </is>
       </c>
       <c r="P294" t="inlineStr">
@@ -32707,12 +32689,12 @@
       </c>
       <c r="R294" t="inlineStr">
         <is>
-          <t>10.21966/q2e0-j004</t>
+          <t>10.21966/hjkj-6611</t>
         </is>
       </c>
       <c r="S294" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
         </is>
       </c>
       <c r="T294" t="inlineStr">
@@ -32722,7 +32704,7 @@
       </c>
       <c r="U294" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V294" t="n">
@@ -32733,9 +32715,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X294" t="n">
-        <v>1</v>
-      </c>
+      <c r="X294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -32743,12 +32723,12 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
+          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
+          <t>ca-cioos_dce15b7b-3772-4106-ab20-c3979c4c3f57</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
@@ -32758,7 +32738,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Fulmore River - Shoal Creek Estuary Complex (Provisional)</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -32804,7 +32784,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.08798, 50.4777], [-126.09599, 50.48418], [-126.09046, 50.50918], [-126.0647, 50.52425], [-125.99698, 50.53569], [-125.93459, 50.56717], [-125.93173, 50.56202], [-125.93764, 50.55458], [-125.91055, 50.55134], [-125.89853, 50.54943], [-125.90063, 50.54466], [-125.96416, 50.53989], [-125.98973, 50.52043], [-126.06566, 50.5067], [-126.08779, 50.47789], [-126.08798, 50.4777]]]}</t>
         </is>
       </c>
       <c r="P295" t="inlineStr">
@@ -32819,12 +32799,12 @@
       </c>
       <c r="R295" t="inlineStr">
         <is>
-          <t>10.21966/hjkj-6611</t>
+          <t>10.21966/g1cn-xs92</t>
         </is>
       </c>
       <c r="S295" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptdJ8iUmLeOrdmqzrQ</t>
         </is>
       </c>
       <c r="T295" t="inlineStr">
@@ -32834,7 +32814,7 @@
       </c>
       <c r="U295" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V295" t="n">
@@ -32845,9 +32825,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X295" t="n">
-        <v>1</v>
-      </c>
+      <c r="X295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -32855,12 +32833,12 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
+          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>ca-cioos_dce15b7b-3772-4106-ab20-c3979c4c3f57</t>
+          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -32870,7 +32848,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Fulmore River - Shoal Creek Estuary Complex (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -32916,7 +32894,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.08798, 50.4777], [-126.09599, 50.48418], [-126.09046, 50.50918], [-126.0647, 50.52425], [-125.99698, 50.53569], [-125.93459, 50.56717], [-125.93173, 50.56202], [-125.93764, 50.55458], [-125.91055, 50.55134], [-125.89853, 50.54943], [-125.90063, 50.54466], [-125.96416, 50.53989], [-125.98973, 50.52043], [-126.06566, 50.5067], [-126.08779, 50.47789], [-126.08798, 50.4777]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
         </is>
       </c>
       <c r="P296" t="inlineStr">
@@ -32931,12 +32909,12 @@
       </c>
       <c r="R296" t="inlineStr">
         <is>
-          <t>10.21966/g1cn-xs92</t>
+          <t>10.21966/npe4-3036</t>
         </is>
       </c>
       <c r="S296" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptdJ8iUmLeOrdmqzrQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
         </is>
       </c>
       <c r="T296" t="inlineStr">
@@ -32946,7 +32924,7 @@
       </c>
       <c r="U296" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V296" t="n">
@@ -32957,9 +32935,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X296" t="n">
-        <v>1</v>
-      </c>
+      <c r="X296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="n">
@@ -32967,12 +32943,12 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
+          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
+          <t>ca-cioos_e9b72149-8cf1-4000-ae3e-6b29ad60b078</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
@@ -32982,7 +32958,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Malksope River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -33028,7 +33004,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.46569, 50.12556], [-127.45723, 50.13142], [-127.43281, 50.13338], [-127.42845, 50.13765], [-127.41181, 50.14408], [-127.40973, 50.14233], [-127.41999, 50.13627], [-127.41803, 50.13195], [-127.43106, 50.12796], [-127.46545, 50.12446], [-127.46569, 50.12548], [-127.46569, 50.12556]]]}</t>
         </is>
       </c>
       <c r="P297" t="inlineStr">
@@ -33043,12 +33019,12 @@
       </c>
       <c r="R297" t="inlineStr">
         <is>
-          <t>10.21966/npe4-3036</t>
+          <t>10.21966/21sf-ey03</t>
         </is>
       </c>
       <c r="S297" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq77iyWJfPg4z-FvOSb</t>
         </is>
       </c>
       <c r="T297" t="inlineStr">
@@ -33058,7 +33034,7 @@
       </c>
       <c r="U297" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V297" t="n">
@@ -33069,9 +33045,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X297" t="n">
-        <v>1</v>
-      </c>
+      <c r="X297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="n">
@@ -33079,12 +33053,12 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
+          <t>5177d019-598e-4415-b778-9688403652c8</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>ca-cioos_e9b72149-8cf1-4000-ae3e-6b29ad60b078</t>
+          <t>ca-cioos_ed84df74-5a2d-4a7d-87c8-a7b93f11088e</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
@@ -33094,7 +33068,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Malksope River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Nalaxdlala River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
@@ -33140,7 +33114,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.46569, 50.12556], [-127.45723, 50.13142], [-127.43281, 50.13338], [-127.42845, 50.13765], [-127.41181, 50.14408], [-127.40973, 50.14233], [-127.41999, 50.13627], [-127.41803, 50.13195], [-127.43106, 50.12796], [-127.46545, 50.12446], [-127.46569, 50.12548], [-127.46569, 50.12556]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.9489, 50.70902], [-125.9696, 50.70291], [-126.00938, 50.69118], [-126.00108, 50.66848], [-125.98257, 50.68374], [-125.98152, 50.69271], [-125.95462, 50.70263], [-125.94785, 50.70768], [-125.9489, 50.70911], [-125.9489, 50.70902]]]}</t>
         </is>
       </c>
       <c r="P298" t="inlineStr">
@@ -33155,12 +33129,12 @@
       </c>
       <c r="R298" t="inlineStr">
         <is>
-          <t>10.21966/21sf-ey03</t>
+          <t>10.21966/4krv-aw23</t>
         </is>
       </c>
       <c r="S298" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq77iyWJfPg4z-FvOSb</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptbxmpkBsfyWWfSxOJ</t>
         </is>
       </c>
       <c r="T298" t="inlineStr">
@@ -33170,7 +33144,7 @@
       </c>
       <c r="U298" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V298" t="n">
@@ -33181,9 +33155,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X298" t="n">
-        <v>1</v>
-      </c>
+      <c r="X298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="n">
@@ -33191,12 +33163,12 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>5177d019-598e-4415-b778-9688403652c8</t>
+          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>ca-cioos_ed84df74-5a2d-4a7d-87c8-a7b93f11088e</t>
+          <t>ca-cioos_b922699f-69b6-4d63-b538-7c290086a408</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
@@ -33206,7 +33178,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Nalaxdlala River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Quw'utsun/Xwulqw'selu River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -33252,7 +33224,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.9489, 50.70902], [-125.9696, 50.70291], [-126.00938, 50.69118], [-126.00108, 50.66848], [-125.98257, 50.68374], [-125.98152, 50.69271], [-125.95462, 50.70263], [-125.94785, 50.70768], [-125.9489, 50.70911], [-125.9489, 50.70902]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.56201, 48.73508], [-123.59772, 48.75559], [-123.62127, 48.76514], [-123.63885, 48.77426], [-123.66935, 48.78033], [-123.67901, 48.75472], [-123.65155, 48.74322], [-123.63017, 48.7405], [-123.60792, 48.74289], [-123.56494, 48.72987], [-123.56179, 48.73529], [-123.56201, 48.73508]]]}</t>
         </is>
       </c>
       <c r="P299" t="inlineStr">
@@ -33267,22 +33239,22 @@
       </c>
       <c r="R299" t="inlineStr">
         <is>
-          <t>10.21966/4krv-aw23</t>
+          <t>10.21966/2ha7-9p26</t>
         </is>
       </c>
       <c r="S299" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptbxmpkBsfyWWfSxOJ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpsCA3ycwZ7bFTDIQxh</t>
         </is>
       </c>
       <c r="T299" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="U299" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V299" t="n">
@@ -33293,9 +33265,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X299" t="n">
-        <v>1</v>
-      </c>
+      <c r="X299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="n">
@@ -33504,7 +33474,7 @@
       </c>
       <c r="U301" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V301" t="n">

</xml_diff>

<commit_message>
Deployed 8ee57cc19 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5557,12 +5557,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5618,7 +5618,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5628,17 +5628,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5659,7 +5659,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X48" t="inlineStr"/>
+      <c r="X48" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -5667,12 +5669,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5682,7 +5684,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5700,7 +5702,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -5728,7 +5730,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5738,17 +5740,17 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/1.715740</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5758,7 +5760,7 @@
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V49" t="n">
@@ -5777,12 +5779,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5792,7 +5794,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5838,7 +5840,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5848,17 +5850,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/1.715740</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5868,7 +5870,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -9067,12 +9069,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -9082,7 +9084,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -9100,7 +9102,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -9128,12 +9130,12 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -9143,12 +9145,12 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T80" t="inlineStr">
@@ -9177,12 +9179,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9192,7 +9194,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9210,7 +9212,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -9238,12 +9240,12 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -9253,12 +9255,12 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -11599,12 +11601,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11614,7 +11616,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping Project - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11632,7 +11634,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11656,16 +11658,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.6286, 48.1332], [-122.8941, 48.1332], [-122.8941, 51.9689], [-128.6286, 51.9689], [-128.6286, 48.1332]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11675,12 +11677,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11690,7 +11692,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11709,12 +11711,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11724,7 +11726,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping Project - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11742,7 +11744,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11766,16 +11768,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.6286, 48.1332], [-122.8941, 48.1332], [-122.8941, 51.9689], [-128.6286, 51.9689], [-128.6286, 48.1332]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11785,12 +11787,12 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11800,7 +11802,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -13029,12 +13031,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -13044,7 +13046,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -13067,7 +13069,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -13086,11 +13088,11 @@
         </is>
       </c>
       <c r="N116" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -13105,12 +13107,12 @@
       </c>
       <c r="R116" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T116" t="inlineStr">
@@ -13120,7 +13122,7 @@
       </c>
       <c r="U116" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V116" t="n">
@@ -13128,7 +13130,7 @@
       </c>
       <c r="W116" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X116" t="inlineStr"/>
@@ -13139,12 +13141,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13154,7 +13156,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13177,7 +13179,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13196,11 +13198,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13215,12 +13217,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13230,7 +13232,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13238,7 +13240,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -13359,12 +13361,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -13374,7 +13376,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -13392,12 +13394,12 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -13416,16 +13418,16 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr">
@@ -13435,12 +13437,12 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T119" t="inlineStr">
@@ -13469,12 +13471,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13484,7 +13486,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13502,12 +13504,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13526,16 +13528,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13545,12 +13547,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -15111,7 +15113,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X134" t="inlineStr"/>
+      <c r="X134" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -20615,7 +20619,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X184" t="inlineStr"/>
+      <c r="X184" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -31183,12 +31189,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
+          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -31198,17 +31204,17 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
+          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>collection</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H281" t="b">
@@ -31221,7 +31227,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -31244,23 +31250,27 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
         </is>
       </c>
       <c r="P281" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '600.0'}]</t>
+          <t>[{'max': '2.5', 'min': '2.5'}]</t>
         </is>
       </c>
       <c r="Q281" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R281" t="inlineStr"/>
+          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr">
+        <is>
+          <t>10.21966/rrzq-yw32</t>
+        </is>
+      </c>
       <c r="S281" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
         </is>
       </c>
       <c r="T281" t="inlineStr">
@@ -31270,14 +31280,18 @@
       </c>
       <c r="U281" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="V281" t="inlineStr"/>
-      <c r="W281" t="inlineStr"/>
-      <c r="X281" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="V281" t="n">
+        <v>0</v>
+      </c>
+      <c r="W281" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -31285,12 +31299,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
+          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -31300,17 +31314,17 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
+          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>collection</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H282" t="b">
@@ -31323,7 +31337,7 @@
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -31346,27 +31360,23 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
         </is>
       </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>[{'max': '2.5', 'min': '2.5'}]</t>
+          <t>[{'max': '0.0', 'min': '600.0'}]</t>
         </is>
       </c>
       <c r="Q282" t="inlineStr">
         <is>
-          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R282" t="inlineStr">
-        <is>
-          <t>10.21966/rrzq-yw32</t>
-        </is>
-      </c>
+          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr"/>
       <c r="S282" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
         </is>
       </c>
       <c r="T282" t="inlineStr">
@@ -31376,19 +31386,13 @@
       </c>
       <c r="U282" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="V282" t="n">
-        <v>0</v>
-      </c>
-      <c r="W282" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="V282" t="inlineStr"/>
+      <c r="W282" t="inlineStr"/>
       <c r="X282" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="283">

</xml_diff>

<commit_message>
Deployed 593319b6a to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5557,12 +5557,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5618,7 +5618,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5628,17 +5628,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -5659,9 +5659,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X48" t="n">
-        <v>1</v>
-      </c>
+      <c r="X48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -5669,12 +5667,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -5684,7 +5682,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -5702,7 +5700,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -5730,7 +5728,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
@@ -5740,17 +5738,17 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/1.715740</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
         </is>
       </c>
       <c r="T49" t="inlineStr">
@@ -5760,7 +5758,7 @@
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V49" t="n">
@@ -5779,12 +5777,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>876027b6-cf37-4d49-8c3d-22d40b5f5b0b</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ca-cioos_3d7d93d0-73be-4c1b-af09-307e60a3576d</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -5794,7 +5792,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Water column carbonate system measurements from the Pacific Salmon Foundation Citizen Science Program stations from July 2016 to October 2017 in the northern Salish Sea, British Columbia, Canada</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -5840,7 +5838,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.35968411, 49.4351949], [-124.37299598, 49.4351949], [-124.37299598, 50.10196506], [-125.35968411, 50.10196506], [-125.35968411, 49.4351949]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
@@ -5850,17 +5848,17 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>10.21966/1.715740</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW9ENGY0VHBJTUd6blo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -5870,7 +5868,7 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -6109,12 +6107,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6124,7 +6122,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6170,7 +6168,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6180,17 +6178,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6200,7 +6198,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -6219,12 +6217,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6234,7 +6232,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6280,7 +6278,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6290,17 +6288,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6310,7 +6308,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -9069,12 +9067,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -9084,7 +9082,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -9102,7 +9100,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -9130,12 +9128,12 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -9145,12 +9143,12 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T80" t="inlineStr">
@@ -9179,12 +9177,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9194,7 +9192,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9212,7 +9210,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -9240,12 +9238,12 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -9255,12 +9253,12 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -11601,12 +11599,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11616,7 +11614,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping Project - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11634,7 +11632,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11658,16 +11656,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.6286, 48.1332], [-122.8941, 48.1332], [-122.8941, 51.9689], [-128.6286, 51.9689], [-128.6286, 48.1332]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11677,12 +11675,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11692,7 +11690,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11711,12 +11709,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11726,7 +11724,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping Project - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11744,7 +11742,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11768,16 +11766,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.6286, 48.1332], [-122.8941, 48.1332], [-122.8941, 51.9689], [-128.6286, 51.9689], [-128.6286, 48.1332]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11787,12 +11785,12 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11802,7 +11800,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -13031,12 +13029,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -13046,7 +13044,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -13069,7 +13067,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -13088,11 +13086,11 @@
         </is>
       </c>
       <c r="N116" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -13107,12 +13105,12 @@
       </c>
       <c r="R116" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T116" t="inlineStr">
@@ -13122,7 +13120,7 @@
       </c>
       <c r="U116" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V116" t="n">
@@ -13130,7 +13128,7 @@
       </c>
       <c r="W116" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X116" t="inlineStr"/>
@@ -13141,12 +13139,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13156,7 +13154,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13179,7 +13177,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13198,11 +13196,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13217,12 +13215,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13232,7 +13230,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13240,7 +13238,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -15113,9 +15111,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X134" t="n">
-        <v>1</v>
-      </c>
+      <c r="X134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -20619,9 +20615,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X184" t="n">
-        <v>1</v>
-      </c>
+      <c r="X184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">

</xml_diff>

<commit_message>
Deployed 80eccb76f to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X302"/>
+  <dimension ref="A1:X301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6105,12 +6105,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6176,17 +6176,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -6215,12 +6215,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6286,17 +6286,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -8405,12 +8405,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8420,7 +8420,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -8462,16 +8462,16 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -8481,12 +8481,12 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T74" t="inlineStr">
@@ -8496,7 +8496,7 @@
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V74" t="n">
@@ -8515,12 +8515,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8530,7 +8530,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8572,16 +8572,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8591,12 +8591,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -11595,12 +11595,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
+          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
+          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -11610,7 +11610,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
+          <t>Rocky Intertidal RPAS Mapping Project - BC Central Coast - Canada</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -11628,7 +11628,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Geospatial, Nearshore</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -11652,16 +11652,16 @@
         </is>
       </c>
       <c r="N103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.6286, 48.1332], [-122.8941, 48.1332], [-122.8941, 51.9689], [-128.6286, 51.9689], [-128.6286, 48.1332]]]}</t>
         </is>
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr">
@@ -11671,12 +11671,12 @@
       </c>
       <c r="R103" t="inlineStr">
         <is>
-          <t>10.21966/3yew-5r94</t>
+          <t>10.21966/mc7v-dx06</t>
         </is>
       </c>
       <c r="S103" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
         </is>
       </c>
       <c r="T103" t="inlineStr">
@@ -11686,7 +11686,7 @@
       </c>
       <c r="U103" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="V103" t="n">
@@ -11705,12 +11705,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>70f29525-f17b-4bc7-ae7f-d1e7205ba16c</t>
+          <t>b3e5b67d-2425-4a4f-80b0-d1076df5492a</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>ca-cioos_7de69ca8-b3f3-4761-b441-dfc9e63b1fbc</t>
+          <t>ca-cioos_7e0f0bbc-507a-4ca0-bafc-1cc3e56db028</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -11720,7 +11720,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Rocky Intertidal RPAS Mapping Project - BC Central Coast - Canada</t>
+          <t>Hakai physical plan and utility lines – Calvert Island Field Station - 2006</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -11738,7 +11738,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Geospatial, Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -11762,16 +11762,16 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.6286, 48.1332], [-122.8941, 48.1332], [-122.8941, 51.9689], [-128.6286, 51.9689], [-128.6286, 48.1332]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13541603114572, 51.65216411387959], [-128.12786293055976, 51.65216411387959], [-128.12786293055976, 51.6557318761607], [-128.13541603114572, 51.6557318761607], [-128.13541603114572, 51.65216411387959]]]}</t>
         </is>
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr">
@@ -11781,12 +11781,12 @@
       </c>
       <c r="R104" t="inlineStr">
         <is>
-          <t>10.21966/mc7v-dx06</t>
+          <t>10.21966/3yew-5r94</t>
         </is>
       </c>
       <c r="S104" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXBVWDBQSFpnWjBBS0Q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU9IR0RmSHlkRW1sd2k</t>
         </is>
       </c>
       <c r="T104" t="inlineStr">
@@ -11796,7 +11796,7 @@
       </c>
       <c r="U104" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V104" t="n">
@@ -15005,12 +15005,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -15020,7 +15020,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -15038,7 +15038,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -15058,20 +15058,20 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N134" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -15081,12 +15081,12 @@
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -15096,7 +15096,7 @@
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V134" t="n">
@@ -15115,12 +15115,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15130,7 +15130,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15148,7 +15148,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15168,20 +15168,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15191,12 +15191,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15206,7 +15206,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -20609,9 +20609,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X184" t="n">
-        <v>1</v>
-      </c>
+      <c r="X184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -27431,12 +27429,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>7b1120bc-4a2c-432c-9e54-879d66751a59</t>
+          <t>49374495-400f-4acc-aac6-d7d0b7cae297</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>ca-cioos_b2b18171-35b6-4345-b81b-497a90c2e7c5</t>
+          <t>ca-cioos_bafcd0eb-8249-471b-b93b-0797cfeea287</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -27446,7 +27444,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Seagrass fish and macroinvertebrate swaths BC Central Coast</t>
+          <t>Spatial extent of surface canopy kelp derived from fixed-wing surveys (2020), Central Coast, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
@@ -27464,12 +27462,12 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Nearshore, Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -27492,37 +27490,37 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 52.09], [-128.5, 52.04], [-128.5, 51.97], [-128.5, 51.93], [-128.5, 51.9], [-128.4, 51.88], [-128.3, 51.86], [-128.3, 51.83], [-128.2, 51.63], [-127.9, 51.62], [-127.8, 51.77], [-127.8, 51.83], [-127.9, 51.99], [-128.4, 52.09]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 51.64], [-128.1, 51.64], [-128.1, 52.01], [-128.5, 52.01], [-128.5, 51.64]]]}</t>
         </is>
       </c>
       <c r="P247" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q247" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
+          <t>macroalgalCanopyCoverAndComposition, other</t>
         </is>
       </c>
       <c r="R247" t="inlineStr">
         <is>
-          <t>10.21966/NMNG-SF35</t>
+          <t>10.21966/20ym-8826</t>
         </is>
       </c>
       <c r="S247" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7327bul36pby-Odi</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Miha19AtLQ2u1uo0b_q</t>
         </is>
       </c>
       <c r="T247" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="U247" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="V247" t="n">
@@ -27541,12 +27539,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>49374495-400f-4acc-aac6-d7d0b7cae297</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>ca-cioos_bafcd0eb-8249-471b-b93b-0797cfeea287</t>
+          <t>ca-cioos_ba41d935-f293-447f-be3d-7098e569b431</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -27556,7 +27554,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Spatial extent of surface canopy kelp derived from fixed-wing surveys (2020), Central Coast, British Columbia, Canada</t>
+          <t>Water Property Measurements from Conductivity-Temperature-Depth Profilers, BC, Canada (Research)</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -27574,12 +27572,12 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>Nearshore, Airborne Coastal Observatory, Geospatial</t>
+          <t>Oceanography, Nearshore, Watersheds, Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -27598,41 +27596,41 @@
         </is>
       </c>
       <c r="N248" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 51.64], [-128.1, 51.64], [-128.1, 52.01], [-128.5, 52.01], [-128.5, 51.64]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 52.27], [-127.4, 52.21], [-127.2, 51.66], [-125.6, 51.13], [-124.8, 50.96], [-124.1, 50.43], [-124.7, 49.98], [-124.9, 49.8], [-126.7, 50.45], [-128.1, 51.37], [-128.4, 51.69], [-128.5, 52.27]]]}</t>
         </is>
       </c>
       <c r="P248" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '700.0', 'min': '1.0'}]</t>
         </is>
       </c>
       <c r="Q248" t="inlineStr">
         <is>
-          <t>macroalgalCanopyCoverAndComposition, other</t>
+          <t>oxygen, subSurfaceSalinity, subSurfaceTemperature</t>
         </is>
       </c>
       <c r="R248" t="inlineStr">
         <is>
-          <t>10.21966/20ym-8826</t>
+          <t>10.21966/kace-2d24</t>
         </is>
       </c>
       <c r="S248" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Miha19AtLQ2u1uo0b_q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MX35qgX-BrwJDdeJKe1</t>
         </is>
       </c>
       <c r="T248" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="U248" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="V248" t="n">
@@ -27651,12 +27649,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>ca-cioos_ba41d935-f293-447f-be3d-7098e569b431</t>
+          <t>ca-cioos_fb5c9e1e-a911-46b7-8c1d-e34215a105ed</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -27666,7 +27664,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Water Property Measurements from Conductivity-Temperature-Depth Profilers, BC, Canada (Research)</t>
+          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 Analyzer located at Bamfield Marine Sciences Centre, Bamfield, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -27684,12 +27682,12 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>Oceanography, Nearshore, Watersheds, Juvenile Salmon Program</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -27708,31 +27706,31 @@
         </is>
       </c>
       <c r="N249" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 52.27], [-127.4, 52.21], [-127.2, 51.66], [-125.6, 51.13], [-124.8, 50.96], [-124.1, 50.43], [-124.7, 49.98], [-124.9, 49.8], [-126.7, 50.45], [-128.1, 51.37], [-128.4, 51.69], [-128.5, 52.27]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.13535, 48.83515]}</t>
         </is>
       </c>
       <c r="P249" t="inlineStr">
         <is>
-          <t>[{'max': '700.0', 'min': '1.0'}]</t>
+          <t>[{'max': '20.0', 'min': '20.0'}]</t>
         </is>
       </c>
       <c r="Q249" t="inlineStr">
         <is>
-          <t>oxygen, subSurfaceSalinity, subSurfaceTemperature</t>
+          <t>seaSurfaceTemperature, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
         </is>
       </c>
       <c r="R249" t="inlineStr">
         <is>
-          <t>10.21966/kace-2d24</t>
+          <t>10.21966/65d8-k051</t>
         </is>
       </c>
       <c r="S249" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MX35qgX-BrwJDdeJKe1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-NdH-jgHZQzKrYdb2nw_</t>
         </is>
       </c>
       <c r="T249" t="inlineStr">
@@ -27742,7 +27740,7 @@
       </c>
       <c r="U249" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V249" t="n">
@@ -27761,12 +27759,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>ca-cioos_fb5c9e1e-a911-46b7-8c1d-e34215a105ed</t>
+          <t>ca-cioos_91107fce-93a4-4bc9-bce4-e7d9e1cf02a0</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -27776,7 +27774,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 Analyzer located at Bamfield Marine Sciences Centre, Bamfield, BC, Canada (Provisional)</t>
+          <t>Sentinel 3A and 3B Chlorophyll and Suspended Matter Concentrations for Coastal British Columbia and Southeast Alaska, 8-Day Average (Research)</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -27799,7 +27797,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -27822,37 +27820,37 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.13535, 48.83515]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
         </is>
       </c>
       <c r="P250" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '20.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q250" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
+          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
         </is>
       </c>
       <c r="R250" t="inlineStr">
         <is>
-          <t>10.21966/65d8-k051</t>
+          <t>10.21966/175j-8k96</t>
         </is>
       </c>
       <c r="S250" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-NdH-jgHZQzKrYdb2nw_</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-Nueis-TZEnz_78f8PYf</t>
         </is>
       </c>
       <c r="T250" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="U250" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="V250" t="n">
@@ -27863,7 +27861,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X250" t="inlineStr"/>
+      <c r="X250" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -27871,12 +27871,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>ca-cioos_91107fce-93a4-4bc9-bce4-e7d9e1cf02a0</t>
+          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -27886,7 +27886,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Sentinel 3A and 3B Chlorophyll and Suspended Matter Concentrations for Coastal British Columbia and Southeast Alaska, 8-Day Average (Research)</t>
+          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -27947,12 +27947,12 @@
       </c>
       <c r="R251" t="inlineStr">
         <is>
-          <t>10.21966/175j-8k96</t>
+          <t>10.21966/dveq-bt48</t>
         </is>
       </c>
       <c r="S251" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-Nueis-TZEnz_78f8PYf</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
         </is>
       </c>
       <c r="T251" t="inlineStr">
@@ -27962,7 +27962,7 @@
       </c>
       <c r="U251" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="V251" t="n">
@@ -27983,12 +27983,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
+          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -27998,7 +27998,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
+          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -28016,12 +28016,12 @@
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -28040,54 +28040,52 @@
         </is>
       </c>
       <c r="N252" t="n">
+        <v>2</v>
+      </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
+        </is>
+      </c>
+      <c r="P252" t="inlineStr">
+        <is>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R252" t="inlineStr">
+        <is>
+          <t>10.21966/RZVW-4A72</t>
+        </is>
+      </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
+        </is>
+      </c>
+      <c r="T252" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="V252" t="n">
         <v>1</v>
       </c>
-      <c r="O252" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
-        </is>
-      </c>
-      <c r="P252" t="inlineStr">
-        <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q252" t="inlineStr">
-        <is>
-          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
-        </is>
-      </c>
-      <c r="R252" t="inlineStr">
-        <is>
-          <t>10.21966/dveq-bt48</t>
-        </is>
-      </c>
-      <c r="S252" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
-        </is>
-      </c>
-      <c r="T252" t="inlineStr">
-        <is>
-          <t>2026-04-15</t>
-        </is>
-      </c>
-      <c r="U252" t="inlineStr">
-        <is>
-          <t>2026-05-26</t>
-        </is>
-      </c>
-      <c r="V252" t="n">
-        <v>0</v>
-      </c>
       <c r="W252" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X252" t="n">
-        <v>2</v>
-      </c>
+          <t>[{'year': '2022', 'total': 1}]</t>
+        </is>
+      </c>
+      <c r="X252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -28095,12 +28093,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
+          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -28110,7 +28108,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
+          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -28128,7 +28126,7 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
@@ -28156,45 +28154,45 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
         </is>
       </c>
       <c r="P253" t="inlineStr">
         <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q253" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R253" t="inlineStr">
         <is>
-          <t>10.21966/RZVW-4A72</t>
+          <t>10.21966/0xvh-1318</t>
         </is>
       </c>
       <c r="S253" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
         </is>
       </c>
       <c r="T253" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="U253" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V253" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W253" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X253" t="inlineStr"/>
@@ -28205,12 +28203,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
+          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -28220,7 +28218,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
+          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
@@ -28238,12 +28236,12 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -28266,37 +28264,37 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
         </is>
       </c>
       <c r="P254" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q254" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
+          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R254" t="inlineStr">
         <is>
-          <t>10.21966/0xvh-1318</t>
+          <t>10.21966/3q5j-n957</t>
         </is>
       </c>
       <c r="S254" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
         </is>
       </c>
       <c r="T254" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="U254" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="V254" t="n">
@@ -28315,12 +28313,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
+          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -28330,7 +28328,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
+          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
@@ -28348,12 +28346,12 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -28372,41 +28370,41 @@
         </is>
       </c>
       <c r="N255" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
         </is>
       </c>
       <c r="P255" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q255" t="inlineStr">
         <is>
-          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
+          <t>invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R255" t="inlineStr">
         <is>
-          <t>10.21966/3q5j-n957</t>
+          <t>10.21966/kmc2-5r12</t>
         </is>
       </c>
       <c r="S255" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
         </is>
       </c>
       <c r="T255" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="U255" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="V255" t="n">
@@ -28425,12 +28423,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
+          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -28440,7 +28438,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
+          <t>Horne Lake Bathymetry Mapping</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -28458,7 +28456,7 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
@@ -28482,41 +28480,41 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
         </is>
       </c>
       <c r="P256" t="inlineStr">
         <is>
-          <t>[{'max': '30.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q256" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R256" t="inlineStr">
         <is>
-          <t>10.21966/kmc2-5r12</t>
+          <t>10.21966/vwee-e004</t>
         </is>
       </c>
       <c r="S256" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
         </is>
       </c>
       <c r="T256" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="U256" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V256" t="n">
@@ -28535,12 +28533,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
+          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -28550,7 +28548,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Horne Lake Bathymetry Mapping</t>
+          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -28568,7 +28566,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
@@ -28596,12 +28594,12 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
         </is>
       </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '475.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q257" t="inlineStr">
@@ -28611,12 +28609,12 @@
       </c>
       <c r="R257" t="inlineStr">
         <is>
-          <t>10.21966/vwee-e004</t>
+          <t>10.21966/k0z0-3z50</t>
         </is>
       </c>
       <c r="S257" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
         </is>
       </c>
       <c r="T257" t="inlineStr">
@@ -28626,7 +28624,7 @@
       </c>
       <c r="U257" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="V257" t="n">
@@ -28645,12 +28643,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
+          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -28660,7 +28658,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
+          <t>Knight Inlet Multibeam Bathymetry Survey</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -28678,7 +28676,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
@@ -28706,12 +28704,12 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
         </is>
       </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t>[{'max': '475.0', 'min': '0.0'}]</t>
+          <t>[{'max': '288.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q258" t="inlineStr">
@@ -28721,17 +28719,17 @@
       </c>
       <c r="R258" t="inlineStr">
         <is>
-          <t>10.21966/k0z0-3z50</t>
+          <t>10.21966/8dgz-1z27</t>
         </is>
       </c>
       <c r="S258" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
         </is>
       </c>
       <c r="T258" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="U258" t="inlineStr">
@@ -28755,12 +28753,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
+          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -28770,7 +28768,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Knight Inlet Multibeam Bathymetry Survey</t>
+          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -28788,7 +28786,7 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
@@ -28816,12 +28814,12 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
         </is>
       </c>
       <c r="P259" t="inlineStr">
         <is>
-          <t>[{'max': '288.0', 'min': '0.0'}]</t>
+          <t>[{'max': '450.0', 'min': '200.0'}]</t>
         </is>
       </c>
       <c r="Q259" t="inlineStr">
@@ -28831,12 +28829,12 @@
       </c>
       <c r="R259" t="inlineStr">
         <is>
-          <t>10.21966/8dgz-1z27</t>
+          <t>10.21966/g8f2-jw82</t>
         </is>
       </c>
       <c r="S259" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
         </is>
       </c>
       <c r="T259" t="inlineStr">
@@ -28865,12 +28863,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
+          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
+          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -28880,7 +28878,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -28926,12 +28924,12 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
         </is>
       </c>
       <c r="P260" t="inlineStr">
         <is>
-          <t>[{'max': '450.0', 'min': '200.0'}]</t>
+          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q260" t="inlineStr">
@@ -28941,22 +28939,22 @@
       </c>
       <c r="R260" t="inlineStr">
         <is>
-          <t>10.21966/g8f2-jw82</t>
+          <t>10.21966/n6ga-nc24</t>
         </is>
       </c>
       <c r="S260" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
         </is>
       </c>
       <c r="T260" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="U260" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="V260" t="n">
@@ -28975,12 +28973,12 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
+          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
+          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -28990,7 +28988,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
+          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -29008,7 +29006,7 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
@@ -29036,12 +29034,12 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
         </is>
       </c>
       <c r="P261" t="inlineStr">
         <is>
-          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q261" t="inlineStr">
@@ -29051,12 +29049,12 @@
       </c>
       <c r="R261" t="inlineStr">
         <is>
-          <t>10.21966/n6ga-nc24</t>
+          <t>10.21966/kn3e-fn08</t>
         </is>
       </c>
       <c r="S261" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
         </is>
       </c>
       <c r="T261" t="inlineStr">
@@ -29085,12 +29083,12 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
+          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
+          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -29100,7 +29098,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
+          <t>Sea surface temperature data in False Creek, British Columbia</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -29118,7 +29116,7 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
@@ -29146,37 +29144,37 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
         </is>
       </c>
       <c r="P262" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.5', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q262" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>seaSurfaceTemperature</t>
         </is>
       </c>
       <c r="R262" t="inlineStr">
         <is>
-          <t>10.21966/kn3e-fn08</t>
+          <t>10.21966/0g6d-pk30</t>
         </is>
       </c>
       <c r="S262" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
         </is>
       </c>
       <c r="T262" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="U262" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V262" t="n">
@@ -29195,12 +29193,12 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
+          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -29210,7 +29208,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Sea surface temperature data in False Creek, British Columbia</t>
+          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -29228,12 +29226,12 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -29256,37 +29254,37 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
         </is>
       </c>
       <c r="P263" t="inlineStr">
         <is>
-          <t>[{'max': '0.5', 'min': '0.5'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q263" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R263" t="inlineStr">
         <is>
-          <t>10.21966/0g6d-pk30</t>
+          <t>10.21966/03pw-2190</t>
         </is>
       </c>
       <c r="S263" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
         </is>
       </c>
       <c r="T263" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="U263" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V263" t="n">
@@ -29305,12 +29303,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
+          <t>ca-cioos_79368bf3-8f02-4355-837e-3a6cef0d2886</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -29320,7 +29318,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
+          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -29338,12 +29336,12 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -29362,11 +29360,11 @@
         </is>
       </c>
       <c r="N264" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P264" t="inlineStr">
@@ -29376,27 +29374,27 @@
       </c>
       <c r="Q264" t="inlineStr">
         <is>
-          <t>other, seagrassCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R264" t="inlineStr">
         <is>
-          <t>10.21966/03pw-2190</t>
+          <t>10.21966/c6xs-y324</t>
         </is>
       </c>
       <c r="S264" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OtAIe6lv3elLZd4c-V1</t>
         </is>
       </c>
       <c r="T264" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="U264" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="V264" t="n">
@@ -29415,12 +29413,12 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>ca-cioos_79368bf3-8f02-4355-837e-3a6cef0d2886</t>
+          <t>ca-cioos_d986aade-6bf1-4dfa-97c2-686975f944d5</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -29430,7 +29428,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Provisional)</t>
+          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Research)</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -29453,7 +29451,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -29476,12 +29474,12 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1, 51.64], [-128.0, 51.64], [-128.0, 51.67], [-128.1, 51.67], [-128.1, 51.64]]]}</t>
         </is>
       </c>
       <c r="P265" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q265" t="inlineStr">
@@ -29491,17 +29489,17 @@
       </c>
       <c r="R265" t="inlineStr">
         <is>
-          <t>10.21966/c6xs-y324</t>
+          <t>10.21966/47m7-ev69</t>
         </is>
       </c>
       <c r="S265" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OtAIe6lv3elLZd4c-V1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OHj73dBYs1okPPjDXKY</t>
         </is>
       </c>
       <c r="T265" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="U265" t="inlineStr">
@@ -29525,12 +29523,12 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>71c6db20-a521-451b-b371-a2560f6af25e</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>ca-cioos_d986aade-6bf1-4dfa-97c2-686975f944d5</t>
+          <t>ca-cioos_999da1dd-efde-4a55-868b-ce2d6ca3b983</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -29540,7 +29538,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Research)</t>
+          <t>Observations from the 2017 Hakai MarineGEO Bioblitz</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -29558,12 +29556,12 @@
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Genomics</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -29582,41 +29580,41 @@
         </is>
       </c>
       <c r="N266" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1, 51.64], [-128.0, 51.64], [-128.0, 51.67], [-128.1, 51.67], [-128.1, 51.64]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.951, 51.48631], [-127.76165, 51.48631], [-127.76165, 52.05347], [-128.951, 52.05347], [-128.951, 51.48631]]]}</t>
         </is>
       </c>
       <c r="P266" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '40.0', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q266" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R266" t="inlineStr">
         <is>
-          <t>10.21966/47m7-ev69</t>
+          <t>10.21966/0jfr-7b65</t>
         </is>
       </c>
       <c r="S266" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OHj73dBYs1okPPjDXKY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCmJU0B97JSOfOpj6J</t>
         </is>
       </c>
       <c r="T266" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="U266" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="V266" t="n">
@@ -29635,12 +29633,12 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>71c6db20-a521-451b-b371-a2560f6af25e</t>
+          <t>f0ae5f04-2c3a-4b67-8fbf-c6dc3771257d</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>ca-cioos_999da1dd-efde-4a55-868b-ce2d6ca3b983</t>
+          <t>ca-cioos_482d2463-0c81-4d62-a22a-1c0942b3c1fa</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -29650,7 +29648,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Observations from the 2017 Hakai MarineGEO Bioblitz</t>
+          <t>Observations from the 2019 Hakai Deep Water Bioblitz</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -29696,12 +29694,12 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.951, 51.48631], [-127.76165, 51.48631], [-127.76165, 52.05347], [-128.951, 52.05347], [-128.951, 51.48631]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.14433, 51.615734], [-127.76327, 51.615734], [-127.76327, 51.787], [-128.14433, 51.787], [-128.14433, 51.615734]]]}</t>
         </is>
       </c>
       <c r="P267" t="inlineStr">
         <is>
-          <t>[{'max': '40.0', 'min': '0.5'}]</t>
+          <t>[{'max': '255.0', 'min': '5.0'}]</t>
         </is>
       </c>
       <c r="Q267" t="inlineStr">
@@ -29711,22 +29709,22 @@
       </c>
       <c r="R267" t="inlineStr">
         <is>
-          <t>10.21966/0jfr-7b65</t>
+          <t>10.21966/3p06-vt55</t>
         </is>
       </c>
       <c r="S267" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCmJU0B97JSOfOpj6J</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCoStSubGWAdV78XNC</t>
         </is>
       </c>
       <c r="T267" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="U267" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="V267" t="n">
@@ -29745,12 +29743,12 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>f0ae5f04-2c3a-4b67-8fbf-c6dc3771257d</t>
+          <t>91d2ddf0-ea25-4ef9-b990-26d2957cb3bd</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>ca-cioos_482d2463-0c81-4d62-a22a-1c0942b3c1fa</t>
+          <t>ca-cioos_542a20b8-242e-4199-a062-5b76ea9cbf2d</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -29760,7 +29758,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Observations from the 2019 Hakai Deep Water Bioblitz</t>
+          <t>Observations from the 2018 Hakai Terrestrial Bioblitz</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
@@ -29806,27 +29804,27 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.14433, 51.615734], [-127.76327, 51.615734], [-127.76327, 51.787], [-128.14433, 51.787], [-128.14433, 51.615734]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.98366, 51.5919], [-125.0032, 51.5919], [-125.0032, 53.9998], [-128.98366, 53.9998], [-128.98366, 51.5919]]]}</t>
         </is>
       </c>
       <c r="P268" t="inlineStr">
         <is>
-          <t>[{'max': '255.0', 'min': '5.0'}]</t>
+          <t>[{'max': '1012.0', 'min': '50.0'}]</t>
         </is>
       </c>
       <c r="Q268" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R268" t="inlineStr">
         <is>
-          <t>10.21966/3p06-vt55</t>
+          <t>10.21966/t0h7-8g95</t>
         </is>
       </c>
       <c r="S268" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCoStSubGWAdV78XNC</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCpwd5hTju8QOKVY-E</t>
         </is>
       </c>
       <c r="T268" t="inlineStr">
@@ -29836,7 +29834,7 @@
       </c>
       <c r="U268" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V268" t="n">
@@ -29855,12 +29853,12 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>91d2ddf0-ea25-4ef9-b990-26d2957cb3bd</t>
+          <t>fa42f16a-3693-4c51-b45c-a36e709fdac3</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>ca-cioos_542a20b8-242e-4199-a062-5b76ea9cbf2d</t>
+          <t>ca-cioos_d69bf79e-b616-404e-bbfc-92932ca74087</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -29870,7 +29868,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Observations from the 2018 Hakai Terrestrial Bioblitz</t>
+          <t>Observations from the 2018 Hakai Seagrass Bioblitz</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -29888,7 +29886,7 @@
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>Genomics</t>
+          <t>Genomics, Nearshore</t>
         </is>
       </c>
       <c r="J269" t="inlineStr">
@@ -29916,27 +29914,27 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.98366, 51.5919], [-125.0032, 51.5919], [-125.0032, 53.9998], [-128.98366, 53.9998], [-128.98366, 51.5919]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.8123, 51.8438], [-128.2105, 51.684], [-128.1968, 51.6158], [-127.8837, 51.6192], [-127.8123, 51.8438]]]}</t>
         </is>
       </c>
       <c r="P269" t="inlineStr">
         <is>
-          <t>[{'max': '1012.0', 'min': '50.0'}]</t>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q269" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R269" t="inlineStr">
         <is>
-          <t>10.21966/t0h7-8g95</t>
+          <t>10.21966/yf1f-jx85</t>
         </is>
       </c>
       <c r="S269" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCpwd5hTju8QOKVY-E</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCnP9OAghmAmYObj0D</t>
         </is>
       </c>
       <c r="T269" t="inlineStr">
@@ -29946,7 +29944,7 @@
       </c>
       <c r="U269" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="V269" t="n">
@@ -29965,12 +29963,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>fa42f16a-3693-4c51-b45c-a36e709fdac3</t>
+          <t>fc3d2ea5-b60c-42c9-97e9-542024bec9fa</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>ca-cioos_d69bf79e-b616-404e-bbfc-92932ca74087</t>
+          <t>ca-cioos_4add33cd-b182-4825-900a-5695f333125a</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -29980,7 +29978,7 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Observations from the 2018 Hakai Seagrass Bioblitz</t>
+          <t>Weather Station Time Series, Hyacinthe Bay, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
@@ -29998,12 +29996,12 @@
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>Genomics, Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -30026,47 +30024,37 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.8123, 51.8438], [-128.2105, 51.684], [-128.1968, 51.6158], [-127.8837, 51.6192], [-127.8123, 51.8438]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.2221111, 50.1162556]}</t>
         </is>
       </c>
       <c r="P270" t="inlineStr">
         <is>
-          <t>[{'max': '300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q270" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution, seagrassCoverAndComposition</t>
-        </is>
-      </c>
-      <c r="R270" t="inlineStr">
-        <is>
-          <t>10.21966/yf1f-jx85</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R270" t="inlineStr"/>
       <c r="S270" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCnP9OAghmAmYObj0D</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OyesAm4pxUK1wqBMn7x</t>
         </is>
       </c>
       <c r="T270" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U270" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="V270" t="n">
-        <v>0</v>
-      </c>
-      <c r="W270" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="V270" t="inlineStr"/>
+      <c r="W270" t="inlineStr"/>
       <c r="X270" t="inlineStr"/>
     </row>
     <row r="271">
@@ -30075,12 +30063,12 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>fc3d2ea5-b60c-42c9-97e9-542024bec9fa</t>
+          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>ca-cioos_4add33cd-b182-4825-900a-5695f333125a</t>
+          <t>ca-cioos_3f40326a-23f9-4e30-a16a-f332ace14e2f</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -30090,7 +30078,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>Weather Station Time Series, Hyacinthe Bay, BC, Canada (Provisional)</t>
+          <t>Nereocystis kelp canopy productivity data from BC Central Coast</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
@@ -30108,12 +30096,12 @@
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -30136,37 +30124,47 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.2221111, 50.1162556]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.6, 51.19], [-127.1, 51.19], [-127.1, 52.28], [-128.6, 52.28], [-128.6, 51.19]]]}</t>
         </is>
       </c>
       <c r="P271" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q271" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R271" t="inlineStr"/>
+          <t>macroalgalCanopyCoverAndComposition</t>
+        </is>
+      </c>
+      <c r="R271" t="inlineStr">
+        <is>
+          <t>10.21966/d1s2-s530</t>
+        </is>
+      </c>
       <c r="S271" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OyesAm4pxUK1wqBMn7x</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/df5J7W5Hk4e0p4yvlOAI0qcU9Gs2/-MtG8b48aDAEdJoqNT6N</t>
         </is>
       </c>
       <c r="T271" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U271" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="V271" t="inlineStr"/>
-      <c r="W271" t="inlineStr"/>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="V271" t="n">
+        <v>1</v>
+      </c>
+      <c r="W271" t="inlineStr">
+        <is>
+          <t>[{'year': '2024', 'total': 1}]</t>
+        </is>
+      </c>
       <c r="X271" t="inlineStr"/>
     </row>
     <row r="272">
@@ -30175,12 +30173,12 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>aab940b9-bb7f-49c0-ae62-4f78d26897b3</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>ca-cioos_3f40326a-23f9-4e30-a16a-f332ace14e2f</t>
+          <t>ca-cioos_0219e1d6-8dfc-4718-b89b-ea3dff06a70d</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -30190,7 +30188,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Nereocystis kelp canopy productivity data from BC Central Coast</t>
+          <t>Modeled Eelgrass Extent, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
@@ -30208,12 +30206,12 @@
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -30232,49 +30230,49 @@
         </is>
       </c>
       <c r="N272" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.6, 51.19], [-127.1, 51.19], [-127.1, 52.28], [-128.6, 52.28], [-128.6, 51.19]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-133.7841801345348, 48.23443097294032], [-122.49023482203482, 48.23443097294032], [-122.49023482203482, 54.52958287232971], [-133.7841801345348, 54.52958287232971], [-133.7841801345348, 48.23443097294032]]]}</t>
         </is>
       </c>
       <c r="P272" t="inlineStr">
         <is>
-          <t>[{'max': '30.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q272" t="inlineStr">
         <is>
-          <t>macroalgalCanopyCoverAndComposition</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R272" t="inlineStr">
         <is>
-          <t>10.21966/d1s2-s530</t>
+          <t>10.21966/1ty5-e654</t>
         </is>
       </c>
       <c r="S272" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/df5J7W5Hk4e0p4yvlOAI0qcU9Gs2/-MtG8b48aDAEdJoqNT6N</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWtuNVpwdEdLRXZTODc</t>
         </is>
       </c>
       <c r="T272" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="U272" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="V272" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W272" t="inlineStr">
         <is>
-          <t>[{'year': '2024', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X272" t="inlineStr"/>
@@ -30285,12 +30283,12 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>aab940b9-bb7f-49c0-ae62-4f78d26897b3</t>
+          <t>3988f8e8-36ea-4cda-9bd9-a03157116ef5</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>ca-cioos_0219e1d6-8dfc-4718-b89b-ea3dff06a70d</t>
+          <t>ca-cioos_d43a79c1-a6ba-4e37-8dc2-6ced6312828e</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -30300,7 +30298,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>Modeled Eelgrass Extent, British Columbia, Canada</t>
+          <t>Data from Manuscript: Parasites of the hermit crab Pagurus hirsutiusculus; distribution, prevalence, and thermal ecology</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
@@ -30318,7 +30316,7 @@
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
@@ -30342,11 +30340,11 @@
         </is>
       </c>
       <c r="N273" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-133.7841801345348, 48.23443097294032], [-122.49023482203482, 48.23443097294032], [-122.49023482203482, 54.52958287232971], [-133.7841801345348, 54.52958287232971], [-133.7841801345348, 48.23443097294032]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.66], [-127.9, 51.81], [-122.2, 49.03], [-123.3, 49.01], [-123.0, 48.83], [-123.0, 48.78], [-123.3, 48.7], [-123.3, 48.53], [-123.6, 48.59], [-125.2, 48.73], [-125.6, 48.95], [-125.6, 50.11], [-128.4, 51.66]]]}</t>
         </is>
       </c>
       <c r="P273" t="inlineStr">
@@ -30356,17 +30354,17 @@
       </c>
       <c r="Q273" t="inlineStr">
         <is>
-          <t>other, seagrassCoverAndComposition</t>
+          <t>invertebrateAbundanceAndDistribution, seaSurfaceSalinity</t>
         </is>
       </c>
       <c r="R273" t="inlineStr">
         <is>
-          <t>10.21966/1ty5-e654</t>
+          <t>10.21966/xb3t-qb88</t>
         </is>
       </c>
       <c r="S273" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWtuNVpwdEdLRXZTODc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3eh7IMAvm8ZUtcMBeifFL0eJCIA3/-O5Kei32z9cfatfgKj5y</t>
         </is>
       </c>
       <c r="T273" t="inlineStr">
@@ -30376,7 +30374,7 @@
       </c>
       <c r="U273" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="V273" t="n">
@@ -30395,12 +30393,12 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>3988f8e8-36ea-4cda-9bd9-a03157116ef5</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>ca-cioos_d43a79c1-a6ba-4e37-8dc2-6ced6312828e</t>
+          <t>ca-cioos_53189107-9df5-426b-acb4-f903468554fe</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -30410,7 +30408,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Data from Manuscript: Parasites of the hermit crab Pagurus hirsutiusculus; distribution, prevalence, and thermal ecology</t>
+          <t>Comparing invertebrate and seaweed diversity in kelp forests and urchin barrens in Owen Bay, British Columbia, using Autonomous Reef Monitoring Structures (ARMS)</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -30428,7 +30426,7 @@
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Sentinels of Change, Genomics</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
@@ -30452,41 +30450,41 @@
         </is>
       </c>
       <c r="N274" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.66], [-127.9, 51.81], [-122.2, 49.03], [-123.3, 49.01], [-123.0, 48.83], [-123.0, 48.78], [-123.3, 48.7], [-123.3, 48.53], [-123.6, 48.59], [-125.2, 48.73], [-125.6, 48.95], [-125.6, 50.11], [-128.4, 51.66]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.2335, 50.2999], [-125.2163, 50.2999], [-125.2163, 50.313], [-125.2335, 50.313], [-125.2335, 50.2999]]]}</t>
         </is>
       </c>
       <c r="P274" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '6.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q274" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, seaSurfaceSalinity</t>
+          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R274" t="inlineStr">
         <is>
-          <t>10.21966/xb3t-qb88</t>
+          <t>10.21966/e5mw-tr82</t>
         </is>
       </c>
       <c r="S274" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3eh7IMAvm8ZUtcMBeifFL0eJCIA3/-O5Kei32z9cfatfgKj5y</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/5Jh4rsxoBsRd4mVFqZ0XJoMtMHI2/-P-tq8uNjGhWtk4rBny0</t>
         </is>
       </c>
       <c r="T274" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="U274" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="V274" t="n">
@@ -30497,7 +30495,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X274" t="inlineStr"/>
+      <c r="X274" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -30505,12 +30505,12 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>ca-cioos_53189107-9df5-426b-acb4-f903468554fe</t>
+          <t>ca-cioos_73abfecf-d35c-4f9c-a991-eee5cece08ea</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -30520,7 +30520,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>Comparing invertebrate and seaweed diversity in kelp forests and urchin barrens in Owen Bay, British Columbia, using Autonomous Reef Monitoring Structures (ARMS)</t>
+          <t>Kelp Canopy Extent 2012 - NW Calvert Island</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -30538,7 +30538,7 @@
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>Sentinels of Change, Genomics</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
@@ -30562,41 +30562,41 @@
         </is>
       </c>
       <c r="N275" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.2335, 50.2999], [-125.2163, 50.2999], [-125.2163, 50.313], [-125.2335, 50.313], [-125.2335, 50.2999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16959381103513, 51.63613234359897], [-128.11191558837888, 51.63613234359897], [-128.11191558837888, 51.681709494104325], [-128.16959381103513, 51.681709494104325], [-128.16959381103513, 51.63613234359897]]]}</t>
         </is>
       </c>
       <c r="P275" t="inlineStr">
         <is>
-          <t>[{'max': '6.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q275" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
+          <t>other, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R275" t="inlineStr">
         <is>
-          <t>10.21966/e5mw-tr82</t>
+          <t>10.21966/63rs-yt91</t>
         </is>
       </c>
       <c r="S275" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/5Jh4rsxoBsRd4mVFqZ0XJoMtMHI2/-P-tq8uNjGhWtk4rBny0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxUM01laTFaREhKbWE</t>
         </is>
       </c>
       <c r="T275" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="U275" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="V275" t="n">
@@ -30617,12 +30617,12 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
+          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>ca-cioos_73abfecf-d35c-4f9c-a991-eee5cece08ea</t>
+          <t>ca-cioos_940218ef-d7f8-4f3f-9e69-52150ecdbec5</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -30632,7 +30632,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Kelp Canopy Extent 2012 - NW Calvert Island</t>
+          <t>North Vancouver Island Aerial Survey - 2024 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -30650,7 +30650,7 @@
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
@@ -30674,31 +30674,31 @@
         </is>
       </c>
       <c r="N276" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16959381103513, 51.63613234359897], [-128.11191558837888, 51.63613234359897], [-128.11191558837888, 51.681709494104325], [-128.16959381103513, 51.681709494104325], [-128.16959381103513, 51.63613234359897]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.7, 50.35], [-125.4, 50.35], [-125.4, 50.63], [-126.7, 50.63], [-126.7, 50.35]]]}</t>
         </is>
       </c>
       <c r="P276" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q276" t="inlineStr">
         <is>
-          <t>other, macroalgalCanopyCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R276" t="inlineStr">
         <is>
-          <t>10.21966/63rs-yt91</t>
+          <t>10.21966/kdhe-hz07</t>
         </is>
       </c>
       <c r="S276" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxUM01laTFaREhKbWE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OCoHpqOwDbp834fqRY3</t>
         </is>
       </c>
       <c r="T276" t="inlineStr">
@@ -30708,7 +30708,7 @@
       </c>
       <c r="U276" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="V276" t="n">
@@ -30729,12 +30729,12 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
+          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>ca-cioos_940218ef-d7f8-4f3f-9e69-52150ecdbec5</t>
+          <t>ca-cioos_c7466354-bacc-4781-acdc-543dd03d1eab</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -30744,7 +30744,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>North Vancouver Island Aerial Survey - 2024 - Airborne Coastal Observatory</t>
+          <t>Nanwakolas LiDAR Surveys - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -30790,12 +30790,12 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.7, 50.35], [-125.4, 50.35], [-125.4, 50.63], [-126.7, 50.63], [-126.7, 50.35]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.8, 49.26], [-124.5, 49.26], [-124.5, 50.83], [-126.8, 50.83], [-126.8, 49.26]]]}</t>
         </is>
       </c>
       <c r="P277" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1700.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q277" t="inlineStr">
@@ -30805,12 +30805,12 @@
       </c>
       <c r="R277" t="inlineStr">
         <is>
-          <t>10.21966/kdhe-hz07</t>
+          <t>10.21966/e0r7-ge27</t>
         </is>
       </c>
       <c r="S277" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OCoHpqOwDbp834fqRY3</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OjbuSE_uZcCs3Fit_mg</t>
         </is>
       </c>
       <c r="T277" t="inlineStr">
@@ -30820,7 +30820,7 @@
       </c>
       <c r="U277" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="V277" t="n">
@@ -30839,12 +30839,12 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
+          <t>f7433c1a-3aad-4761-81c4-c191a5e6ac92</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>ca-cioos_c7466354-bacc-4781-acdc-543dd03d1eab</t>
+          <t>ca-cioos_52e97374-bee5-4b1a-9b85-7170a5df8d6b</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -30854,7 +30854,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Nanwakolas LiDAR Surveys - Airborne Coastal Observatory</t>
+          <t>Biomass and density of Pycnopodia helianthoides from the central coast of BC</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -30872,7 +30872,7 @@
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Oceanography, Nearshore</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
@@ -30900,37 +30900,37 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.8, 49.26], [-124.5, 49.26], [-124.5, 50.83], [-126.8, 50.83], [-126.8, 49.26]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.617, 51.3321], [-127.3509, 51.3321], [-127.3509, 52.3317], [-128.617, 52.3317], [-128.617, 51.3321]]]}</t>
         </is>
       </c>
       <c r="P278" t="inlineStr">
         <is>
-          <t>[{'max': '1700.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q278" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>seaSurfaceSalinity, subSurfaceSalinity, seaSurfaceTemperature, subSurfaceTemperature, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R278" t="inlineStr">
         <is>
-          <t>10.21966/e0r7-ge27</t>
+          <t>10.21966/xy6n-qz76</t>
         </is>
       </c>
       <c r="S278" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OjbuSE_uZcCs3Fit_mg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-OteEfuBSvhg-2RySC4a</t>
         </is>
       </c>
       <c r="T278" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="U278" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="V278" t="n">
@@ -30949,12 +30949,12 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>f7433c1a-3aad-4761-81c4-c191a5e6ac92</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>ca-cioos_52e97374-bee5-4b1a-9b85-7170a5df8d6b</t>
+          <t>ca-cioos_b4844ae2-d9c1-42f2-ae4d-a8f994c395a0</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -30964,7 +30964,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Biomass and density of Pycnopodia helianthoides from the central coast of BC</t>
+          <t>Putting fjord biodiversity on the map for British Columbia conservation planning</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -30982,7 +30982,7 @@
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>Oceanography, Nearshore</t>
+          <t>Genomics, Oceanography</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
@@ -31002,56 +31002,58 @@
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N279" t="n">
+        <v>2</v>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.0471, 52.2577], [-128.9141, 51.7033], [-127.6841, 50.7687], [-123.7744, 48.9864], [-122.764, 49.331], [-122.8299, 49.9706], [-127.0471, 52.2577]]]}</t>
+        </is>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t>[{'max': '595.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>fishAbundanceAndDistribution, subSurfaceTemperature, subSurfaceSalinity</t>
+        </is>
+      </c>
+      <c r="R279" t="inlineStr">
+        <is>
+          <t>10.21966/n141-m959</t>
+        </is>
+      </c>
+      <c r="S279" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-Ow-ZgW1jkC5-WyrtlLV</t>
+        </is>
+      </c>
+      <c r="T279" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="U279" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="V279" t="n">
+        <v>0</v>
+      </c>
+      <c r="W279" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X279" t="n">
         <v>1</v>
       </c>
-      <c r="O279" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.617, 51.3321], [-127.3509, 51.3321], [-127.3509, 52.3317], [-128.617, 52.3317], [-128.617, 51.3321]]]}</t>
-        </is>
-      </c>
-      <c r="P279" t="inlineStr">
-        <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q279" t="inlineStr">
-        <is>
-          <t>seaSurfaceSalinity, subSurfaceSalinity, seaSurfaceTemperature, subSurfaceTemperature, invertebrateAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R279" t="inlineStr">
-        <is>
-          <t>10.21966/xy6n-qz76</t>
-        </is>
-      </c>
-      <c r="S279" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-OteEfuBSvhg-2RySC4a</t>
-        </is>
-      </c>
-      <c r="T279" t="inlineStr">
-        <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="U279" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="V279" t="n">
-        <v>0</v>
-      </c>
-      <c r="W279" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -31059,12 +31061,12 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>ca-cioos_b4844ae2-d9c1-42f2-ae4d-a8f994c395a0</t>
+          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -31074,7 +31076,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Putting fjord biodiversity on the map for British Columbia conservation planning</t>
+          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -31092,7 +31094,7 @@
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>Genomics, Oceanography</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
@@ -31112,45 +31114,45 @@
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N280" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.0471, 52.2577], [-128.9141, 51.7033], [-127.6841, 50.7687], [-123.7744, 48.9864], [-122.764, 49.331], [-122.8299, 49.9706], [-127.0471, 52.2577]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
         </is>
       </c>
       <c r="P280" t="inlineStr">
         <is>
-          <t>[{'max': '595.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2.5', 'min': '2.5'}]</t>
         </is>
       </c>
       <c r="Q280" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, subSurfaceTemperature, subSurfaceSalinity</t>
+          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
         </is>
       </c>
       <c r="R280" t="inlineStr">
         <is>
-          <t>10.21966/n141-m959</t>
+          <t>10.21966/rrzq-yw32</t>
         </is>
       </c>
       <c r="S280" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-Ow-ZgW1jkC5-WyrtlLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
         </is>
       </c>
       <c r="T280" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="U280" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="V280" t="n">
@@ -31161,9 +31163,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X280" t="n">
-        <v>1</v>
-      </c>
+      <c r="X280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -31171,12 +31171,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
+          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -31186,17 +31186,17 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
+          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>collection</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H281" t="b">
@@ -31209,7 +31209,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -31232,27 +31232,23 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
         </is>
       </c>
       <c r="P281" t="inlineStr">
         <is>
-          <t>[{'max': '2.5', 'min': '2.5'}]</t>
+          <t>[{'max': '0.0', 'min': '600.0'}]</t>
         </is>
       </c>
       <c r="Q281" t="inlineStr">
         <is>
-          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R281" t="inlineStr">
-        <is>
-          <t>10.21966/rrzq-yw32</t>
-        </is>
-      </c>
+          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr"/>
       <c r="S281" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
         </is>
       </c>
       <c r="T281" t="inlineStr">
@@ -31262,17 +31258,11 @@
       </c>
       <c r="U281" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="V281" t="n">
-        <v>0</v>
-      </c>
-      <c r="W281" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="V281" t="inlineStr"/>
+      <c r="W281" t="inlineStr"/>
       <c r="X281" t="inlineStr"/>
     </row>
     <row r="282">
@@ -31281,12 +31271,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
+          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -31296,17 +31286,17 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
+          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>collection</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H282" t="b">
@@ -31314,12 +31304,12 @@
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Estuary Resilience</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -31342,40 +31332,48 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
         </is>
       </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '600.0'}]</t>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
         </is>
       </c>
       <c r="Q282" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R282" t="inlineStr"/>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr">
+        <is>
+          <t>10.21966/r9zr-xz33</t>
+        </is>
+      </c>
       <c r="S282" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
         </is>
       </c>
       <c r="T282" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="U282" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="V282" t="inlineStr"/>
-      <c r="W282" t="inlineStr"/>
-      <c r="X282" t="n">
-        <v>2</v>
-      </c>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="V282" t="n">
+        <v>0</v>
+      </c>
+      <c r="W282" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="n">
@@ -31383,12 +31381,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
+          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
+          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -31398,7 +31396,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -31444,7 +31442,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
         </is>
       </c>
       <c r="P283" t="inlineStr">
@@ -31459,12 +31457,12 @@
       </c>
       <c r="R283" t="inlineStr">
         <is>
-          <t>10.21966/r9zr-xz33</t>
+          <t>10.21966/9dbb-5d54</t>
         </is>
       </c>
       <c r="S283" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
         </is>
       </c>
       <c r="T283" t="inlineStr">
@@ -31493,12 +31491,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
+          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
+          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -31508,7 +31506,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -31554,7 +31552,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
         </is>
       </c>
       <c r="P284" t="inlineStr">
@@ -31569,12 +31567,12 @@
       </c>
       <c r="R284" t="inlineStr">
         <is>
-          <t>10.21966/9dbb-5d54</t>
+          <t>10.21966/vpz7-mm73</t>
         </is>
       </c>
       <c r="S284" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
         </is>
       </c>
       <c r="T284" t="inlineStr">
@@ -31603,12 +31601,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
+          <t>0ce3ee5b-425b-4eb0-a201-96bdfb795a3f</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
+          <t>ca-cioos_354b5b83-e752-4ffb-a740-d1cdc02ac8c6</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -31618,7 +31616,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Dtlaxsiwè River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -31664,7 +31662,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.1721, 50.61011], [-127.17933, 50.612], [-127.1873, 50.6098], [-127.19703, 50.61072], [-127.20524, 50.61585], [-127.19007, 50.61844], [-127.18675, 50.61393], [-127.17744, 50.61359], [-127.17161, 50.61118], [-127.17203, 50.61011], [-127.1721, 50.61011]]]}</t>
         </is>
       </c>
       <c r="P285" t="inlineStr">
@@ -31679,12 +31677,12 @@
       </c>
       <c r="R285" t="inlineStr">
         <is>
-          <t>10.21966/vpz7-mm73</t>
+          <t>10.21966/ydm2-m238</t>
         </is>
       </c>
       <c r="S285" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7Dng-ZtRd05hnZCq1</t>
         </is>
       </c>
       <c r="T285" t="inlineStr">
@@ -31713,12 +31711,12 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>0ce3ee5b-425b-4eb0-a201-96bdfb795a3f</t>
+          <t>1a2aa5c8-9a83-46f7-967d-1127436c2084</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>ca-cioos_354b5b83-e752-4ffb-a740-d1cdc02ac8c6</t>
+          <t>ca-cioos_58a5140a-0b2c-4186-a648-53d9f58e5226</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -31728,7 +31726,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Dtlaxsiwè River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kvai River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -31774,7 +31772,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.1721, 50.61011], [-127.17933, 50.612], [-127.1873, 50.6098], [-127.19703, 50.61072], [-127.20524, 50.61585], [-127.19007, 50.61844], [-127.18675, 50.61393], [-127.17744, 50.61359], [-127.17161, 50.61118], [-127.17203, 50.61011], [-127.1721, 50.61011]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.81882, 51.77547], [-127.83122, 51.77986], [-127.85192, 51.781], [-127.86785, 51.78358], [-127.8958, 51.77366], [-127.89418, 51.77118], [-127.87834, 51.77309], [-127.86508, 51.77748], [-127.84009, 51.77519], [-127.82731, 51.77452], [-127.82025, 51.77309], [-127.81853, 51.77566], [-127.81882, 51.77547]]]}</t>
         </is>
       </c>
       <c r="P286" t="inlineStr">
@@ -31789,12 +31787,12 @@
       </c>
       <c r="R286" t="inlineStr">
         <is>
-          <t>10.21966/ydm2-m238</t>
+          <t>10.21966/pm9m-h431</t>
         </is>
       </c>
       <c r="S286" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7Dng-ZtRd05hnZCq1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7QQE3ifLCAPcu3Jih</t>
         </is>
       </c>
       <c r="T286" t="inlineStr">
@@ -31823,12 +31821,12 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>1a2aa5c8-9a83-46f7-967d-1127436c2084</t>
+          <t>c035b81c-0fc3-446e-bec5-8b8933ae874b</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>ca-cioos_58a5140a-0b2c-4186-a648-53d9f58e5226</t>
+          <t>ca-cioos_7fbc28f7-ee87-4361-bbee-0ed8ce24522d</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -31838,7 +31836,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kvai River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Gwa'dzi River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -31884,7 +31882,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.81882, 51.77547], [-127.83122, 51.77986], [-127.85192, 51.781], [-127.86785, 51.78358], [-127.8958, 51.77366], [-127.89418, 51.77118], [-127.87834, 51.77309], [-127.86508, 51.77748], [-127.84009, 51.77519], [-127.82731, 51.77452], [-127.82025, 51.77309], [-127.81853, 51.77566], [-127.81882, 51.77547]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.46176, 50.74217], [-127.49022, 50.72165], [-127.49167, 50.71188], [-127.4832, 50.70356], [-127.4874, 50.69181], [-127.46443, 50.6928], [-127.47282, 50.70776], [-127.47992, 50.71424], [-127.48305, 50.72058], [-127.45901, 50.74011], [-127.46153, 50.74217], [-127.46176, 50.74217]]]}</t>
         </is>
       </c>
       <c r="P287" t="inlineStr">
@@ -31899,12 +31897,12 @@
       </c>
       <c r="R287" t="inlineStr">
         <is>
-          <t>10.21966/pm9m-h431</t>
+          <t>10.21966/xq99-x273</t>
         </is>
       </c>
       <c r="S287" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7QQE3ifLCAPcu3Jih</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7BCRnF2C30YPkxIyd</t>
         </is>
       </c>
       <c r="T287" t="inlineStr">
@@ -31933,12 +31931,12 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>c035b81c-0fc3-446e-bec5-8b8933ae874b</t>
+          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>ca-cioos_7fbc28f7-ee87-4361-bbee-0ed8ce24522d</t>
+          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -31948,7 +31946,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Gwa'dzi River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -31994,7 +31992,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.46176, 50.74217], [-127.49022, 50.72165], [-127.49167, 50.71188], [-127.4832, 50.70356], [-127.4874, 50.69181], [-127.46443, 50.6928], [-127.47282, 50.70776], [-127.47992, 50.71424], [-127.48305, 50.72058], [-127.45901, 50.74011], [-127.46153, 50.74217], [-127.46176, 50.74217]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
         </is>
       </c>
       <c r="P288" t="inlineStr">
@@ -32009,12 +32007,12 @@
       </c>
       <c r="R288" t="inlineStr">
         <is>
-          <t>10.21966/xq99-x273</t>
+          <t>10.21966/kde9-8g12</t>
         </is>
       </c>
       <c r="S288" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7BCRnF2C30YPkxIyd</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
         </is>
       </c>
       <c r="T288" t="inlineStr">
@@ -32043,12 +32041,12 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
+          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
+          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -32058,7 +32056,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -32104,7 +32102,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
         </is>
       </c>
       <c r="P289" t="inlineStr">
@@ -32119,12 +32117,12 @@
       </c>
       <c r="R289" t="inlineStr">
         <is>
-          <t>10.21966/kde9-8g12</t>
+          <t>10.21966/9a97-2j48</t>
         </is>
       </c>
       <c r="S289" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
         </is>
       </c>
       <c r="T289" t="inlineStr">
@@ -32153,12 +32151,12 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
+          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
+          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -32168,7 +32166,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -32214,7 +32212,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
         </is>
       </c>
       <c r="P290" t="inlineStr">
@@ -32229,12 +32227,12 @@
       </c>
       <c r="R290" t="inlineStr">
         <is>
-          <t>10.21966/9a97-2j48</t>
+          <t>10.21966/ed9w-2653</t>
         </is>
       </c>
       <c r="S290" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
         </is>
       </c>
       <c r="T290" t="inlineStr">
@@ -32263,12 +32261,12 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
+          <t>1af6a43a-e73b-4774-8e10-b9f2928ab133</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
+          <t>ca-cioos_ae7e017c-9211-4f98-b56e-90a4bbac161c</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -32278,7 +32276,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Snuneymuxw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -32324,7 +32322,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.88685, 49.19332], [-123.92494, 49.1612], [-123.92581, 49.13841], [-123.91159, 49.123], [-123.88023, 49.11117], [-123.85971, 49.12766], [-123.89792, 49.16196], [-123.88099, 49.18866], [-123.88685, 49.19332]]]}</t>
         </is>
       </c>
       <c r="P291" t="inlineStr">
@@ -32339,12 +32337,12 @@
       </c>
       <c r="R291" t="inlineStr">
         <is>
-          <t>10.21966/ed9w-2653</t>
+          <t>10.21966/k01q-wb27</t>
         </is>
       </c>
       <c r="S291" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt459vxCIH7YPRN9fp</t>
         </is>
       </c>
       <c r="T291" t="inlineStr">
@@ -32373,12 +32371,12 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>1af6a43a-e73b-4774-8e10-b9f2928ab133</t>
+          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>ca-cioos_ae7e017c-9211-4f98-b56e-90a4bbac161c</t>
+          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -32388,7 +32386,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Snuneymuxw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
@@ -32434,7 +32432,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.88685, 49.19332], [-123.92494, 49.1612], [-123.92581, 49.13841], [-123.91159, 49.123], [-123.88023, 49.11117], [-123.85971, 49.12766], [-123.89792, 49.16196], [-123.88099, 49.18866], [-123.88685, 49.19332]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635], [-123.66843, 48.91641]]]}</t>
         </is>
       </c>
       <c r="P292" t="inlineStr">
@@ -32449,12 +32447,12 @@
       </c>
       <c r="R292" t="inlineStr">
         <is>
-          <t>10.21966/k01q-wb27</t>
+          <t>10.21966/q2e0-j004</t>
         </is>
       </c>
       <c r="S292" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt459vxCIH7YPRN9fp</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
         </is>
       </c>
       <c r="T292" t="inlineStr">
@@ -32483,12 +32481,12 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
+          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
+          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -32498,7 +32496,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
@@ -32544,7 +32542,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635], [-123.66843, 48.91641]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
         </is>
       </c>
       <c r="P293" t="inlineStr">
@@ -32559,12 +32557,12 @@
       </c>
       <c r="R293" t="inlineStr">
         <is>
-          <t>10.21966/q2e0-j004</t>
+          <t>10.21966/hjkj-6611</t>
         </is>
       </c>
       <c r="S293" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
         </is>
       </c>
       <c r="T293" t="inlineStr">
@@ -32593,12 +32591,12 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
+          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
+          <t>ca-cioos_dce15b7b-3772-4106-ab20-c3979c4c3f57</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -32608,7 +32606,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Fulmore River - Shoal Creek Estuary Complex (Provisional)</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -32654,7 +32652,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.08798, 50.4777], [-126.09599, 50.48418], [-126.09046, 50.50918], [-126.0647, 50.52425], [-125.99698, 50.53569], [-125.93459, 50.56717], [-125.93173, 50.56202], [-125.93764, 50.55458], [-125.91055, 50.55134], [-125.89853, 50.54943], [-125.90063, 50.54466], [-125.96416, 50.53989], [-125.98973, 50.52043], [-126.06566, 50.5067], [-126.08779, 50.47789], [-126.08798, 50.4777]]]}</t>
         </is>
       </c>
       <c r="P294" t="inlineStr">
@@ -32669,12 +32667,12 @@
       </c>
       <c r="R294" t="inlineStr">
         <is>
-          <t>10.21966/hjkj-6611</t>
+          <t>10.21966/g1cn-xs92</t>
         </is>
       </c>
       <c r="S294" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptdJ8iUmLeOrdmqzrQ</t>
         </is>
       </c>
       <c r="T294" t="inlineStr">
@@ -32703,12 +32701,12 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
+          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>ca-cioos_dce15b7b-3772-4106-ab20-c3979c4c3f57</t>
+          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
@@ -32718,7 +32716,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Fulmore River - Shoal Creek Estuary Complex (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -32764,7 +32762,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.08798, 50.4777], [-126.09599, 50.48418], [-126.09046, 50.50918], [-126.0647, 50.52425], [-125.99698, 50.53569], [-125.93459, 50.56717], [-125.93173, 50.56202], [-125.93764, 50.55458], [-125.91055, 50.55134], [-125.89853, 50.54943], [-125.90063, 50.54466], [-125.96416, 50.53989], [-125.98973, 50.52043], [-126.06566, 50.5067], [-126.08779, 50.47789], [-126.08798, 50.4777]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
         </is>
       </c>
       <c r="P295" t="inlineStr">
@@ -32779,12 +32777,12 @@
       </c>
       <c r="R295" t="inlineStr">
         <is>
-          <t>10.21966/g1cn-xs92</t>
+          <t>10.21966/npe4-3036</t>
         </is>
       </c>
       <c r="S295" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptdJ8iUmLeOrdmqzrQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
         </is>
       </c>
       <c r="T295" t="inlineStr">
@@ -32813,12 +32811,12 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
+          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
+          <t>ca-cioos_e9b72149-8cf1-4000-ae3e-6b29ad60b078</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -32828,7 +32826,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Malksope River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -32874,7 +32872,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.46569, 50.12556], [-127.45723, 50.13142], [-127.43281, 50.13338], [-127.42845, 50.13765], [-127.41181, 50.14408], [-127.40973, 50.14233], [-127.41999, 50.13627], [-127.41803, 50.13195], [-127.43106, 50.12796], [-127.46545, 50.12446], [-127.46569, 50.12548], [-127.46569, 50.12556]]]}</t>
         </is>
       </c>
       <c r="P296" t="inlineStr">
@@ -32889,12 +32887,12 @@
       </c>
       <c r="R296" t="inlineStr">
         <is>
-          <t>10.21966/npe4-3036</t>
+          <t>10.21966/21sf-ey03</t>
         </is>
       </c>
       <c r="S296" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq77iyWJfPg4z-FvOSb</t>
         </is>
       </c>
       <c r="T296" t="inlineStr">
@@ -32923,12 +32921,12 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
+          <t>5177d019-598e-4415-b778-9688403652c8</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>ca-cioos_e9b72149-8cf1-4000-ae3e-6b29ad60b078</t>
+          <t>ca-cioos_ed84df74-5a2d-4a7d-87c8-a7b93f11088e</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
@@ -32938,7 +32936,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Malksope River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Nalaxdlala River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -32984,7 +32982,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.46569, 50.12556], [-127.45723, 50.13142], [-127.43281, 50.13338], [-127.42845, 50.13765], [-127.41181, 50.14408], [-127.40973, 50.14233], [-127.41999, 50.13627], [-127.41803, 50.13195], [-127.43106, 50.12796], [-127.46545, 50.12446], [-127.46569, 50.12548], [-127.46569, 50.12556]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.9489, 50.70902], [-125.9696, 50.70291], [-126.00938, 50.69118], [-126.00108, 50.66848], [-125.98257, 50.68374], [-125.98152, 50.69271], [-125.95462, 50.70263], [-125.94785, 50.70768], [-125.9489, 50.70911], [-125.9489, 50.70902]]]}</t>
         </is>
       </c>
       <c r="P297" t="inlineStr">
@@ -32999,12 +32997,12 @@
       </c>
       <c r="R297" t="inlineStr">
         <is>
-          <t>10.21966/21sf-ey03</t>
+          <t>10.21966/4krv-aw23</t>
         </is>
       </c>
       <c r="S297" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq77iyWJfPg4z-FvOSb</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptbxmpkBsfyWWfSxOJ</t>
         </is>
       </c>
       <c r="T297" t="inlineStr">
@@ -33033,12 +33031,12 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>5177d019-598e-4415-b778-9688403652c8</t>
+          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>ca-cioos_ed84df74-5a2d-4a7d-87c8-a7b93f11088e</t>
+          <t>ca-cioos_b922699f-69b6-4d63-b538-7c290086a408</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
@@ -33048,7 +33046,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Nalaxdlala River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Quw'utsun/Xwulqw'selu River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
@@ -33094,7 +33092,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.9489, 50.70902], [-125.9696, 50.70291], [-126.00938, 50.69118], [-126.00108, 50.66848], [-125.98257, 50.68374], [-125.98152, 50.69271], [-125.95462, 50.70263], [-125.94785, 50.70768], [-125.9489, 50.70911], [-125.9489, 50.70902]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.56201, 48.73508], [-123.59772, 48.75559], [-123.62127, 48.76514], [-123.63885, 48.77426], [-123.66935, 48.78033], [-123.67901, 48.75472], [-123.65155, 48.74322], [-123.63017, 48.7405], [-123.60792, 48.74289], [-123.56494, 48.72987], [-123.56179, 48.73529], [-123.56201, 48.73508]]]}</t>
         </is>
       </c>
       <c r="P298" t="inlineStr">
@@ -33109,17 +33107,17 @@
       </c>
       <c r="R298" t="inlineStr">
         <is>
-          <t>10.21966/4krv-aw23</t>
+          <t>10.21966/2ha7-9p26</t>
         </is>
       </c>
       <c r="S298" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptbxmpkBsfyWWfSxOJ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpsCA3ycwZ7bFTDIQxh</t>
         </is>
       </c>
       <c r="T298" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="U298" t="inlineStr">
@@ -33143,12 +33141,12 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
+          <t>dd471e82-a6b8-4f32-891c-bbea26e9998e</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>ca-cioos_b922699f-69b6-4d63-b538-7c290086a408</t>
+          <t>ca-cioos_aeb30028-a7eb-462e-ac0f-6c5fe101d4a2</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
@@ -33158,7 +33156,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Quw'utsun/Xwulqw'selu River Estuary (Provisional)</t>
+          <t>DNA Metabarcoding Captures Temporal and Vertical Dynamics of Mesozooplankton Communities</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -33176,12 +33174,12 @@
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>Estuary Resilience</t>
+          <t>Genomics, Oceanography</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -33196,45 +33194,45 @@
       </c>
       <c r="M299" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N299" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.56201, 48.73508], [-123.59772, 48.75559], [-123.62127, 48.76514], [-123.63885, 48.77426], [-123.66935, 48.78033], [-123.67901, 48.75472], [-123.65155, 48.74322], [-123.63017, 48.7405], [-123.60792, 48.74289], [-123.56494, 48.72987], [-123.56179, 48.73529], [-123.56201, 48.73508]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.0992, 50.0307]}</t>
         </is>
       </c>
       <c r="P299" t="inlineStr">
         <is>
-          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+          <t>[{'max': '260.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q299" t="inlineStr">
         <is>
-          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
+          <t>zooplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R299" t="inlineStr">
         <is>
-          <t>10.21966/2ha7-9p26</t>
+          <t>10.21966/6b20-7r76</t>
         </is>
       </c>
       <c r="S299" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpsCA3ycwZ7bFTDIQxh</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OvzbmseH_syBXg1RXKd</t>
         </is>
       </c>
       <c r="T299" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="U299" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="V299" t="n">
@@ -33253,12 +33251,12 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>dd471e82-a6b8-4f32-891c-bbea26e9998e</t>
+          <t>b27bb6f9-49ae-4f3a-a02a-098d8edf23e2</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>ca-cioos_aeb30028-a7eb-462e-ac0f-6c5fe101d4a2</t>
+          <t>ca-cioos_ac765dbb-8e47-415d-8685-d9090946b86b</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
@@ -33268,7 +33266,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>DNA Metabarcoding Captures Temporal and Vertical Dynamics of Mesozooplankton Communities</t>
+          <t>Micro-invertebrate DNA Barcodes from Quadra Island, BC (Biomarathon)</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -33286,7 +33284,7 @@
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>Genomics, Oceanography</t>
+          <t>Genomics</t>
         </is>
       </c>
       <c r="J300" t="inlineStr">
@@ -33306,45 +33304,45 @@
       </c>
       <c r="M300" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N300" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.0992, 50.0307]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.5461, 49.947], [-124.6642, 49.947], [-124.6642, 50.457], [-125.5461, 50.457], [-125.5461, 49.947]]]}</t>
         </is>
       </c>
       <c r="P300" t="inlineStr">
         <is>
-          <t>[{'max': '260.0', 'min': '0.0'}]</t>
+          <t>[{'max': '200.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q300" t="inlineStr">
         <is>
-          <t>zooplanktonBiomassAndDiversity</t>
+          <t>invertebrateAbundanceAndDistribution, zooplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R300" t="inlineStr">
         <is>
-          <t>10.21966/6b20-7r76</t>
+          <t>10.21966/qrxk-vb32</t>
         </is>
       </c>
       <c r="S300" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OvzbmseH_syBXg1RXKd</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxClAtvMEmxKRtywIeT</t>
         </is>
       </c>
       <c r="T300" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="U300" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V300" t="n">
@@ -33363,12 +33361,12 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>b27bb6f9-49ae-4f3a-a02a-098d8edf23e2</t>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>ca-cioos_ac765dbb-8e47-415d-8685-d9090946b86b</t>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
@@ -33378,7 +33376,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Micro-invertebrate DNA Barcodes from Quadra Island, BC (Biomarathon)</t>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -33396,7 +33394,7 @@
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>Genomics</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J301" t="inlineStr">
@@ -33416,7 +33414,7 @@
       </c>
       <c r="M301" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>Tula Foundation</t>
         </is>
       </c>
       <c r="N301" t="n">
@@ -33424,37 +33422,33 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.5461, 49.947], [-124.6642, 49.947], [-124.6642, 50.457], [-125.5461, 50.457], [-125.5461, 49.947]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
       <c r="P301" t="inlineStr">
         <is>
-          <t>[{'max': '200.0', 'min': '0.0'}]</t>
+          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
       <c r="Q301" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, zooplanktonBiomassAndDiversity</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R301" t="inlineStr">
         <is>
-          <t>10.21966/qrxk-vb32</t>
+          <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
       <c r="S301" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxClAtvMEmxKRtywIeT</t>
-        </is>
-      </c>
-      <c r="T301" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
+        </is>
+      </c>
+      <c r="T301" t="inlineStr"/>
       <c r="U301" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2025-04-02</t>
         </is>
       </c>
       <c r="V301" t="n">
@@ -33466,112 +33460,6 @@
         </is>
       </c>
       <c r="X301" t="inlineStr"/>
-    </row>
-    <row r="302">
-      <c r="A302" t="n">
-        <v>300</v>
-      </c>
-      <c r="B302" t="inlineStr">
-        <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
-        </is>
-      </c>
-      <c r="C302" t="inlineStr">
-        <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
-        </is>
-      </c>
-      <c r="D302" t="inlineStr">
-        <is>
-          <t>Hakai Institute</t>
-        </is>
-      </c>
-      <c r="E302" t="inlineStr">
-        <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
-        </is>
-      </c>
-      <c r="F302" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="G302" t="inlineStr">
-        <is>
-          <t>CC-BY-4.0</t>
-        </is>
-      </c>
-      <c r="H302" t="b">
-        <v>0</v>
-      </c>
-      <c r="I302" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
-        </is>
-      </c>
-      <c r="J302" t="inlineStr">
-        <is>
-          <t>completed</t>
-        </is>
-      </c>
-      <c r="K302" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="L302" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="M302" t="inlineStr">
-        <is>
-          <t>Tula Foundation</t>
-        </is>
-      </c>
-      <c r="N302" t="n">
-        <v>1</v>
-      </c>
-      <c r="O302" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
-        </is>
-      </c>
-      <c r="P302" t="inlineStr">
-        <is>
-          <t>[{'max': '3954.0', 'min': '800.0'}]</t>
-        </is>
-      </c>
-      <c r="Q302" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R302" t="inlineStr">
-        <is>
-          <t>10.21966/w9n0-kn30</t>
-        </is>
-      </c>
-      <c r="S302" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
-        </is>
-      </c>
-      <c r="T302" t="inlineStr"/>
-      <c r="U302" t="inlineStr">
-        <is>
-          <t>2025-04-02</t>
-        </is>
-      </c>
-      <c r="V302" t="n">
-        <v>0</v>
-      </c>
-      <c r="W302" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X302" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deployed 4c71e665b to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X301"/>
+  <dimension ref="A1:X302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6105,12 +6105,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6176,17 +6176,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -6215,12 +6215,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6286,17 +6286,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -8405,12 +8405,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8420,7 +8420,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -8462,16 +8462,16 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -8481,12 +8481,12 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T74" t="inlineStr">
@@ -8496,7 +8496,7 @@
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V74" t="n">
@@ -8515,12 +8515,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8530,7 +8530,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8572,16 +8572,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8591,12 +8591,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -27429,12 +27429,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>49374495-400f-4acc-aac6-d7d0b7cae297</t>
+          <t>7b1120bc-4a2c-432c-9e54-879d66751a59</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>ca-cioos_bafcd0eb-8249-471b-b93b-0797cfeea287</t>
+          <t>ca-cioos_b2b18171-35b6-4345-b81b-497a90c2e7c5</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -27444,7 +27444,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Spatial extent of surface canopy kelp derived from fixed-wing surveys (2020), Central Coast, British Columbia, Canada</t>
+          <t>Seagrass fish and macroinvertebrate swaths BC Central Coast</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
@@ -27462,12 +27462,12 @@
       </c>
       <c r="I247" t="inlineStr">
         <is>
-          <t>Nearshore, Airborne Coastal Observatory, Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K247" t="inlineStr">
@@ -27490,37 +27490,37 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 51.64], [-128.1, 51.64], [-128.1, 52.01], [-128.5, 52.01], [-128.5, 51.64]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 52.09], [-128.5, 52.04], [-128.5, 51.97], [-128.5, 51.93], [-128.5, 51.9], [-128.4, 51.88], [-128.3, 51.86], [-128.3, 51.83], [-128.2, 51.63], [-127.9, 51.62], [-127.8, 51.77], [-127.8, 51.83], [-127.9, 51.99], [-128.4, 52.09]]]}</t>
         </is>
       </c>
       <c r="P247" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q247" t="inlineStr">
         <is>
-          <t>macroalgalCanopyCoverAndComposition, other</t>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R247" t="inlineStr">
         <is>
-          <t>10.21966/20ym-8826</t>
+          <t>10.21966/NMNG-SF35</t>
         </is>
       </c>
       <c r="S247" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Miha19AtLQ2u1uo0b_q</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/lJHlH9nm20QQOPuk217xLlxWbNv1/-NPt7327bul36pby-Odi</t>
         </is>
       </c>
       <c r="T247" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-27</t>
         </is>
       </c>
       <c r="U247" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="V247" t="n">
@@ -27539,12 +27539,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
+          <t>49374495-400f-4acc-aac6-d7d0b7cae297</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>ca-cioos_ba41d935-f293-447f-be3d-7098e569b431</t>
+          <t>ca-cioos_bafcd0eb-8249-471b-b93b-0797cfeea287</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -27554,7 +27554,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Water Property Measurements from Conductivity-Temperature-Depth Profilers, BC, Canada (Research)</t>
+          <t>Spatial extent of surface canopy kelp derived from fixed-wing surveys (2020), Central Coast, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -27572,12 +27572,12 @@
       </c>
       <c r="I248" t="inlineStr">
         <is>
-          <t>Oceanography, Nearshore, Watersheds, Juvenile Salmon Program</t>
+          <t>Nearshore, Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J248" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K248" t="inlineStr">
@@ -27596,41 +27596,41 @@
         </is>
       </c>
       <c r="N248" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 52.27], [-127.4, 52.21], [-127.2, 51.66], [-125.6, 51.13], [-124.8, 50.96], [-124.1, 50.43], [-124.7, 49.98], [-124.9, 49.8], [-126.7, 50.45], [-128.1, 51.37], [-128.4, 51.69], [-128.5, 52.27]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 51.64], [-128.1, 51.64], [-128.1, 52.01], [-128.5, 52.01], [-128.5, 51.64]]]}</t>
         </is>
       </c>
       <c r="P248" t="inlineStr">
         <is>
-          <t>[{'max': '700.0', 'min': '1.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q248" t="inlineStr">
         <is>
-          <t>oxygen, subSurfaceSalinity, subSurfaceTemperature</t>
+          <t>macroalgalCanopyCoverAndComposition, other</t>
         </is>
       </c>
       <c r="R248" t="inlineStr">
         <is>
-          <t>10.21966/kace-2d24</t>
+          <t>10.21966/20ym-8826</t>
         </is>
       </c>
       <c r="S248" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MX35qgX-BrwJDdeJKe1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Miha19AtLQ2u1uo0b_q</t>
         </is>
       </c>
       <c r="T248" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="U248" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="V248" t="n">
@@ -27649,12 +27649,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
+          <t>613ba2f9-b21d-445f-8eaa-f42950c9350b</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>ca-cioos_fb5c9e1e-a911-46b7-8c1d-e34215a105ed</t>
+          <t>ca-cioos_ba41d935-f293-447f-be3d-7098e569b431</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
@@ -27664,7 +27664,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 Analyzer located at Bamfield Marine Sciences Centre, Bamfield, BC, Canada (Provisional)</t>
+          <t>Water Property Measurements from Conductivity-Temperature-Depth Profilers, BC, Canada (Research)</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -27682,12 +27682,12 @@
       </c>
       <c r="I249" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Oceanography, Nearshore, Watersheds, Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J249" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K249" t="inlineStr">
@@ -27706,31 +27706,31 @@
         </is>
       </c>
       <c r="N249" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.13535, 48.83515]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.5, 52.27], [-127.4, 52.21], [-127.2, 51.66], [-125.6, 51.13], [-124.8, 50.96], [-124.1, 50.43], [-124.7, 49.98], [-124.9, 49.8], [-126.7, 50.45], [-128.1, 51.37], [-128.4, 51.69], [-128.5, 52.27]]]}</t>
         </is>
       </c>
       <c r="P249" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '20.0'}]</t>
+          <t>[{'max': '700.0', 'min': '1.0'}]</t>
         </is>
       </c>
       <c r="Q249" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
+          <t>oxygen, subSurfaceSalinity, subSurfaceTemperature</t>
         </is>
       </c>
       <c r="R249" t="inlineStr">
         <is>
-          <t>10.21966/65d8-k051</t>
+          <t>10.21966/kace-2d24</t>
         </is>
       </c>
       <c r="S249" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-NdH-jgHZQzKrYdb2nw_</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-MX35qgX-BrwJDdeJKe1</t>
         </is>
       </c>
       <c r="T249" t="inlineStr">
@@ -27740,7 +27740,7 @@
       </c>
       <c r="U249" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="V249" t="n">
@@ -27759,12 +27759,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
+          <t>c657dfa1-5970-4794-9c46-7c352df393d7</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>ca-cioos_91107fce-93a4-4bc9-bce4-e7d9e1cf02a0</t>
+          <t>ca-cioos_fb5c9e1e-a911-46b7-8c1d-e34215a105ed</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
@@ -27774,7 +27774,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Sentinel 3A and 3B Chlorophyll and Suspended Matter Concentrations for Coastal British Columbia and Southeast Alaska, 8-Day Average (Research)</t>
+          <t>Seawater Carbon Dioxide (CO2) Content from the Burke-o-Lator pCO2/TCO2 Analyzer located at Bamfield Marine Sciences Centre, Bamfield, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -27797,7 +27797,7 @@
       </c>
       <c r="J250" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K250" t="inlineStr">
@@ -27820,37 +27820,37 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.13535, 48.83515]}</t>
         </is>
       </c>
       <c r="P250" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '20.0', 'min': '20.0'}]</t>
         </is>
       </c>
       <c r="Q250" t="inlineStr">
         <is>
-          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
+          <t>seaSurfaceTemperature, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
         </is>
       </c>
       <c r="R250" t="inlineStr">
         <is>
-          <t>10.21966/175j-8k96</t>
+          <t>10.21966/65d8-k051</t>
         </is>
       </c>
       <c r="S250" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-Nueis-TZEnz_78f8PYf</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/tV5qE0aUgaOjSVmgPgiZ6MyHuSy1/-NdH-jgHZQzKrYdb2nw_</t>
         </is>
       </c>
       <c r="T250" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="U250" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V250" t="n">
@@ -27861,9 +27861,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X250" t="n">
-        <v>2</v>
-      </c>
+      <c r="X250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -27871,12 +27869,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
+          <t>185462b6-5d10-43d8-91b2-b92010e80ff4</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
+          <t>ca-cioos_91107fce-93a4-4bc9-bce4-e7d9e1cf02a0</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
@@ -27886,7 +27884,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
+          <t>Sentinel 3A and 3B Chlorophyll and Suspended Matter Concentrations for Coastal British Columbia and Southeast Alaska, 8-Day Average (Research)</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -27947,12 +27945,12 @@
       </c>
       <c r="R251" t="inlineStr">
         <is>
-          <t>10.21966/dveq-bt48</t>
+          <t>10.21966/175j-8k96</t>
         </is>
       </c>
       <c r="S251" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-Nueis-TZEnz_78f8PYf</t>
         </is>
       </c>
       <c r="T251" t="inlineStr">
@@ -27962,7 +27960,7 @@
       </c>
       <c r="U251" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="V251" t="n">
@@ -27983,12 +27981,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
+          <t>caf810f0-228a-4827-856c-f9b07a2377af</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
+          <t>ca-cioos_d1bef0b7-4d15-4bc1-bf34-faca6352891f</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
@@ -27998,7 +27996,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
+          <t>Daily satellite (Sentinel 3A and 3B) chlorophyll and suspended matter concentrations for coastal British Columbia and southeast Alaska</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -28016,12 +28014,12 @@
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
@@ -28040,52 +28038,54 @@
         </is>
       </c>
       <c r="N252" t="n">
+        <v>1</v>
+      </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-139.0, 47.0], [-121.5, 47.0], [-121.5, 59.5], [-139.0, 59.5], [-139.0, 47.0]]]}</t>
+        </is>
+      </c>
+      <c r="P252" t="inlineStr">
+        <is>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q252" t="inlineStr">
+        <is>
+          <t>phytoplanktonBiomassAndDiversity, particulateMatter, other</t>
+        </is>
+      </c>
+      <c r="R252" t="inlineStr">
+        <is>
+          <t>10.21966/dveq-bt48</t>
+        </is>
+      </c>
+      <c r="S252" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/7U7b8oPpeTN6gjvXlUCTGJr5pga2/-NTteirxDjvnABVz_7Dh</t>
+        </is>
+      </c>
+      <c r="T252" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="U252" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="V252" t="n">
+        <v>0</v>
+      </c>
+      <c r="W252" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X252" t="n">
         <v>2</v>
       </c>
-      <c r="O252" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
-        </is>
-      </c>
-      <c r="P252" t="inlineStr">
-        <is>
-          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q252" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R252" t="inlineStr">
-        <is>
-          <t>10.21966/RZVW-4A72</t>
-        </is>
-      </c>
-      <c r="S252" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
-        </is>
-      </c>
-      <c r="T252" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="U252" t="inlineStr">
-        <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="V252" t="n">
-        <v>1</v>
-      </c>
-      <c r="W252" t="inlineStr">
-        <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
-        </is>
-      </c>
-      <c r="X252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -28093,12 +28093,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
+          <t>b7b923ed-b3fa-48b3-878d-40a3797046bc</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
+          <t>ca-cioos_f7538807-4d49-4ed8-ad36-836c0e71428a</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
@@ -28108,7 +28108,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
+          <t>3m Digital Elevation Model - Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -28126,7 +28126,7 @@
       </c>
       <c r="I253" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J253" t="inlineStr">
@@ -28154,45 +28154,45 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16482, 51.408116], [-127.868831, 51.408116], [-127.868831, 51.734994], [-128.16482, 51.734994], [-128.16482, 51.408116]]]}</t>
         </is>
       </c>
       <c r="P253" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '1013.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q253" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R253" t="inlineStr">
         <is>
-          <t>10.21966/0xvh-1318</t>
+          <t>10.21966/RZVW-4A72</t>
         </is>
       </c>
       <c r="S253" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW13R3BBSGRER2ZkYnM</t>
         </is>
       </c>
       <c r="T253" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="U253" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V253" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W253" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X253" t="inlineStr"/>
@@ -28203,12 +28203,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
+          <t>e14d0456-297e-4636-8e7c-c615791b165e</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
+          <t>ca-cioos_33c8ce77-0674-4933-a305-01a25d253f70</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -28218,7 +28218,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
+          <t>Sea star microbiome data from 16S amplicon sequencing associated with rocky intertidal sites on Calvert and Quadra Islands</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
@@ -28236,12 +28236,12 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -28264,37 +28264,37 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.3, 49.87], [-124.8, 49.87], [-124.8, 51.75], [-128.3, 51.75], [-128.3, 49.87]]]}</t>
         </is>
       </c>
       <c r="P254" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q254" t="inlineStr">
         <is>
-          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
+          <t>invertebrateAbundanceAndDistribution, microbeBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R254" t="inlineStr">
         <is>
-          <t>10.21966/3q5j-n957</t>
+          <t>10.21966/0xvh-1318</t>
         </is>
       </c>
       <c r="S254" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/4TvAwNKXC7PkAi0TEZsZbbAzXfi1/-Oo1MBmr8fW1fputdBh6</t>
         </is>
       </c>
       <c r="T254" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-24</t>
         </is>
       </c>
       <c r="U254" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V254" t="n">
@@ -28313,12 +28313,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
+          <t>2510cc69-bd46-4534-a62f-dae1903b388d</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
+          <t>ca-cioos_a8671db6-81cc-4c92-b681-58595fe66182</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
@@ -28328,7 +28328,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
+          <t>Water Property Measurements from the Bute Inlet Ocean Observing Station (BIOOS) Wirewalker, Bute Inlet, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
@@ -28346,12 +28346,12 @@
       </c>
       <c r="I255" t="inlineStr">
         <is>
-          <t>Nearshore, Genomics</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J255" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K255" t="inlineStr">
@@ -28370,41 +28370,41 @@
         </is>
       </c>
       <c r="N255" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-124.9009, 50.5744]}</t>
         </is>
       </c>
       <c r="P255" t="inlineStr">
         <is>
-          <t>[{'max': '30.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q255" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution</t>
+          <t>subSurfaceTemperature, subSurfaceSalinity, oxygen, phytoplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R255" t="inlineStr">
         <is>
-          <t>10.21966/kmc2-5r12</t>
+          <t>10.21966/3q5j-n957</t>
         </is>
       </c>
       <c r="S255" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OqDQ7wqqJtwSgUoAN1g</t>
         </is>
       </c>
       <c r="T255" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="U255" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="V255" t="n">
@@ -28423,12 +28423,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
+          <t>227eb965-1892-4bad-8ded-dd2e1d68fdf6</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
+          <t>ca-cioos_08d3e779-2f44-4ce3-82cb-c7b763f72175</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
@@ -28438,7 +28438,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Horne Lake Bathymetry Mapping</t>
+          <t>DNA metabarcoding data from Autonomous Reef Monitoring Structures (ARMS) deployed around Calvert Island British Columbia</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
@@ -28456,7 +28456,7 @@
       </c>
       <c r="I256" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore, Genomics</t>
         </is>
       </c>
       <c r="J256" t="inlineStr">
@@ -28480,41 +28480,41 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.61], [-127.8, 51.61], [-127.8, 51.9], [-128.4, 51.9], [-128.4, 51.61]]]}</t>
         </is>
       </c>
       <c r="P256" t="inlineStr">
         <is>
-          <t>[{'max': '50.0', 'min': '0.0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q256" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R256" t="inlineStr">
         <is>
-          <t>10.21966/vwee-e004</t>
+          <t>10.21966/kmc2-5r12</t>
         </is>
       </c>
       <c r="S256" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/pX9Euv7m4yaHRKPuMtylMexACtt2/-ORSLLie2O-FFN8cPV1e</t>
         </is>
       </c>
       <c r="T256" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="U256" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="V256" t="n">
@@ -28533,12 +28533,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
+          <t>ed22dc0f-f2cc-41e5-ac1c-893e1b65c6d0</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
+          <t>ca-cioos_7e49967a-b5ab-443d-860b-e3c0eb0f709c</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
@@ -28548,7 +28548,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
+          <t>Horne Lake Bathymetry Mapping</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
@@ -28566,7 +28566,7 @@
       </c>
       <c r="I257" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J257" t="inlineStr">
@@ -28594,12 +28594,12 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.7872, 49.3105], [-124.6447, 49.3105], [-124.6447, 49.3644], [-124.7872, 49.3644], [-124.7872, 49.3105]]]}</t>
         </is>
       </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t>[{'max': '475.0', 'min': '0.0'}]</t>
+          <t>[{'max': '50.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q257" t="inlineStr">
@@ -28609,12 +28609,12 @@
       </c>
       <c r="R257" t="inlineStr">
         <is>
-          <t>10.21966/k0z0-3z50</t>
+          <t>10.21966/vwee-e004</t>
         </is>
       </c>
       <c r="S257" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/G8LjsjnnPxb5TxWL730BxDTQu532/-Njn-0LeJ-Uwj4L8EmOV</t>
         </is>
       </c>
       <c r="T257" t="inlineStr">
@@ -28624,7 +28624,7 @@
       </c>
       <c r="U257" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="V257" t="n">
@@ -28643,12 +28643,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
+          <t>18f56a52-11af-446a-aea9-07feca8d197e</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
+          <t>ca-cioos_e897c9d0-3fca-4c89-b37f-e571413ffd12</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
@@ -28658,7 +28658,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Knight Inlet Multibeam Bathymetry Survey</t>
+          <t>Joffre Provincial Park Aerial Surveys - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
@@ -28676,7 +28676,7 @@
       </c>
       <c r="I258" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J258" t="inlineStr">
@@ -28704,12 +28704,12 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.5281, 50.3147], [-122.4303, 50.3147], [-122.4303, 50.3796], [-122.5281, 50.3796], [-122.5281, 50.3147]]]}</t>
         </is>
       </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t>[{'max': '288.0', 'min': '0.0'}]</t>
+          <t>[{'max': '475.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q258" t="inlineStr">
@@ -28719,17 +28719,17 @@
       </c>
       <c r="R258" t="inlineStr">
         <is>
-          <t>10.21966/8dgz-1z27</t>
+          <t>10.21966/k0z0-3z50</t>
         </is>
       </c>
       <c r="S258" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ot_OaAHxjund0-w5rXq</t>
         </is>
       </c>
       <c r="T258" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-27</t>
         </is>
       </c>
       <c r="U258" t="inlineStr">
@@ -28753,12 +28753,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
+          <t>6c4803cc-d1c6-4327-806a-7f6796606175</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
+          <t>ca-cioos_6c34ed6e-5a17-41f2-b83a-cd59d1ce07bd</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
@@ -28768,7 +28768,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
+          <t>Knight Inlet Multibeam Bathymetry Survey</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
@@ -28786,7 +28786,7 @@
       </c>
       <c r="I259" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J259" t="inlineStr">
@@ -28814,12 +28814,12 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.0537, 50.6529], [-125.9229, 50.6529], [-125.9229, 50.7077], [-126.0537, 50.7077], [-126.0537, 50.6529]]]}</t>
         </is>
       </c>
       <c r="P259" t="inlineStr">
         <is>
-          <t>[{'max': '450.0', 'min': '200.0'}]</t>
+          <t>[{'max': '288.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q259" t="inlineStr">
@@ -28829,12 +28829,12 @@
       </c>
       <c r="R259" t="inlineStr">
         <is>
-          <t>10.21966/g8f2-jw82</t>
+          <t>10.21966/8dgz-1z27</t>
         </is>
       </c>
       <c r="S259" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OG7EOynnzSIOU7LPWgs</t>
         </is>
       </c>
       <c r="T259" t="inlineStr">
@@ -28863,12 +28863,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
+          <t>ce6f3f8c-6b57-4f18-be46-8c0b5a4baeb9</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
+          <t>ca-cioos_8755f475-2133-4205-baff-5e2937824f45</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
@@ -28878,7 +28878,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
+          <t>Poole Creek Aerial Surveys - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
@@ -28924,12 +28924,12 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.9075, 50.2436], [-122.8124, 50.2436], [-122.8124, 50.3016], [-122.9075, 50.3016], [-122.9075, 50.2436]]]}</t>
         </is>
       </c>
       <c r="P260" t="inlineStr">
         <is>
-          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
+          <t>[{'max': '450.0', 'min': '200.0'}]</t>
         </is>
       </c>
       <c r="Q260" t="inlineStr">
@@ -28939,22 +28939,22 @@
       </c>
       <c r="R260" t="inlineStr">
         <is>
-          <t>10.21966/n6ga-nc24</t>
+          <t>10.21966/g8f2-jw82</t>
         </is>
       </c>
       <c r="S260" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OtfdtO43um_1J_LdCpn</t>
         </is>
       </c>
       <c r="T260" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="U260" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="V260" t="n">
@@ -28973,12 +28973,12 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
+          <t>e1247209-cc26-4788-82a2-dd8a5c971e22</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
+          <t>ca-cioos_2e5ddbaa-4f0c-4339-8595-1ddbd35c3df4</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
@@ -28988,7 +28988,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
+          <t>Glacier and Icefield Aerial Surveys in British Columbia, Washington, and Alberta - 2025 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
@@ -29006,7 +29006,7 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
@@ -29034,12 +29034,12 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.9263, 48.0077], [-112.7224, 48.0077], [-112.7224, 54.6673], [-127.9263, 54.6673], [-127.9263, 48.0077]]]}</t>
         </is>
       </c>
       <c r="P261" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '4019.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q261" t="inlineStr">
@@ -29049,12 +29049,12 @@
       </c>
       <c r="R261" t="inlineStr">
         <is>
-          <t>10.21966/kn3e-fn08</t>
+          <t>10.21966/n6ga-nc24</t>
         </is>
       </c>
       <c r="S261" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Ou3t_K6rGOHTMO67Xbq</t>
         </is>
       </c>
       <c r="T261" t="inlineStr">
@@ -29083,12 +29083,12 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
+          <t>5ac3ac5f-702e-43d8-bcb7-79f30c4d9e08</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
+          <t>ca-cioos_656ea307-fed0-48ca-b5d8-1bc017dc52d2</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
@@ -29098,7 +29098,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Sea surface temperature data in False Creek, British Columbia</t>
+          <t>Botanical Beach - Juan de Fuca Provincial Park - Drone Mapping</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -29116,7 +29116,7 @@
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
@@ -29144,37 +29144,37 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.45265489, 48.52152402], [-124.43377214, 48.52152402], [-124.43377214, 48.53061904], [-124.45265489, 48.53061904], [-124.45265489, 48.52152402]]]}</t>
         </is>
       </c>
       <c r="P262" t="inlineStr">
         <is>
-          <t>[{'max': '0.5', 'min': '0.5'}]</t>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q262" t="inlineStr">
         <is>
-          <t>seaSurfaceTemperature</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R262" t="inlineStr">
         <is>
-          <t>10.21966/0g6d-pk30</t>
+          <t>10.21966/kn3e-fn08</t>
         </is>
       </c>
       <c r="S262" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUdvcmtQME1NZmdWcDY</t>
         </is>
       </c>
       <c r="T262" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="U262" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="V262" t="n">
@@ -29193,12 +29193,12 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
+          <t>05dac0a6-a26c-4cb5-895d-132b5e2134cd</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
+          <t>ca-cioos_b45dbc9d-bf7a-4734-86cd-3397e7c9ac62</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
@@ -29208,7 +29208,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
+          <t>Sea surface temperature data in False Creek, British Columbia</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
@@ -29226,12 +29226,12 @@
       </c>
       <c r="I263" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J263" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K263" t="inlineStr">
@@ -29254,37 +29254,37 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.27], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28], [-123.1, 49.28]]]}</t>
         </is>
       </c>
       <c r="P263" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.5', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q263" t="inlineStr">
         <is>
-          <t>other, seagrassCoverAndComposition</t>
+          <t>seaSurfaceTemperature</t>
         </is>
       </c>
       <c r="R263" t="inlineStr">
         <is>
-          <t>10.21966/03pw-2190</t>
+          <t>10.21966/0g6d-pk30</t>
         </is>
       </c>
       <c r="S263" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/57FPdLIBPcb9BOLfIOW44RJVywN2/-NHaXDtgFZr0-Oul6FZG</t>
         </is>
       </c>
       <c r="T263" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="U263" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="V263" t="n">
@@ -29303,12 +29303,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
+          <t>6eb46e26-dac5-4964-8b29-8e8541381aac</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>ca-cioos_79368bf3-8f02-4355-837e-3a6cef0d2886</t>
+          <t>ca-cioos_5e4f925a-9cf2-4e33-ae22-75c5b326ce6c</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
@@ -29318,7 +29318,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Provisional)</t>
+          <t>Time series of eelgrass (Zostera marina) meadow extent derived from drone surveys, Central Coast, British Columbia</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -29336,12 +29336,12 @@
       </c>
       <c r="I264" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J264" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K264" t="inlineStr">
@@ -29360,11 +29360,11 @@
         </is>
       </c>
       <c r="N264" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.65354407, 51.37817421], [-127.69773286, 51.37817421], [-127.69773286, 52.1127963], [-128.65354407, 52.1127963], [-128.65354407, 51.37817421]]]}</t>
         </is>
       </c>
       <c r="P264" t="inlineStr">
@@ -29374,27 +29374,27 @@
       </c>
       <c r="Q264" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R264" t="inlineStr">
         <is>
-          <t>10.21966/c6xs-y324</t>
+          <t>10.21966/03pw-2190</t>
         </is>
       </c>
       <c r="S264" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OtAIe6lv3elLZd4c-V1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTA3NnQ0NnRiemVLSFU</t>
         </is>
       </c>
       <c r="T264" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="U264" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V264" t="n">
@@ -29413,12 +29413,12 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
+          <t>67b81524-e385-439e-9bc1-03bd4652eba6</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>ca-cioos_d986aade-6bf1-4dfa-97c2-686975f944d5</t>
+          <t>ca-cioos_79368bf3-8f02-4355-837e-3a6cef0d2886</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
@@ -29428,7 +29428,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Research)</t>
+          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
@@ -29451,7 +29451,7 @@
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -29474,12 +29474,12 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.1, 51.64], [-128.0, 51.64], [-128.0, 51.67], [-128.1, 51.67], [-128.1, 51.64]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P265" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q265" t="inlineStr">
@@ -29489,17 +29489,17 @@
       </c>
       <c r="R265" t="inlineStr">
         <is>
-          <t>10.21966/47m7-ev69</t>
+          <t>10.21966/c6xs-y324</t>
         </is>
       </c>
       <c r="S265" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OHj73dBYs1okPPjDXKY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OtAIe6lv3elLZd4c-V1</t>
         </is>
       </c>
       <c r="T265" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="U265" t="inlineStr">
@@ -29523,12 +29523,12 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>71c6db20-a521-451b-b371-a2560f6af25e</t>
+          <t>ff456916-01f7-4eb0-961f-3658f0b4f39b</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>ca-cioos_999da1dd-efde-4a55-868b-ce2d6ca3b983</t>
+          <t>ca-cioos_d986aade-6bf1-4dfa-97c2-686975f944d5</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
@@ -29538,7 +29538,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Observations from the 2017 Hakai MarineGEO Bioblitz</t>
+          <t>Watersheds Stream Stations Timeseries, Calvert and Hecate Islands, BC, Canada (Research)</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -29556,12 +29556,12 @@
       </c>
       <c r="I266" t="inlineStr">
         <is>
-          <t>Genomics</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J266" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K266" t="inlineStr">
@@ -29580,41 +29580,41 @@
         </is>
       </c>
       <c r="N266" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.951, 51.48631], [-127.76165, 51.48631], [-127.76165, 52.05347], [-128.951, 52.05347], [-128.951, 51.48631]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.1, 51.64], [-128.0, 51.64], [-128.0, 51.67], [-128.1, 51.67], [-128.1, 51.64]]]}</t>
         </is>
       </c>
       <c r="P266" t="inlineStr">
         <is>
-          <t>[{'max': '40.0', 'min': '0.5'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q266" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R266" t="inlineStr">
         <is>
-          <t>10.21966/0jfr-7b65</t>
+          <t>10.21966/47m7-ev69</t>
         </is>
       </c>
       <c r="S266" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCmJU0B97JSOfOpj6J</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/zBOULF9sDAgC4rkoZUFQq7sBGCf2/-OHj73dBYs1okPPjDXKY</t>
         </is>
       </c>
       <c r="T266" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="U266" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="V266" t="n">
@@ -29633,12 +29633,12 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>f0ae5f04-2c3a-4b67-8fbf-c6dc3771257d</t>
+          <t>71c6db20-a521-451b-b371-a2560f6af25e</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>ca-cioos_482d2463-0c81-4d62-a22a-1c0942b3c1fa</t>
+          <t>ca-cioos_999da1dd-efde-4a55-868b-ce2d6ca3b983</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
@@ -29648,7 +29648,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Observations from the 2019 Hakai Deep Water Bioblitz</t>
+          <t>Observations from the 2017 Hakai MarineGEO Bioblitz</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
@@ -29694,12 +29694,12 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.14433, 51.615734], [-127.76327, 51.615734], [-127.76327, 51.787], [-128.14433, 51.787], [-128.14433, 51.615734]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.951, 51.48631], [-127.76165, 51.48631], [-127.76165, 52.05347], [-128.951, 52.05347], [-128.951, 51.48631]]]}</t>
         </is>
       </c>
       <c r="P267" t="inlineStr">
         <is>
-          <t>[{'max': '255.0', 'min': '5.0'}]</t>
+          <t>[{'max': '40.0', 'min': '0.5'}]</t>
         </is>
       </c>
       <c r="Q267" t="inlineStr">
@@ -29709,22 +29709,22 @@
       </c>
       <c r="R267" t="inlineStr">
         <is>
-          <t>10.21966/3p06-vt55</t>
+          <t>10.21966/0jfr-7b65</t>
         </is>
       </c>
       <c r="S267" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCoStSubGWAdV78XNC</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCmJU0B97JSOfOpj6J</t>
         </is>
       </c>
       <c r="T267" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="U267" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="V267" t="n">
@@ -29743,12 +29743,12 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>91d2ddf0-ea25-4ef9-b990-26d2957cb3bd</t>
+          <t>f0ae5f04-2c3a-4b67-8fbf-c6dc3771257d</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>ca-cioos_542a20b8-242e-4199-a062-5b76ea9cbf2d</t>
+          <t>ca-cioos_482d2463-0c81-4d62-a22a-1c0942b3c1fa</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
@@ -29758,7 +29758,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Observations from the 2018 Hakai Terrestrial Bioblitz</t>
+          <t>Observations from the 2019 Hakai Deep Water Bioblitz</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
@@ -29804,27 +29804,27 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.98366, 51.5919], [-125.0032, 51.5919], [-125.0032, 53.9998], [-128.98366, 53.9998], [-128.98366, 51.5919]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.14433, 51.615734], [-127.76327, 51.615734], [-127.76327, 51.787], [-128.14433, 51.787], [-128.14433, 51.615734]]]}</t>
         </is>
       </c>
       <c r="P268" t="inlineStr">
         <is>
-          <t>[{'max': '1012.0', 'min': '50.0'}]</t>
+          <t>[{'max': '255.0', 'min': '5.0'}]</t>
         </is>
       </c>
       <c r="Q268" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R268" t="inlineStr">
         <is>
-          <t>10.21966/t0h7-8g95</t>
+          <t>10.21966/3p06-vt55</t>
         </is>
       </c>
       <c r="S268" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCpwd5hTju8QOKVY-E</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCoStSubGWAdV78XNC</t>
         </is>
       </c>
       <c r="T268" t="inlineStr">
@@ -29834,7 +29834,7 @@
       </c>
       <c r="U268" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="V268" t="n">
@@ -29853,12 +29853,12 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>fa42f16a-3693-4c51-b45c-a36e709fdac3</t>
+          <t>91d2ddf0-ea25-4ef9-b990-26d2957cb3bd</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>ca-cioos_d69bf79e-b616-404e-bbfc-92932ca74087</t>
+          <t>ca-cioos_542a20b8-242e-4199-a062-5b76ea9cbf2d</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
@@ -29868,7 +29868,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Observations from the 2018 Hakai Seagrass Bioblitz</t>
+          <t>Observations from the 2018 Hakai Terrestrial Bioblitz</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -29886,7 +29886,7 @@
       </c>
       <c r="I269" t="inlineStr">
         <is>
-          <t>Genomics, Nearshore</t>
+          <t>Genomics</t>
         </is>
       </c>
       <c r="J269" t="inlineStr">
@@ -29914,27 +29914,27 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.8123, 51.8438], [-128.2105, 51.684], [-128.1968, 51.6158], [-127.8837, 51.6192], [-127.8123, 51.8438]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.98366, 51.5919], [-125.0032, 51.5919], [-125.0032, 53.9998], [-128.98366, 53.9998], [-128.98366, 51.5919]]]}</t>
         </is>
       </c>
       <c r="P269" t="inlineStr">
         <is>
-          <t>[{'max': '300.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1012.0', 'min': '50.0'}]</t>
         </is>
       </c>
       <c r="Q269" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution, seagrassCoverAndComposition</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R269" t="inlineStr">
         <is>
-          <t>10.21966/yf1f-jx85</t>
+          <t>10.21966/t0h7-8g95</t>
         </is>
       </c>
       <c r="S269" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCnP9OAghmAmYObj0D</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCpwd5hTju8QOKVY-E</t>
         </is>
       </c>
       <c r="T269" t="inlineStr">
@@ -29944,7 +29944,7 @@
       </c>
       <c r="U269" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="V269" t="n">
@@ -29963,12 +29963,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>fc3d2ea5-b60c-42c9-97e9-542024bec9fa</t>
+          <t>fa42f16a-3693-4c51-b45c-a36e709fdac3</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>ca-cioos_4add33cd-b182-4825-900a-5695f333125a</t>
+          <t>ca-cioos_d69bf79e-b616-404e-bbfc-92932ca74087</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
@@ -29978,7 +29978,7 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Weather Station Time Series, Hyacinthe Bay, BC, Canada (Provisional)</t>
+          <t>Observations from the 2018 Hakai Seagrass Bioblitz</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
@@ -29996,12 +29996,12 @@
       </c>
       <c r="I270" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Genomics, Nearshore</t>
         </is>
       </c>
       <c r="J270" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K270" t="inlineStr">
@@ -30024,37 +30024,47 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.2221111, 50.1162556]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.8123, 51.8438], [-128.2105, 51.684], [-128.1968, 51.6158], [-127.8837, 51.6192], [-127.8123, 51.8438]]]}</t>
         </is>
       </c>
       <c r="P270" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '300.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q270" t="inlineStr">
         <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="R270" t="inlineStr"/>
+          <t>fishAbundanceAndDistribution, invertebrateAbundanceAndDistribution, seagrassCoverAndComposition</t>
+        </is>
+      </c>
+      <c r="R270" t="inlineStr">
+        <is>
+          <t>10.21966/yf1f-jx85</t>
+        </is>
+      </c>
       <c r="S270" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OyesAm4pxUK1wqBMn7x</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxCnP9OAghmAmYObj0D</t>
         </is>
       </c>
       <c r="T270" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="U270" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
-        </is>
-      </c>
-      <c r="V270" t="inlineStr"/>
-      <c r="W270" t="inlineStr"/>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="V270" t="n">
+        <v>0</v>
+      </c>
+      <c r="W270" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="X270" t="inlineStr"/>
     </row>
     <row r="271">
@@ -30063,12 +30073,12 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
+          <t>fc3d2ea5-b60c-42c9-97e9-542024bec9fa</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>ca-cioos_3f40326a-23f9-4e30-a16a-f332ace14e2f</t>
+          <t>ca-cioos_4add33cd-b182-4825-900a-5695f333125a</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
@@ -30078,7 +30088,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>Nereocystis kelp canopy productivity data from BC Central Coast</t>
+          <t>Weather Station Time Series, Hyacinthe Bay, BC, Canada (Provisional)</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
@@ -30096,12 +30106,12 @@
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -30124,47 +30134,37 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.6, 51.19], [-127.1, 51.19], [-127.1, 52.28], [-128.6, 52.28], [-128.6, 51.19]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.2221111, 50.1162556]}</t>
         </is>
       </c>
       <c r="P271" t="inlineStr">
         <is>
-          <t>[{'max': '30.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q271" t="inlineStr">
         <is>
-          <t>macroalgalCanopyCoverAndComposition</t>
-        </is>
-      </c>
-      <c r="R271" t="inlineStr">
-        <is>
-          <t>10.21966/d1s2-s530</t>
-        </is>
-      </c>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="R271" t="inlineStr"/>
       <c r="S271" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/df5J7W5Hk4e0p4yvlOAI0qcU9Gs2/-MtG8b48aDAEdJoqNT6N</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-OyesAm4pxUK1wqBMn7x</t>
         </is>
       </c>
       <c r="T271" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="U271" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="V271" t="n">
-        <v>1</v>
-      </c>
-      <c r="W271" t="inlineStr">
-        <is>
-          <t>[{'year': '2024', 'total': 1}]</t>
-        </is>
-      </c>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="V271" t="inlineStr"/>
+      <c r="W271" t="inlineStr"/>
       <c r="X271" t="inlineStr"/>
     </row>
     <row r="272">
@@ -30173,12 +30173,12 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>aab940b9-bb7f-49c0-ae62-4f78d26897b3</t>
+          <t>4b04cbfe-71f4-47b4-b028-3fcd24e7cff2</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>ca-cioos_0219e1d6-8dfc-4718-b89b-ea3dff06a70d</t>
+          <t>ca-cioos_3f40326a-23f9-4e30-a16a-f332ace14e2f</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
@@ -30188,7 +30188,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Modeled Eelgrass Extent, British Columbia, Canada</t>
+          <t>Nereocystis kelp canopy productivity data from BC Central Coast</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
@@ -30206,12 +30206,12 @@
       </c>
       <c r="I272" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J272" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K272" t="inlineStr">
@@ -30230,49 +30230,49 @@
         </is>
       </c>
       <c r="N272" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-133.7841801345348, 48.23443097294032], [-122.49023482203482, 48.23443097294032], [-122.49023482203482, 54.52958287232971], [-133.7841801345348, 54.52958287232971], [-133.7841801345348, 48.23443097294032]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.6, 51.19], [-127.1, 51.19], [-127.1, 52.28], [-128.6, 52.28], [-128.6, 51.19]]]}</t>
         </is>
       </c>
       <c r="P272" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '30.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q272" t="inlineStr">
         <is>
-          <t>other, seagrassCoverAndComposition</t>
+          <t>macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R272" t="inlineStr">
         <is>
-          <t>10.21966/1ty5-e654</t>
+          <t>10.21966/d1s2-s530</t>
         </is>
       </c>
       <c r="S272" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWtuNVpwdEdLRXZTODc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/df5J7W5Hk4e0p4yvlOAI0qcU9Gs2/-MtG8b48aDAEdJoqNT6N</t>
         </is>
       </c>
       <c r="T272" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="U272" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="V272" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W272" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2024', 'total': 1}]</t>
         </is>
       </c>
       <c r="X272" t="inlineStr"/>
@@ -30283,12 +30283,12 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>3988f8e8-36ea-4cda-9bd9-a03157116ef5</t>
+          <t>aab940b9-bb7f-49c0-ae62-4f78d26897b3</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>ca-cioos_d43a79c1-a6ba-4e37-8dc2-6ced6312828e</t>
+          <t>ca-cioos_0219e1d6-8dfc-4718-b89b-ea3dff06a70d</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
@@ -30298,7 +30298,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>Data from Manuscript: Parasites of the hermit crab Pagurus hirsutiusculus; distribution, prevalence, and thermal ecology</t>
+          <t>Modeled Eelgrass Extent, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
@@ -30316,7 +30316,7 @@
       </c>
       <c r="I273" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J273" t="inlineStr">
@@ -30340,11 +30340,11 @@
         </is>
       </c>
       <c r="N273" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.66], [-127.9, 51.81], [-122.2, 49.03], [-123.3, 49.01], [-123.0, 48.83], [-123.0, 48.78], [-123.3, 48.7], [-123.3, 48.53], [-123.6, 48.59], [-125.2, 48.73], [-125.6, 48.95], [-125.6, 50.11], [-128.4, 51.66]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-133.7841801345348, 48.23443097294032], [-122.49023482203482, 48.23443097294032], [-122.49023482203482, 54.52958287232971], [-133.7841801345348, 54.52958287232971], [-133.7841801345348, 48.23443097294032]]]}</t>
         </is>
       </c>
       <c r="P273" t="inlineStr">
@@ -30354,17 +30354,17 @@
       </c>
       <c r="Q273" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, seaSurfaceSalinity</t>
+          <t>other, seagrassCoverAndComposition</t>
         </is>
       </c>
       <c r="R273" t="inlineStr">
         <is>
-          <t>10.21966/xb3t-qb88</t>
+          <t>10.21966/1ty5-e654</t>
         </is>
       </c>
       <c r="S273" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3eh7IMAvm8ZUtcMBeifFL0eJCIA3/-O5Kei32z9cfatfgKj5y</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWtuNVpwdEdLRXZTODc</t>
         </is>
       </c>
       <c r="T273" t="inlineStr">
@@ -30374,7 +30374,7 @@
       </c>
       <c r="U273" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="V273" t="n">
@@ -30393,12 +30393,12 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>3988f8e8-36ea-4cda-9bd9-a03157116ef5</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>ca-cioos_53189107-9df5-426b-acb4-f903468554fe</t>
+          <t>ca-cioos_d43a79c1-a6ba-4e37-8dc2-6ced6312828e</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -30408,7 +30408,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Comparing invertebrate and seaweed diversity in kelp forests and urchin barrens in Owen Bay, British Columbia, using Autonomous Reef Monitoring Structures (ARMS)</t>
+          <t>Data from Manuscript: Parasites of the hermit crab Pagurus hirsutiusculus; distribution, prevalence, and thermal ecology</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -30426,7 +30426,7 @@
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>Sentinels of Change, Genomics</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
@@ -30450,41 +30450,41 @@
         </is>
       </c>
       <c r="N274" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.2335, 50.2999], [-125.2163, 50.2999], [-125.2163, 50.313], [-125.2335, 50.313], [-125.2335, 50.2999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.66], [-127.9, 51.81], [-122.2, 49.03], [-123.3, 49.01], [-123.0, 48.83], [-123.0, 48.78], [-123.3, 48.7], [-123.3, 48.53], [-123.6, 48.59], [-125.2, 48.73], [-125.6, 48.95], [-125.6, 50.11], [-128.4, 51.66]]]}</t>
         </is>
       </c>
       <c r="P274" t="inlineStr">
         <is>
-          <t>[{'max': '6.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q274" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
+          <t>invertebrateAbundanceAndDistribution, seaSurfaceSalinity</t>
         </is>
       </c>
       <c r="R274" t="inlineStr">
         <is>
-          <t>10.21966/e5mw-tr82</t>
+          <t>10.21966/xb3t-qb88</t>
         </is>
       </c>
       <c r="S274" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/5Jh4rsxoBsRd4mVFqZ0XJoMtMHI2/-P-tq8uNjGhWtk4rBny0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3eh7IMAvm8ZUtcMBeifFL0eJCIA3/-O5Kei32z9cfatfgKj5y</t>
         </is>
       </c>
       <c r="T274" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="U274" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="V274" t="n">
@@ -30495,9 +30495,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X274" t="n">
-        <v>1</v>
-      </c>
+      <c r="X274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -30505,12 +30503,12 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>ca-cioos_73abfecf-d35c-4f9c-a991-eee5cece08ea</t>
+          <t>ca-cioos_53189107-9df5-426b-acb4-f903468554fe</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -30520,7 +30518,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>Kelp Canopy Extent 2012 - NW Calvert Island</t>
+          <t>Comparing invertebrate and seaweed diversity in kelp forests and urchin barrens in Owen Bay, British Columbia, using Autonomous Reef Monitoring Structures (ARMS)</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -30538,7 +30536,7 @@
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Sentinels of Change, Genomics</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
@@ -30562,41 +30560,41 @@
         </is>
       </c>
       <c r="N275" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16959381103513, 51.63613234359897], [-128.11191558837888, 51.63613234359897], [-128.11191558837888, 51.681709494104325], [-128.16959381103513, 51.681709494104325], [-128.16959381103513, 51.63613234359897]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.2335, 50.2999], [-125.2163, 50.2999], [-125.2163, 50.313], [-125.2335, 50.313], [-125.2335, 50.2999]]]}</t>
         </is>
       </c>
       <c r="P275" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '6.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q275" t="inlineStr">
         <is>
-          <t>other, macroalgalCanopyCoverAndComposition</t>
+          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R275" t="inlineStr">
         <is>
-          <t>10.21966/63rs-yt91</t>
+          <t>10.21966/e5mw-tr82</t>
         </is>
       </c>
       <c r="S275" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxUM01laTFaREhKbWE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/5Jh4rsxoBsRd4mVFqZ0XJoMtMHI2/-P-tq8uNjGhWtk4rBny0</t>
         </is>
       </c>
       <c r="T275" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="U275" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="V275" t="n">
@@ -30617,12 +30615,12 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
+          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>ca-cioos_940218ef-d7f8-4f3f-9e69-52150ecdbec5</t>
+          <t>ca-cioos_73abfecf-d35c-4f9c-a991-eee5cece08ea</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -30632,7 +30630,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>North Vancouver Island Aerial Survey - 2024 - Airborne Coastal Observatory</t>
+          <t>Kelp Canopy Extent 2012 - NW Calvert Island</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -30650,7 +30648,7 @@
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
@@ -30674,31 +30672,31 @@
         </is>
       </c>
       <c r="N276" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.7, 50.35], [-125.4, 50.35], [-125.4, 50.63], [-126.7, 50.63], [-126.7, 50.35]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16959381103513, 51.63613234359897], [-128.11191558837888, 51.63613234359897], [-128.11191558837888, 51.681709494104325], [-128.16959381103513, 51.681709494104325], [-128.16959381103513, 51.63613234359897]]]}</t>
         </is>
       </c>
       <c r="P276" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q276" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R276" t="inlineStr">
         <is>
-          <t>10.21966/kdhe-hz07</t>
+          <t>10.21966/63rs-yt91</t>
         </is>
       </c>
       <c r="S276" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OCoHpqOwDbp834fqRY3</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxUM01laTFaREhKbWE</t>
         </is>
       </c>
       <c r="T276" t="inlineStr">
@@ -30708,7 +30706,7 @@
       </c>
       <c r="U276" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="V276" t="n">
@@ -30729,12 +30727,12 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
+          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>ca-cioos_c7466354-bacc-4781-acdc-543dd03d1eab</t>
+          <t>ca-cioos_940218ef-d7f8-4f3f-9e69-52150ecdbec5</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -30744,7 +30742,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Nanwakolas LiDAR Surveys - Airborne Coastal Observatory</t>
+          <t>North Vancouver Island Aerial Survey - 2024 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -30790,12 +30788,12 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.8, 49.26], [-124.5, 49.26], [-124.5, 50.83], [-126.8, 50.83], [-126.8, 49.26]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.7, 50.35], [-125.4, 50.35], [-125.4, 50.63], [-126.7, 50.63], [-126.7, 50.35]]]}</t>
         </is>
       </c>
       <c r="P277" t="inlineStr">
         <is>
-          <t>[{'max': '1700.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q277" t="inlineStr">
@@ -30805,12 +30803,12 @@
       </c>
       <c r="R277" t="inlineStr">
         <is>
-          <t>10.21966/e0r7-ge27</t>
+          <t>10.21966/kdhe-hz07</t>
         </is>
       </c>
       <c r="S277" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OjbuSE_uZcCs3Fit_mg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OCoHpqOwDbp834fqRY3</t>
         </is>
       </c>
       <c r="T277" t="inlineStr">
@@ -30820,7 +30818,7 @@
       </c>
       <c r="U277" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="V277" t="n">
@@ -30839,12 +30837,12 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>f7433c1a-3aad-4761-81c4-c191a5e6ac92</t>
+          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>ca-cioos_52e97374-bee5-4b1a-9b85-7170a5df8d6b</t>
+          <t>ca-cioos_c7466354-bacc-4781-acdc-543dd03d1eab</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -30854,7 +30852,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Biomass and density of Pycnopodia helianthoides from the central coast of BC</t>
+          <t>Nanwakolas LiDAR Surveys - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -30872,7 +30870,7 @@
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>Oceanography, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
@@ -30900,37 +30898,37 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.617, 51.3321], [-127.3509, 51.3321], [-127.3509, 52.3317], [-128.617, 52.3317], [-128.617, 51.3321]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.8, 49.26], [-124.5, 49.26], [-124.5, 50.83], [-126.8, 50.83], [-126.8, 49.26]]]}</t>
         </is>
       </c>
       <c r="P278" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1700.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q278" t="inlineStr">
         <is>
-          <t>seaSurfaceSalinity, subSurfaceSalinity, seaSurfaceTemperature, subSurfaceTemperature, invertebrateAbundanceAndDistribution</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R278" t="inlineStr">
         <is>
-          <t>10.21966/xy6n-qz76</t>
+          <t>10.21966/e0r7-ge27</t>
         </is>
       </c>
       <c r="S278" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-OteEfuBSvhg-2RySC4a</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OjbuSE_uZcCs3Fit_mg</t>
         </is>
       </c>
       <c r="T278" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="U278" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="V278" t="n">
@@ -30949,12 +30947,12 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>f7433c1a-3aad-4761-81c4-c191a5e6ac92</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>ca-cioos_b4844ae2-d9c1-42f2-ae4d-a8f994c395a0</t>
+          <t>ca-cioos_52e97374-bee5-4b1a-9b85-7170a5df8d6b</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -30964,7 +30962,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Putting fjord biodiversity on the map for British Columbia conservation planning</t>
+          <t>Biomass and density of Pycnopodia helianthoides from the central coast of BC</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -30982,7 +30980,7 @@
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>Genomics, Oceanography</t>
+          <t>Oceanography, Nearshore</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
@@ -31002,45 +31000,45 @@
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N279" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.0471, 52.2577], [-128.9141, 51.7033], [-127.6841, 50.7687], [-123.7744, 48.9864], [-122.764, 49.331], [-122.8299, 49.9706], [-127.0471, 52.2577]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.617, 51.3321], [-127.3509, 51.3321], [-127.3509, 52.3317], [-128.617, 52.3317], [-128.617, 51.3321]]]}</t>
         </is>
       </c>
       <c r="P279" t="inlineStr">
         <is>
-          <t>[{'max': '595.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q279" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, subSurfaceTemperature, subSurfaceSalinity</t>
+          <t>seaSurfaceSalinity, subSurfaceSalinity, seaSurfaceTemperature, subSurfaceTemperature, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R279" t="inlineStr">
         <is>
-          <t>10.21966/n141-m959</t>
+          <t>10.21966/xy6n-qz76</t>
         </is>
       </c>
       <c r="S279" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-Ow-ZgW1jkC5-WyrtlLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-OteEfuBSvhg-2RySC4a</t>
         </is>
       </c>
       <c r="T279" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="U279" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="V279" t="n">
@@ -31051,9 +31049,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X279" t="n">
-        <v>1</v>
-      </c>
+      <c r="X279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -31061,12 +31057,12 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
+          <t>ca-cioos_b4844ae2-d9c1-42f2-ae4d-a8f994c395a0</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -31076,7 +31072,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
+          <t>Putting fjord biodiversity on the map for British Columbia conservation planning</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -31094,7 +31090,7 @@
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Genomics, Oceanography</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
@@ -31114,56 +31110,58 @@
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N280" t="n">
+        <v>2</v>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.0471, 52.2577], [-128.9141, 51.7033], [-127.6841, 50.7687], [-123.7744, 48.9864], [-122.764, 49.331], [-122.8299, 49.9706], [-127.0471, 52.2577]]]}</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>[{'max': '595.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>fishAbundanceAndDistribution, subSurfaceTemperature, subSurfaceSalinity</t>
+        </is>
+      </c>
+      <c r="R280" t="inlineStr">
+        <is>
+          <t>10.21966/n141-m959</t>
+        </is>
+      </c>
+      <c r="S280" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-Ow-ZgW1jkC5-WyrtlLV</t>
+        </is>
+      </c>
+      <c r="T280" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="U280" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="V280" t="n">
+        <v>0</v>
+      </c>
+      <c r="W280" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X280" t="n">
         <v>1</v>
       </c>
-      <c r="O280" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
-        </is>
-      </c>
-      <c r="P280" t="inlineStr">
-        <is>
-          <t>[{'max': '2.5', 'min': '2.5'}]</t>
-        </is>
-      </c>
-      <c r="Q280" t="inlineStr">
-        <is>
-          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R280" t="inlineStr">
-        <is>
-          <t>10.21966/rrzq-yw32</t>
-        </is>
-      </c>
-      <c r="S280" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
-        </is>
-      </c>
-      <c r="T280" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="U280" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="V280" t="n">
-        <v>0</v>
-      </c>
-      <c r="W280" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -31171,12 +31169,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
+          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -31186,17 +31184,17 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
+          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>collection</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H281" t="b">
@@ -31209,7 +31207,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -31232,23 +31230,27 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
         </is>
       </c>
       <c r="P281" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '600.0'}]</t>
+          <t>[{'max': '2.5', 'min': '2.5'}]</t>
         </is>
       </c>
       <c r="Q281" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R281" t="inlineStr"/>
+          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr">
+        <is>
+          <t>10.21966/rrzq-yw32</t>
+        </is>
+      </c>
       <c r="S281" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
         </is>
       </c>
       <c r="T281" t="inlineStr">
@@ -31258,11 +31260,17 @@
       </c>
       <c r="U281" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="V281" t="inlineStr"/>
-      <c r="W281" t="inlineStr"/>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="V281" t="n">
+        <v>0</v>
+      </c>
+      <c r="W281" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="X281" t="inlineStr"/>
     </row>
     <row r="282">
@@ -31271,12 +31279,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
+          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -31286,17 +31294,17 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
+          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>collection</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H282" t="b">
@@ -31304,12 +31312,12 @@
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>Estuary Resilience</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -31332,47 +31340,37 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
         </is>
       </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+          <t>[{'max': '0.0', 'min': '600.0'}]</t>
         </is>
       </c>
       <c r="Q282" t="inlineStr">
         <is>
-          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
-        </is>
-      </c>
-      <c r="R282" t="inlineStr">
-        <is>
-          <t>10.21966/r9zr-xz33</t>
-        </is>
-      </c>
+          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr"/>
       <c r="S282" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
         </is>
       </c>
       <c r="T282" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="U282" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="V282" t="n">
-        <v>0</v>
-      </c>
-      <c r="W282" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="V282" t="inlineStr"/>
+      <c r="W282" t="inlineStr"/>
       <c r="X282" t="inlineStr"/>
     </row>
     <row r="283">
@@ -31381,12 +31379,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
+          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
+          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -31396,7 +31394,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -31442,7 +31440,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
         </is>
       </c>
       <c r="P283" t="inlineStr">
@@ -31457,12 +31455,12 @@
       </c>
       <c r="R283" t="inlineStr">
         <is>
-          <t>10.21966/9dbb-5d54</t>
+          <t>10.21966/r9zr-xz33</t>
         </is>
       </c>
       <c r="S283" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
         </is>
       </c>
       <c r="T283" t="inlineStr">
@@ -31491,12 +31489,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
+          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
+          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -31506,7 +31504,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -31552,7 +31550,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
         </is>
       </c>
       <c r="P284" t="inlineStr">
@@ -31567,12 +31565,12 @@
       </c>
       <c r="R284" t="inlineStr">
         <is>
-          <t>10.21966/vpz7-mm73</t>
+          <t>10.21966/9dbb-5d54</t>
         </is>
       </c>
       <c r="S284" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
         </is>
       </c>
       <c r="T284" t="inlineStr">
@@ -31601,12 +31599,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>0ce3ee5b-425b-4eb0-a201-96bdfb795a3f</t>
+          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>ca-cioos_354b5b83-e752-4ffb-a740-d1cdc02ac8c6</t>
+          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -31616,7 +31614,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Dtlaxsiwè River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -31662,7 +31660,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.1721, 50.61011], [-127.17933, 50.612], [-127.1873, 50.6098], [-127.19703, 50.61072], [-127.20524, 50.61585], [-127.19007, 50.61844], [-127.18675, 50.61393], [-127.17744, 50.61359], [-127.17161, 50.61118], [-127.17203, 50.61011], [-127.1721, 50.61011]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
         </is>
       </c>
       <c r="P285" t="inlineStr">
@@ -31677,12 +31675,12 @@
       </c>
       <c r="R285" t="inlineStr">
         <is>
-          <t>10.21966/ydm2-m238</t>
+          <t>10.21966/vpz7-mm73</t>
         </is>
       </c>
       <c r="S285" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7Dng-ZtRd05hnZCq1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
         </is>
       </c>
       <c r="T285" t="inlineStr">
@@ -31711,12 +31709,12 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>1a2aa5c8-9a83-46f7-967d-1127436c2084</t>
+          <t>0ce3ee5b-425b-4eb0-a201-96bdfb795a3f</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>ca-cioos_58a5140a-0b2c-4186-a648-53d9f58e5226</t>
+          <t>ca-cioos_354b5b83-e752-4ffb-a740-d1cdc02ac8c6</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -31726,7 +31724,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kvai River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Dtlaxsiwè River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -31772,7 +31770,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.81882, 51.77547], [-127.83122, 51.77986], [-127.85192, 51.781], [-127.86785, 51.78358], [-127.8958, 51.77366], [-127.89418, 51.77118], [-127.87834, 51.77309], [-127.86508, 51.77748], [-127.84009, 51.77519], [-127.82731, 51.77452], [-127.82025, 51.77309], [-127.81853, 51.77566], [-127.81882, 51.77547]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.1721, 50.61011], [-127.17933, 50.612], [-127.1873, 50.6098], [-127.19703, 50.61072], [-127.20524, 50.61585], [-127.19007, 50.61844], [-127.18675, 50.61393], [-127.17744, 50.61359], [-127.17161, 50.61118], [-127.17203, 50.61011], [-127.1721, 50.61011]]]}</t>
         </is>
       </c>
       <c r="P286" t="inlineStr">
@@ -31787,12 +31785,12 @@
       </c>
       <c r="R286" t="inlineStr">
         <is>
-          <t>10.21966/pm9m-h431</t>
+          <t>10.21966/ydm2-m238</t>
         </is>
       </c>
       <c r="S286" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7QQE3ifLCAPcu3Jih</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7Dng-ZtRd05hnZCq1</t>
         </is>
       </c>
       <c r="T286" t="inlineStr">
@@ -31821,12 +31819,12 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>c035b81c-0fc3-446e-bec5-8b8933ae874b</t>
+          <t>1a2aa5c8-9a83-46f7-967d-1127436c2084</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>ca-cioos_7fbc28f7-ee87-4361-bbee-0ed8ce24522d</t>
+          <t>ca-cioos_58a5140a-0b2c-4186-a648-53d9f58e5226</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -31836,7 +31834,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Gwa'dzi River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kvai River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -31882,7 +31880,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.46176, 50.74217], [-127.49022, 50.72165], [-127.49167, 50.71188], [-127.4832, 50.70356], [-127.4874, 50.69181], [-127.46443, 50.6928], [-127.47282, 50.70776], [-127.47992, 50.71424], [-127.48305, 50.72058], [-127.45901, 50.74011], [-127.46153, 50.74217], [-127.46176, 50.74217]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.81882, 51.77547], [-127.83122, 51.77986], [-127.85192, 51.781], [-127.86785, 51.78358], [-127.8958, 51.77366], [-127.89418, 51.77118], [-127.87834, 51.77309], [-127.86508, 51.77748], [-127.84009, 51.77519], [-127.82731, 51.77452], [-127.82025, 51.77309], [-127.81853, 51.77566], [-127.81882, 51.77547]]]}</t>
         </is>
       </c>
       <c r="P287" t="inlineStr">
@@ -31897,12 +31895,12 @@
       </c>
       <c r="R287" t="inlineStr">
         <is>
-          <t>10.21966/xq99-x273</t>
+          <t>10.21966/pm9m-h431</t>
         </is>
       </c>
       <c r="S287" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7BCRnF2C30YPkxIyd</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7QQE3ifLCAPcu3Jih</t>
         </is>
       </c>
       <c r="T287" t="inlineStr">
@@ -31931,12 +31929,12 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
+          <t>c035b81c-0fc3-446e-bec5-8b8933ae874b</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
+          <t>ca-cioos_7fbc28f7-ee87-4361-bbee-0ed8ce24522d</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -31946,7 +31944,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Gwa'dzi River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -31992,7 +31990,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.46176, 50.74217], [-127.49022, 50.72165], [-127.49167, 50.71188], [-127.4832, 50.70356], [-127.4874, 50.69181], [-127.46443, 50.6928], [-127.47282, 50.70776], [-127.47992, 50.71424], [-127.48305, 50.72058], [-127.45901, 50.74011], [-127.46153, 50.74217], [-127.46176, 50.74217]]]}</t>
         </is>
       </c>
       <c r="P288" t="inlineStr">
@@ -32007,12 +32005,12 @@
       </c>
       <c r="R288" t="inlineStr">
         <is>
-          <t>10.21966/kde9-8g12</t>
+          <t>10.21966/xq99-x273</t>
         </is>
       </c>
       <c r="S288" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7BCRnF2C30YPkxIyd</t>
         </is>
       </c>
       <c r="T288" t="inlineStr">
@@ -32041,12 +32039,12 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
+          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
+          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -32056,7 +32054,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -32102,7 +32100,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
         </is>
       </c>
       <c r="P289" t="inlineStr">
@@ -32117,12 +32115,12 @@
       </c>
       <c r="R289" t="inlineStr">
         <is>
-          <t>10.21966/9a97-2j48</t>
+          <t>10.21966/kde9-8g12</t>
         </is>
       </c>
       <c r="S289" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
         </is>
       </c>
       <c r="T289" t="inlineStr">
@@ -32151,12 +32149,12 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
+          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
+          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -32166,7 +32164,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -32212,7 +32210,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
         </is>
       </c>
       <c r="P290" t="inlineStr">
@@ -32227,12 +32225,12 @@
       </c>
       <c r="R290" t="inlineStr">
         <is>
-          <t>10.21966/ed9w-2653</t>
+          <t>10.21966/9a97-2j48</t>
         </is>
       </c>
       <c r="S290" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
         </is>
       </c>
       <c r="T290" t="inlineStr">
@@ -32261,12 +32259,12 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>1af6a43a-e73b-4774-8e10-b9f2928ab133</t>
+          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>ca-cioos_ae7e017c-9211-4f98-b56e-90a4bbac161c</t>
+          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -32276,7 +32274,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Snuneymuxw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -32322,7 +32320,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.88685, 49.19332], [-123.92494, 49.1612], [-123.92581, 49.13841], [-123.91159, 49.123], [-123.88023, 49.11117], [-123.85971, 49.12766], [-123.89792, 49.16196], [-123.88099, 49.18866], [-123.88685, 49.19332]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
         </is>
       </c>
       <c r="P291" t="inlineStr">
@@ -32337,12 +32335,12 @@
       </c>
       <c r="R291" t="inlineStr">
         <is>
-          <t>10.21966/k01q-wb27</t>
+          <t>10.21966/ed9w-2653</t>
         </is>
       </c>
       <c r="S291" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt459vxCIH7YPRN9fp</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
         </is>
       </c>
       <c r="T291" t="inlineStr">
@@ -32371,12 +32369,12 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
+          <t>1af6a43a-e73b-4774-8e10-b9f2928ab133</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
+          <t>ca-cioos_ae7e017c-9211-4f98-b56e-90a4bbac161c</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -32386,7 +32384,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Snuneymuxw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
@@ -32432,7 +32430,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635], [-123.66843, 48.91641]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.88685, 49.19332], [-123.92494, 49.1612], [-123.92581, 49.13841], [-123.91159, 49.123], [-123.88023, 49.11117], [-123.85971, 49.12766], [-123.89792, 49.16196], [-123.88099, 49.18866], [-123.88685, 49.19332]]]}</t>
         </is>
       </c>
       <c r="P292" t="inlineStr">
@@ -32447,12 +32445,12 @@
       </c>
       <c r="R292" t="inlineStr">
         <is>
-          <t>10.21966/q2e0-j004</t>
+          <t>10.21966/k01q-wb27</t>
         </is>
       </c>
       <c r="S292" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt459vxCIH7YPRN9fp</t>
         </is>
       </c>
       <c r="T292" t="inlineStr">
@@ -32481,12 +32479,12 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
+          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
+          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -32496,7 +32494,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
@@ -32542,7 +32540,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635], [-123.66843, 48.91641]]]}</t>
         </is>
       </c>
       <c r="P293" t="inlineStr">
@@ -32557,12 +32555,12 @@
       </c>
       <c r="R293" t="inlineStr">
         <is>
-          <t>10.21966/hjkj-6611</t>
+          <t>10.21966/q2e0-j004</t>
         </is>
       </c>
       <c r="S293" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
         </is>
       </c>
       <c r="T293" t="inlineStr">
@@ -32591,12 +32589,12 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
+          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>ca-cioos_dce15b7b-3772-4106-ab20-c3979c4c3f57</t>
+          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -32606,7 +32604,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Fulmore River - Shoal Creek Estuary Complex (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -32652,7 +32650,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.08798, 50.4777], [-126.09599, 50.48418], [-126.09046, 50.50918], [-126.0647, 50.52425], [-125.99698, 50.53569], [-125.93459, 50.56717], [-125.93173, 50.56202], [-125.93764, 50.55458], [-125.91055, 50.55134], [-125.89853, 50.54943], [-125.90063, 50.54466], [-125.96416, 50.53989], [-125.98973, 50.52043], [-126.06566, 50.5067], [-126.08779, 50.47789], [-126.08798, 50.4777]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
         </is>
       </c>
       <c r="P294" t="inlineStr">
@@ -32667,12 +32665,12 @@
       </c>
       <c r="R294" t="inlineStr">
         <is>
-          <t>10.21966/g1cn-xs92</t>
+          <t>10.21966/hjkj-6611</t>
         </is>
       </c>
       <c r="S294" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptdJ8iUmLeOrdmqzrQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
         </is>
       </c>
       <c r="T294" t="inlineStr">
@@ -32701,12 +32699,12 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
+          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
+          <t>ca-cioos_dce15b7b-3772-4106-ab20-c3979c4c3f57</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
@@ -32716,7 +32714,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Fulmore River - Shoal Creek Estuary Complex (Provisional)</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -32762,7 +32760,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.08798, 50.4777], [-126.09599, 50.48418], [-126.09046, 50.50918], [-126.0647, 50.52425], [-125.99698, 50.53569], [-125.93459, 50.56717], [-125.93173, 50.56202], [-125.93764, 50.55458], [-125.91055, 50.55134], [-125.89853, 50.54943], [-125.90063, 50.54466], [-125.96416, 50.53989], [-125.98973, 50.52043], [-126.06566, 50.5067], [-126.08779, 50.47789], [-126.08798, 50.4777]]]}</t>
         </is>
       </c>
       <c r="P295" t="inlineStr">
@@ -32777,12 +32775,12 @@
       </c>
       <c r="R295" t="inlineStr">
         <is>
-          <t>10.21966/npe4-3036</t>
+          <t>10.21966/g1cn-xs92</t>
         </is>
       </c>
       <c r="S295" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptdJ8iUmLeOrdmqzrQ</t>
         </is>
       </c>
       <c r="T295" t="inlineStr">
@@ -32811,12 +32809,12 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
+          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>ca-cioos_e9b72149-8cf1-4000-ae3e-6b29ad60b078</t>
+          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -32826,7 +32824,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Malksope River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -32872,7 +32870,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.46569, 50.12556], [-127.45723, 50.13142], [-127.43281, 50.13338], [-127.42845, 50.13765], [-127.41181, 50.14408], [-127.40973, 50.14233], [-127.41999, 50.13627], [-127.41803, 50.13195], [-127.43106, 50.12796], [-127.46545, 50.12446], [-127.46569, 50.12548], [-127.46569, 50.12556]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
         </is>
       </c>
       <c r="P296" t="inlineStr">
@@ -32887,12 +32885,12 @@
       </c>
       <c r="R296" t="inlineStr">
         <is>
-          <t>10.21966/21sf-ey03</t>
+          <t>10.21966/npe4-3036</t>
         </is>
       </c>
       <c r="S296" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq77iyWJfPg4z-FvOSb</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
         </is>
       </c>
       <c r="T296" t="inlineStr">
@@ -32921,12 +32919,12 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>5177d019-598e-4415-b778-9688403652c8</t>
+          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>ca-cioos_ed84df74-5a2d-4a7d-87c8-a7b93f11088e</t>
+          <t>ca-cioos_e9b72149-8cf1-4000-ae3e-6b29ad60b078</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
@@ -32936,7 +32934,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Nalaxdlala River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Malksope River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -32982,7 +32980,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.9489, 50.70902], [-125.9696, 50.70291], [-126.00938, 50.69118], [-126.00108, 50.66848], [-125.98257, 50.68374], [-125.98152, 50.69271], [-125.95462, 50.70263], [-125.94785, 50.70768], [-125.9489, 50.70911], [-125.9489, 50.70902]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.46569, 50.12556], [-127.45723, 50.13142], [-127.43281, 50.13338], [-127.42845, 50.13765], [-127.41181, 50.14408], [-127.40973, 50.14233], [-127.41999, 50.13627], [-127.41803, 50.13195], [-127.43106, 50.12796], [-127.46545, 50.12446], [-127.46569, 50.12548], [-127.46569, 50.12556]]]}</t>
         </is>
       </c>
       <c r="P297" t="inlineStr">
@@ -32997,12 +32995,12 @@
       </c>
       <c r="R297" t="inlineStr">
         <is>
-          <t>10.21966/4krv-aw23</t>
+          <t>10.21966/21sf-ey03</t>
         </is>
       </c>
       <c r="S297" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptbxmpkBsfyWWfSxOJ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq77iyWJfPg4z-FvOSb</t>
         </is>
       </c>
       <c r="T297" t="inlineStr">
@@ -33031,12 +33029,12 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
+          <t>5177d019-598e-4415-b778-9688403652c8</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>ca-cioos_b922699f-69b6-4d63-b538-7c290086a408</t>
+          <t>ca-cioos_ed84df74-5a2d-4a7d-87c8-a7b93f11088e</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
@@ -33046,7 +33044,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Quw'utsun/Xwulqw'selu River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Nalaxdlala River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
@@ -33092,7 +33090,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.56201, 48.73508], [-123.59772, 48.75559], [-123.62127, 48.76514], [-123.63885, 48.77426], [-123.66935, 48.78033], [-123.67901, 48.75472], [-123.65155, 48.74322], [-123.63017, 48.7405], [-123.60792, 48.74289], [-123.56494, 48.72987], [-123.56179, 48.73529], [-123.56201, 48.73508]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.9489, 50.70902], [-125.9696, 50.70291], [-126.00938, 50.69118], [-126.00108, 50.66848], [-125.98257, 50.68374], [-125.98152, 50.69271], [-125.95462, 50.70263], [-125.94785, 50.70768], [-125.9489, 50.70911], [-125.9489, 50.70902]]]}</t>
         </is>
       </c>
       <c r="P298" t="inlineStr">
@@ -33107,17 +33105,17 @@
       </c>
       <c r="R298" t="inlineStr">
         <is>
-          <t>10.21966/2ha7-9p26</t>
+          <t>10.21966/4krv-aw23</t>
         </is>
       </c>
       <c r="S298" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpsCA3ycwZ7bFTDIQxh</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptbxmpkBsfyWWfSxOJ</t>
         </is>
       </c>
       <c r="T298" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="U298" t="inlineStr">
@@ -33141,12 +33139,12 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>dd471e82-a6b8-4f32-891c-bbea26e9998e</t>
+          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>ca-cioos_aeb30028-a7eb-462e-ac0f-6c5fe101d4a2</t>
+          <t>ca-cioos_b922699f-69b6-4d63-b538-7c290086a408</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
@@ -33156,7 +33154,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>DNA Metabarcoding Captures Temporal and Vertical Dynamics of Mesozooplankton Communities</t>
+          <t>BC Estuary Water Quality Monitoring Data - Quw'utsun/Xwulqw'selu River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -33174,12 +33172,12 @@
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>Genomics, Oceanography</t>
+          <t>Estuary Resilience</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -33194,45 +33192,45 @@
       </c>
       <c r="M299" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N299" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.0992, 50.0307]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.56201, 48.73508], [-123.59772, 48.75559], [-123.62127, 48.76514], [-123.63885, 48.77426], [-123.66935, 48.78033], [-123.67901, 48.75472], [-123.65155, 48.74322], [-123.63017, 48.7405], [-123.60792, 48.74289], [-123.56494, 48.72987], [-123.56179, 48.73529], [-123.56201, 48.73508]]]}</t>
         </is>
       </c>
       <c r="P299" t="inlineStr">
         <is>
-          <t>[{'max': '260.0', 'min': '0.0'}]</t>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
         </is>
       </c>
       <c r="Q299" t="inlineStr">
         <is>
-          <t>zooplanktonBiomassAndDiversity</t>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
         </is>
       </c>
       <c r="R299" t="inlineStr">
         <is>
-          <t>10.21966/6b20-7r76</t>
+          <t>10.21966/2ha7-9p26</t>
         </is>
       </c>
       <c r="S299" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OvzbmseH_syBXg1RXKd</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpsCA3ycwZ7bFTDIQxh</t>
         </is>
       </c>
       <c r="T299" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="U299" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V299" t="n">
@@ -33251,12 +33249,12 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>b27bb6f9-49ae-4f3a-a02a-098d8edf23e2</t>
+          <t>dd471e82-a6b8-4f32-891c-bbea26e9998e</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>ca-cioos_ac765dbb-8e47-415d-8685-d9090946b86b</t>
+          <t>ca-cioos_aeb30028-a7eb-462e-ac0f-6c5fe101d4a2</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
@@ -33266,7 +33264,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Micro-invertebrate DNA Barcodes from Quadra Island, BC (Biomarathon)</t>
+          <t>DNA Metabarcoding Captures Temporal and Vertical Dynamics of Mesozooplankton Communities</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
@@ -33284,7 +33282,7 @@
       </c>
       <c r="I300" t="inlineStr">
         <is>
-          <t>Genomics</t>
+          <t>Genomics, Oceanography</t>
         </is>
       </c>
       <c r="J300" t="inlineStr">
@@ -33304,45 +33302,45 @@
       </c>
       <c r="M300" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N300" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.5461, 49.947], [-124.6642, 49.947], [-124.6642, 50.457], [-125.5461, 50.457], [-125.5461, 49.947]]]}</t>
+          <t>{'type': 'Point', 'coordinates': [-125.0992, 50.0307]}</t>
         </is>
       </c>
       <c r="P300" t="inlineStr">
         <is>
-          <t>[{'max': '200.0', 'min': '0.0'}]</t>
+          <t>[{'max': '260.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q300" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, zooplanktonBiomassAndDiversity</t>
+          <t>zooplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R300" t="inlineStr">
         <is>
-          <t>10.21966/qrxk-vb32</t>
+          <t>10.21966/6b20-7r76</t>
         </is>
       </c>
       <c r="S300" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxClAtvMEmxKRtywIeT</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OvzbmseH_syBXg1RXKd</t>
         </is>
       </c>
       <c r="T300" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="U300" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="V300" t="n">
@@ -33361,12 +33359,12 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+          <t>b27bb6f9-49ae-4f3a-a02a-098d8edf23e2</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+          <t>ca-cioos_ac765dbb-8e47-415d-8685-d9090946b86b</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
@@ -33376,7 +33374,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+          <t>Micro-invertebrate DNA Barcodes from Quadra Island, BC (Biomarathon)</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -33394,7 +33392,7 @@
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Genomics</t>
         </is>
       </c>
       <c r="J301" t="inlineStr">
@@ -33414,7 +33412,7 @@
       </c>
       <c r="M301" t="inlineStr">
         <is>
-          <t>Tula Foundation</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N301" t="n">
@@ -33422,44 +33420,154 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.5461, 49.947], [-124.6642, 49.947], [-124.6642, 50.457], [-125.5461, 50.457], [-125.5461, 49.947]]]}</t>
+        </is>
+      </c>
+      <c r="P301" t="inlineStr">
+        <is>
+          <t>[{'max': '200.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q301" t="inlineStr">
+        <is>
+          <t>invertebrateAbundanceAndDistribution, zooplanktonBiomassAndDiversity</t>
+        </is>
+      </c>
+      <c r="R301" t="inlineStr">
+        <is>
+          <t>10.21966/qrxk-vb32</t>
+        </is>
+      </c>
+      <c r="S301" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OxClAtvMEmxKRtywIeT</t>
+        </is>
+      </c>
+      <c r="T301" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="U301" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="V301" t="n">
+        <v>0</v>
+      </c>
+      <c r="W301" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X301" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>300</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H302" t="b">
+        <v>0</v>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory, Geospatial</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>Tula Foundation</t>
+        </is>
+      </c>
+      <c r="N302" t="n">
+        <v>1</v>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
           <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
-      <c r="P301" t="inlineStr">
+      <c r="P302" t="inlineStr">
         <is>
           <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
-      <c r="Q301" t="inlineStr">
+      <c r="Q302" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="R301" t="inlineStr">
+      <c r="R302" t="inlineStr">
         <is>
           <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
-      <c r="S301" t="inlineStr">
+      <c r="S302" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
         </is>
       </c>
-      <c r="T301" t="inlineStr"/>
-      <c r="U301" t="inlineStr">
+      <c r="T302" t="inlineStr"/>
+      <c r="U302" t="inlineStr">
         <is>
           <t>2025-04-02</t>
         </is>
       </c>
-      <c r="V301" t="n">
-        <v>0</v>
-      </c>
-      <c r="W301" t="inlineStr">
+      <c r="V302" t="n">
+        <v>0</v>
+      </c>
+      <c r="W302" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="X301" t="inlineStr"/>
+      <c r="X302" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deployed ff40f103a to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -8075,12 +8075,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>6338c2fa-3d4d-42dc-9c91-31761365e11e</t>
+          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ca-cioos_77a256cd-baf7-434e-9f62-53ba809e48cb</t>
+          <t>ca-cioos_804b5b42-5550-4620-b789-7c2fe9572c03</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>High-resolution record of 8-m seawater CO2 content entering Fanny Bay Oysters in Baynes Sound, British Columbia, Canada from March 2017 to November 2017</t>
+          <t>Zooplankton - Taxonomy – Northern Strait of Georgia, Discovery Islands, Johnstone Strait, and Queen Charlotte Strait – April to July 2015 and 2016</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -8113,7 +8113,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -8132,11 +8132,11 @@
         </is>
       </c>
       <c r="N71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.88983154296876, 49.44759314103575], [-124.70993041992188, 49.44759314103575], [-124.70993041992188, 49.56975910961884], [-124.88983154296876, 49.56975910961884], [-124.88983154296876, 49.44759314103575]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.93452704, 49.56730131], [-124.18481219, 49.56730131], [-124.18481219, 50.90762515], [-126.93452704, 50.90762515], [-126.93452704, 49.56730131]]]}</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -8146,17 +8146,17 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, zooplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>10.21966/1.622315</t>
+          <t>10.21966/bhqd-9361</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTV4aEZoVWsyRXpHWno</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZhamNPb0U3cThnR0o</t>
         </is>
       </c>
       <c r="T71" t="inlineStr">
@@ -8166,15 +8166,15 @@
       </c>
       <c r="U71" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="V71" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W71" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>[{'year': '2026', 'total': 1}]</t>
         </is>
       </c>
       <c r="X71" t="inlineStr"/>
@@ -8185,12 +8185,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
+          <t>6338c2fa-3d4d-42dc-9c91-31761365e11e</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ca-cioos_804b5b42-5550-4620-b789-7c2fe9572c03</t>
+          <t>ca-cioos_77a256cd-baf7-434e-9f62-53ba809e48cb</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Zooplankton - Taxonomy – Northern Strait of Georgia, Discovery Islands, Johnstone Strait, and Queen Charlotte Strait – April to July 2015 and 2016</t>
+          <t>High-resolution record of 8-m seawater CO2 content entering Fanny Bay Oysters in Baynes Sound, British Columbia, Canada from March 2017 to November 2017</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -8242,52 +8242,54 @@
         </is>
       </c>
       <c r="N72" t="n">
+        <v>2</v>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.88983154296876, 49.44759314103575], [-124.70993041992188, 49.44759314103575], [-124.70993041992188, 49.56975910961884], [-124.88983154296876, 49.56975910961884], [-124.88983154296876, 49.44759314103575]]]}</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr">
+        <is>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>other, inorganicCarbon</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>10.21966/1.622315</t>
+        </is>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTV4aEZoVWsyRXpHWno</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>2022-02-04</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="V72" t="n">
+        <v>0</v>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X72" t="n">
         <v>1</v>
       </c>
-      <c r="O72" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.93452704, 49.56730131], [-124.18481219, 49.56730131], [-124.18481219, 50.90762515], [-126.93452704, 50.90762515], [-126.93452704, 49.56730131]]]}</t>
-        </is>
-      </c>
-      <c r="P72" t="inlineStr">
-        <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
-        </is>
-      </c>
-      <c r="Q72" t="inlineStr">
-        <is>
-          <t>other, zooplanktonBiomassAndDiversity</t>
-        </is>
-      </c>
-      <c r="R72" t="inlineStr">
-        <is>
-          <t>10.21966/bhqd-9361</t>
-        </is>
-      </c>
-      <c r="S72" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZhamNPb0U3cThnR0o</t>
-        </is>
-      </c>
-      <c r="T72" t="inlineStr">
-        <is>
-          <t>2022-02-04</t>
-        </is>
-      </c>
-      <c r="U72" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="V72" t="n">
-        <v>1</v>
-      </c>
-      <c r="W72" t="inlineStr">
-        <is>
-          <t>[{'year': '2026', 'total': 1}]</t>
-        </is>
-      </c>
-      <c r="X72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -9175,12 +9177,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>8d3f619f-e3e5-44a7-8b35-7e4ed1e6af31</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_d2e83e40-9e95-4a47-a899-b37c744be3ab</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9190,7 +9192,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Fin Island &amp; K'yel - 2020 - Airborne Coastal Observatory Data</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9208,7 +9210,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -9236,7 +9238,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.4, 53.03], [-129.1, 53.03], [-129.1, 53.29], [-129.4, 53.29], [-129.4, 53.03]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
@@ -9251,12 +9253,12 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/q4c4-wx08</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNm5cwomXVNI6vWU-R</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -9266,7 +9268,7 @@
       </c>
       <c r="U81" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V81" t="n">
@@ -9285,12 +9287,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>8d3f619f-e3e5-44a7-8b35-7e4ed1e6af31</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ca-cioos_d2e83e40-9e95-4a47-a899-b37c744be3ab</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9300,7 +9302,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Fin Island &amp; K'yel - 2020 - Airborne Coastal Observatory Data</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -9318,7 +9320,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -9346,7 +9348,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.4, 53.03], [-129.1, 53.03], [-129.1, 53.29], [-129.4, 53.29], [-129.4, 53.03]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
@@ -9361,12 +9363,12 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>10.21966/q4c4-wx08</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNm5cwomXVNI6vWU-R</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -9376,7 +9378,7 @@
       </c>
       <c r="U82" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="V82" t="n">
@@ -9387,7 +9389,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X82" t="inlineStr"/>
+      <c r="X82" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -13025,12 +13029,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -13040,7 +13044,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -13063,7 +13067,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -13082,11 +13086,11 @@
         </is>
       </c>
       <c r="N116" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -13101,12 +13105,12 @@
       </c>
       <c r="R116" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T116" t="inlineStr">
@@ -13116,7 +13120,7 @@
       </c>
       <c r="U116" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V116" t="n">
@@ -13124,7 +13128,7 @@
       </c>
       <c r="W116" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X116" t="inlineStr"/>
@@ -13135,12 +13139,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13150,7 +13154,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13173,7 +13177,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13192,11 +13196,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13211,12 +13215,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13226,7 +13230,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13234,7 +13238,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -15005,12 +15009,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -15020,7 +15024,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -15038,7 +15042,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -15058,20 +15062,20 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N134" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -15081,12 +15085,12 @@
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -15096,7 +15100,7 @@
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V134" t="n">
@@ -15115,12 +15119,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15130,7 +15134,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15148,7 +15152,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15168,20 +15172,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15191,12 +15195,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15206,7 +15210,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -31371,7 +31375,9 @@
       </c>
       <c r="V282" t="inlineStr"/>
       <c r="W282" t="inlineStr"/>
-      <c r="X282" t="inlineStr"/>
+      <c r="X282" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="n">

</xml_diff>

<commit_message>
Deployed 41448842f to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -8075,12 +8075,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
+          <t>6338c2fa-3d4d-42dc-9c91-31761365e11e</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>ca-cioos_804b5b42-5550-4620-b789-7c2fe9572c03</t>
+          <t>ca-cioos_77a256cd-baf7-434e-9f62-53ba809e48cb</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -8090,7 +8090,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Zooplankton - Taxonomy – Northern Strait of Georgia, Discovery Islands, Johnstone Strait, and Queen Charlotte Strait – April to July 2015 and 2016</t>
+          <t>High-resolution record of 8-m seawater CO2 content entering Fanny Bay Oysters in Baynes Sound, British Columbia, Canada from March 2017 to November 2017</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -8113,7 +8113,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>underDevelopment</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -8132,11 +8132,11 @@
         </is>
       </c>
       <c r="N71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.93452704, 49.56730131], [-124.18481219, 49.56730131], [-124.18481219, 50.90762515], [-126.93452704, 50.90762515], [-126.93452704, 49.56730131]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.88983154296876, 49.44759314103575], [-124.70993041992188, 49.44759314103575], [-124.70993041992188, 49.56975910961884], [-124.88983154296876, 49.56975910961884], [-124.88983154296876, 49.44759314103575]]]}</t>
         </is>
       </c>
       <c r="P71" t="inlineStr">
@@ -8146,17 +8146,17 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>other, zooplanktonBiomassAndDiversity</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>10.21966/bhqd-9361</t>
+          <t>10.21966/1.622315</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZhamNPb0U3cThnR0o</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTV4aEZoVWsyRXpHWno</t>
         </is>
       </c>
       <c r="T71" t="inlineStr">
@@ -8166,15 +8166,15 @@
       </c>
       <c r="U71" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W71" t="inlineStr">
         <is>
-          <t>[{'year': '2026', 'total': 1}]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="X71" t="inlineStr"/>
@@ -8185,12 +8185,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>6338c2fa-3d4d-42dc-9c91-31761365e11e</t>
+          <t>d3ed88cb-4f38-4c2e-a966-3dd49c9cafec</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ca-cioos_77a256cd-baf7-434e-9f62-53ba809e48cb</t>
+          <t>ca-cioos_804b5b42-5550-4620-b789-7c2fe9572c03</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -8200,7 +8200,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>High-resolution record of 8-m seawater CO2 content entering Fanny Bay Oysters in Baynes Sound, British Columbia, Canada from March 2017 to November 2017</t>
+          <t>Zooplankton - Taxonomy – Northern Strait of Georgia, Discovery Islands, Johnstone Strait, and Queen Charlotte Strait – April to July 2015 and 2016</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -8223,7 +8223,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>underDevelopment</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -8242,11 +8242,11 @@
         </is>
       </c>
       <c r="N72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.88983154296876, 49.44759314103575], [-124.70993041992188, 49.44759314103575], [-124.70993041992188, 49.56975910961884], [-124.88983154296876, 49.56975910961884], [-124.88983154296876, 49.44759314103575]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.93452704, 49.56730131], [-124.18481219, 49.56730131], [-124.18481219, 50.90762515], [-126.93452704, 50.90762515], [-126.93452704, 49.56730131]]]}</t>
         </is>
       </c>
       <c r="P72" t="inlineStr">
@@ -8256,17 +8256,17 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, zooplanktonBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>10.21966/1.622315</t>
+          <t>10.21966/bhqd-9361</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTV4aEZoVWsyRXpHWno</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZhamNPb0U3cThnR0o</t>
         </is>
       </c>
       <c r="T72" t="inlineStr">
@@ -8276,20 +8276,18 @@
       </c>
       <c r="U72" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="V72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W72" t="inlineStr">
         <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X72" t="n">
-        <v>1</v>
-      </c>
+          <t>[{'year': '2026', 'total': 1}]</t>
+        </is>
+      </c>
+      <c r="X72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -8407,12 +8405,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8422,7 +8420,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -8464,16 +8462,16 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -8483,12 +8481,12 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T74" t="inlineStr">
@@ -8498,7 +8496,7 @@
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V74" t="n">
@@ -8517,12 +8515,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8532,7 +8530,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8574,16 +8572,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8593,12 +8591,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8608,7 +8606,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -9177,12 +9175,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>8d3f619f-e3e5-44a7-8b35-7e4ed1e6af31</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_d2e83e40-9e95-4a47-a899-b37c744be3ab</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9192,7 +9190,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Fin Island &amp; K'yel - 2020 - Airborne Coastal Observatory Data</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9210,7 +9208,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -9238,7 +9236,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.4, 53.03], [-129.1, 53.03], [-129.1, 53.29], [-129.4, 53.29], [-129.4, 53.03]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
@@ -9253,12 +9251,12 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>10.21966/q4c4-wx08</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNm5cwomXVNI6vWU-R</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -9268,7 +9266,7 @@
       </c>
       <c r="U81" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="V81" t="n">
@@ -9287,12 +9285,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>8d3f619f-e3e5-44a7-8b35-7e4ed1e6af31</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_d2e83e40-9e95-4a47-a899-b37c744be3ab</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -9302,7 +9300,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Fin Island &amp; K'yel - 2020 - Airborne Coastal Observatory Data</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -9320,7 +9318,7 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J82" t="inlineStr">
@@ -9348,7 +9346,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.4, 53.03], [-129.1, 53.03], [-129.1, 53.29], [-129.4, 53.29], [-129.4, 53.03]]]}</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
@@ -9363,12 +9361,12 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/q4c4-wx08</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNm5cwomXVNI6vWU-R</t>
         </is>
       </c>
       <c r="T82" t="inlineStr">
@@ -9378,7 +9376,7 @@
       </c>
       <c r="U82" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V82" t="n">
@@ -9389,9 +9387,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X82" t="n">
-        <v>1</v>
-      </c>
+      <c r="X82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -9839,12 +9835,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>6b93216b-4bbe-4204-a2c3-551a667d00fd</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ca-cioos_94cdfcba-bbd4-4053-8976-75de69460c14</t>
+          <t>ca-cioos_6ae1b131-d903-44ca-92a9-64cf6487ddc2</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -9854,7 +9850,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Sea wrack wet to dry biomass calibrations for macroalgae of the Central Coast of British Columbia - 2018</t>
+          <t>Geology - Calvert Island</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -9872,7 +9868,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -9900,27 +9896,27 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16116765, 51.64326925], [-128.11481908, 51.64326925], [-128.11481908, 51.66904109], [-128.16116765, 51.66904109], [-128.16116765, 51.64326925]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.402632657661314], [-127.8204345703125, 51.402632657661314], [-127.8204345703125, 51.7644403180351], [-128.2489013671875, 51.7644403180351], [-128.2489013671875, 51.402632657661314]]]}</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>other, microbeBiomassAndDiversity</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>10.21966/ez7j-cy15</t>
+          <t>10.21966/f6bn-9773</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFWNFc0dmtoV0UyT2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFhaHEzRGxZdnRTMUM</t>
         </is>
       </c>
       <c r="T87" t="inlineStr">
@@ -9930,7 +9926,7 @@
       </c>
       <c r="U87" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V87" t="n">
@@ -9949,12 +9945,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>6b93216b-4bbe-4204-a2c3-551a667d00fd</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ca-cioos_6ae1b131-d903-44ca-92a9-64cf6487ddc2</t>
+          <t>ca-cioos_94cdfcba-bbd4-4053-8976-75de69460c14</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -9964,7 +9960,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Geology - Calvert Island</t>
+          <t>Sea wrack wet to dry biomass calibrations for macroalgae of the Central Coast of British Columbia - 2018</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -9982,7 +9978,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -10010,27 +10006,27 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.402632657661314], [-127.8204345703125, 51.402632657661314], [-127.8204345703125, 51.7644403180351], [-128.2489013671875, 51.7644403180351], [-128.2489013671875, 51.402632657661314]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16116765, 51.64326925], [-128.11481908, 51.64326925], [-128.11481908, 51.66904109], [-128.16116765, 51.66904109], [-128.16116765, 51.64326925]]]}</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, microbeBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>10.21966/f6bn-9773</t>
+          <t>10.21966/ez7j-cy15</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFhaHEzRGxZdnRTMUM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFWNFc0dmtoV0UyT2k</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -10040,7 +10036,7 @@
       </c>
       <c r="U88" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V88" t="n">
@@ -13029,12 +13025,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -13044,7 +13040,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -13067,7 +13063,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -13086,11 +13082,11 @@
         </is>
       </c>
       <c r="N116" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -13105,12 +13101,12 @@
       </c>
       <c r="R116" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T116" t="inlineStr">
@@ -13120,7 +13116,7 @@
       </c>
       <c r="U116" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V116" t="n">
@@ -13128,7 +13124,7 @@
       </c>
       <c r="W116" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X116" t="inlineStr"/>
@@ -13139,12 +13135,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -13154,7 +13150,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -13177,7 +13173,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -13196,11 +13192,11 @@
         </is>
       </c>
       <c r="N117" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P117" t="inlineStr">
@@ -13215,12 +13211,12 @@
       </c>
       <c r="R117" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S117" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T117" t="inlineStr">
@@ -13230,7 +13226,7 @@
       </c>
       <c r="U117" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V117" t="n">
@@ -13238,7 +13234,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X117" t="inlineStr"/>
@@ -22923,7 +22919,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X205" t="inlineStr"/>
+      <c r="X205" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -31375,9 +31373,7 @@
       </c>
       <c r="V282" t="inlineStr"/>
       <c r="W282" t="inlineStr"/>
-      <c r="X282" t="n">
-        <v>1</v>
-      </c>
+      <c r="X282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="n">
@@ -31385,12 +31381,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
+          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
+          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -31400,7 +31396,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -31446,7 +31442,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
         </is>
       </c>
       <c r="P283" t="inlineStr">
@@ -31461,12 +31457,12 @@
       </c>
       <c r="R283" t="inlineStr">
         <is>
-          <t>10.21966/r9zr-xz33</t>
+          <t>10.21966/vpz7-mm73</t>
         </is>
       </c>
       <c r="S283" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
         </is>
       </c>
       <c r="T283" t="inlineStr">
@@ -31495,12 +31491,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
+          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
+          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -31510,7 +31506,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -31556,7 +31552,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
         </is>
       </c>
       <c r="P284" t="inlineStr">
@@ -31571,12 +31567,12 @@
       </c>
       <c r="R284" t="inlineStr">
         <is>
-          <t>10.21966/9dbb-5d54</t>
+          <t>10.21966/r9zr-xz33</t>
         </is>
       </c>
       <c r="S284" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
         </is>
       </c>
       <c r="T284" t="inlineStr">
@@ -31605,12 +31601,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
+          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
+          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -31620,7 +31616,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -31666,7 +31662,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
         </is>
       </c>
       <c r="P285" t="inlineStr">
@@ -31681,12 +31677,12 @@
       </c>
       <c r="R285" t="inlineStr">
         <is>
-          <t>10.21966/vpz7-mm73</t>
+          <t>10.21966/9dbb-5d54</t>
         </is>
       </c>
       <c r="S285" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
         </is>
       </c>
       <c r="T285" t="inlineStr">
@@ -32045,12 +32041,12 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
+          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
+          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -32060,7 +32056,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -32106,7 +32102,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
         </is>
       </c>
       <c r="P289" t="inlineStr">
@@ -32121,12 +32117,12 @@
       </c>
       <c r="R289" t="inlineStr">
         <is>
-          <t>10.21966/kde9-8g12</t>
+          <t>10.21966/9a97-2j48</t>
         </is>
       </c>
       <c r="S289" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
         </is>
       </c>
       <c r="T289" t="inlineStr">
@@ -32155,12 +32151,12 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
+          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
+          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -32170,7 +32166,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -32216,7 +32212,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
         </is>
       </c>
       <c r="P290" t="inlineStr">
@@ -32231,12 +32227,12 @@
       </c>
       <c r="R290" t="inlineStr">
         <is>
-          <t>10.21966/9a97-2j48</t>
+          <t>10.21966/ed9w-2653</t>
         </is>
       </c>
       <c r="S290" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
         </is>
       </c>
       <c r="T290" t="inlineStr">
@@ -32265,12 +32261,12 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
+          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
+          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -32280,7 +32276,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -32326,7 +32322,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
         </is>
       </c>
       <c r="P291" t="inlineStr">
@@ -32341,12 +32337,12 @@
       </c>
       <c r="R291" t="inlineStr">
         <is>
-          <t>10.21966/ed9w-2653</t>
+          <t>10.21966/kde9-8g12</t>
         </is>
       </c>
       <c r="S291" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
         </is>
       </c>
       <c r="T291" t="inlineStr">
@@ -32595,12 +32591,12 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
+          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
+          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -32610,7 +32606,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -32656,7 +32652,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
         </is>
       </c>
       <c r="P294" t="inlineStr">
@@ -32671,12 +32667,12 @@
       </c>
       <c r="R294" t="inlineStr">
         <is>
-          <t>10.21966/hjkj-6611</t>
+          <t>10.21966/npe4-3036</t>
         </is>
       </c>
       <c r="S294" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
         </is>
       </c>
       <c r="T294" t="inlineStr">
@@ -32815,12 +32811,12 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
+          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
+          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -32830,7 +32826,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -32876,7 +32872,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
         </is>
       </c>
       <c r="P296" t="inlineStr">
@@ -32891,12 +32887,12 @@
       </c>
       <c r="R296" t="inlineStr">
         <is>
-          <t>10.21966/npe4-3036</t>
+          <t>10.21966/hjkj-6611</t>
         </is>
       </c>
       <c r="S296" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
         </is>
       </c>
       <c r="T296" t="inlineStr">

</xml_diff>

<commit_message>
Deployed 08fd6fe98 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X302"/>
+  <dimension ref="A1:X304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6105,12 +6105,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6176,17 +6176,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -6215,12 +6215,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6286,17 +6286,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -9835,12 +9835,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>6b93216b-4bbe-4204-a2c3-551a667d00fd</t>
+          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>ca-cioos_6ae1b131-d903-44ca-92a9-64cf6487ddc2</t>
+          <t>ca-cioos_94cdfcba-bbd4-4053-8976-75de69460c14</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -9850,7 +9850,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Geology - Calvert Island</t>
+          <t>Sea wrack wet to dry biomass calibrations for macroalgae of the Central Coast of British Columbia - 2018</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -9868,7 +9868,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Nearshore, Geospatial</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -9896,27 +9896,27 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.402632657661314], [-127.8204345703125, 51.402632657661314], [-127.8204345703125, 51.7644403180351], [-128.2489013671875, 51.7644403180351], [-128.2489013671875, 51.402632657661314]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16116765, 51.64326925], [-128.11481908, 51.64326925], [-128.11481908, 51.66904109], [-128.16116765, 51.66904109], [-128.16116765, 51.64326925]]]}</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, microbeBiomassAndDiversity</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>10.21966/f6bn-9773</t>
+          <t>10.21966/ez7j-cy15</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFhaHEzRGxZdnRTMUM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFWNFc0dmtoV0UyT2k</t>
         </is>
       </c>
       <c r="T87" t="inlineStr">
@@ -9926,7 +9926,7 @@
       </c>
       <c r="U87" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="V87" t="n">
@@ -9945,12 +9945,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>52048599-9a0c-4d33-861f-26eaedc86bd5</t>
+          <t>6b93216b-4bbe-4204-a2c3-551a667d00fd</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>ca-cioos_94cdfcba-bbd4-4053-8976-75de69460c14</t>
+          <t>ca-cioos_6ae1b131-d903-44ca-92a9-64cf6487ddc2</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -9960,7 +9960,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Sea wrack wet to dry biomass calibrations for macroalgae of the Central Coast of British Columbia - 2018</t>
+          <t>Geology - Calvert Island</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>Nearshore, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -10006,27 +10006,27 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16116765, 51.64326925], [-128.11481908, 51.64326925], [-128.11481908, 51.66904109], [-128.16116765, 51.66904109], [-128.16116765, 51.64326925]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.2489013671875, 51.402632657661314], [-127.8204345703125, 51.402632657661314], [-127.8204345703125, 51.7644403180351], [-128.2489013671875, 51.7644403180351], [-128.2489013671875, 51.402632657661314]]]}</t>
         </is>
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>other, microbeBiomassAndDiversity</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>10.21966/ez7j-cy15</t>
+          <t>10.21966/f6bn-9773</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFWNFc0dmtoV0UyT2k</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTFhaHEzRGxZdnRTMUM</t>
         </is>
       </c>
       <c r="T88" t="inlineStr">
@@ -10036,7 +10036,7 @@
       </c>
       <c r="U88" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="V88" t="n">
@@ -15107,7 +15107,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X134" t="inlineStr"/>
+      <c r="X134" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -19399,7 +19401,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X173" t="inlineStr"/>
+      <c r="X173" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -20609,7 +20613,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X184" t="inlineStr"/>
+      <c r="X184" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -22908,7 +22914,7 @@
       </c>
       <c r="U205" t="inlineStr">
         <is>
-          <t>2024-12-19</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="V205" t="n">
@@ -30708,7 +30714,7 @@
       </c>
       <c r="U276" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="V276" t="n">
@@ -30719,9 +30725,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X276" t="n">
-        <v>1</v>
-      </c>
+      <c r="X276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -31381,12 +31385,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
+          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
+          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -31396,7 +31400,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -31442,7 +31446,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
         </is>
       </c>
       <c r="P283" t="inlineStr">
@@ -31457,12 +31461,12 @@
       </c>
       <c r="R283" t="inlineStr">
         <is>
-          <t>10.21966/vpz7-mm73</t>
+          <t>10.21966/r9zr-xz33</t>
         </is>
       </c>
       <c r="S283" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
         </is>
       </c>
       <c r="T283" t="inlineStr">
@@ -31491,12 +31495,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
+          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
+          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -31506,7 +31510,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -31552,7 +31556,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
         </is>
       </c>
       <c r="P284" t="inlineStr">
@@ -31567,12 +31571,12 @@
       </c>
       <c r="R284" t="inlineStr">
         <is>
-          <t>10.21966/r9zr-xz33</t>
+          <t>10.21966/9dbb-5d54</t>
         </is>
       </c>
       <c r="S284" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
         </is>
       </c>
       <c r="T284" t="inlineStr">
@@ -31601,12 +31605,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
+          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
+          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -31616,7 +31620,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -31662,7 +31666,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
         </is>
       </c>
       <c r="P285" t="inlineStr">
@@ -31677,12 +31681,12 @@
       </c>
       <c r="R285" t="inlineStr">
         <is>
-          <t>10.21966/9dbb-5d54</t>
+          <t>10.21966/vpz7-mm73</t>
         </is>
       </c>
       <c r="S285" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
         </is>
       </c>
       <c r="T285" t="inlineStr">
@@ -32041,12 +32045,12 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
+          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
+          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -32056,7 +32060,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -32102,7 +32106,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
         </is>
       </c>
       <c r="P289" t="inlineStr">
@@ -32117,12 +32121,12 @@
       </c>
       <c r="R289" t="inlineStr">
         <is>
-          <t>10.21966/9a97-2j48</t>
+          <t>10.21966/kde9-8g12</t>
         </is>
       </c>
       <c r="S289" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
         </is>
       </c>
       <c r="T289" t="inlineStr">
@@ -32151,12 +32155,12 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
+          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
+          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -32166,7 +32170,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -32212,7 +32216,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
         </is>
       </c>
       <c r="P290" t="inlineStr">
@@ -32227,12 +32231,12 @@
       </c>
       <c r="R290" t="inlineStr">
         <is>
-          <t>10.21966/ed9w-2653</t>
+          <t>10.21966/9a97-2j48</t>
         </is>
       </c>
       <c r="S290" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
         </is>
       </c>
       <c r="T290" t="inlineStr">
@@ -32261,12 +32265,12 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
+          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
+          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -32276,7 +32280,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -32322,7 +32326,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
         </is>
       </c>
       <c r="P291" t="inlineStr">
@@ -32337,12 +32341,12 @@
       </c>
       <c r="R291" t="inlineStr">
         <is>
-          <t>10.21966/kde9-8g12</t>
+          <t>10.21966/ed9w-2653</t>
         </is>
       </c>
       <c r="S291" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
         </is>
       </c>
       <c r="T291" t="inlineStr">
@@ -32591,12 +32595,12 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
+          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
+          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -32606,7 +32610,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -32652,7 +32656,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
         </is>
       </c>
       <c r="P294" t="inlineStr">
@@ -32667,12 +32671,12 @@
       </c>
       <c r="R294" t="inlineStr">
         <is>
-          <t>10.21966/npe4-3036</t>
+          <t>10.21966/hjkj-6611</t>
         </is>
       </c>
       <c r="S294" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
         </is>
       </c>
       <c r="T294" t="inlineStr">
@@ -32811,12 +32815,12 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
+          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
+          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -32826,7 +32830,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -32872,7 +32876,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
         </is>
       </c>
       <c r="P296" t="inlineStr">
@@ -32887,12 +32891,12 @@
       </c>
       <c r="R296" t="inlineStr">
         <is>
-          <t>10.21966/hjkj-6611</t>
+          <t>10.21966/npe4-3036</t>
         </is>
       </c>
       <c r="S296" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
         </is>
       </c>
       <c r="T296" t="inlineStr">
@@ -33471,105 +33475,317 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
+          <t>d269f354-8527-4e94-bb32-9de4fe3fabdf</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>ca-cioos_da232383-781d-4852-8542-cf0cb8aa5f26</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>Data for Paper: Detection differences between eDNA and mid-water trawls are driven by fish biomass and habitat preferences</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>CC-BY-NC-ND-4.0</t>
+        </is>
+      </c>
+      <c r="H302" t="b">
+        <v>0</v>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>Genomics</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N302" t="n">
+        <v>3</v>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.6289, 50.7424], [-127.321, 50.6868], [-124.8052, 48.3262], [-123.2452, 48.1432], [-122.9596, 49.0945], [-126.6289, 50.7424]]]}</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>fishAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>10.21966/hky6-1022</t>
+        </is>
+      </c>
+      <c r="S302" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-P1l_Wv09HnWD1is-Yik</t>
+        </is>
+      </c>
+      <c r="T302" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="U302" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="V302" t="n">
+        <v>0</v>
+      </c>
+      <c r="W302" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X302" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="n">
+        <v>301</v>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>098c52a1-6dde-4e64-8b27-5a34e40870e6</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>ca-cioos_e5e61f93-db9b-48d0-b779-45e73fabfd0a</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>High Resolution Coastal Carbon Monitoring in the Northeast Pacific</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>collection</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H303" t="b">
+        <v>0</v>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>Oceanography</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>onGoing</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="N303" t="n">
+        <v>1</v>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-160.4964, 46.7847], [-118.6667, 46.7847], [-118.6667, 62.7421], [-160.4964, 62.7421], [-160.4964, 46.7847]]]}</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>[{'max': '0', 'min': '0'}]</t>
+        </is>
+      </c>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>inorganicCarbon</t>
+        </is>
+      </c>
+      <c r="R303" t="inlineStr"/>
+      <c r="S303" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-P0csr75piiewsICpJu8</t>
+        </is>
+      </c>
+      <c r="T303" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="U303" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="V303" t="inlineStr"/>
+      <c r="W303" t="inlineStr"/>
+      <c r="X303" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>302</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
           <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
         </is>
       </c>
-      <c r="C302" t="inlineStr">
+      <c r="C304" t="inlineStr">
         <is>
           <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
         </is>
       </c>
-      <c r="D302" t="inlineStr">
-        <is>
-          <t>Hakai Institute</t>
-        </is>
-      </c>
-      <c r="E302" t="inlineStr">
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
         <is>
           <t>Mount Robson Aerial Photo and LiDAR Survey</t>
         </is>
       </c>
-      <c r="F302" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="G302" t="inlineStr">
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
         <is>
           <t>CC-BY-4.0</t>
         </is>
       </c>
-      <c r="H302" t="b">
-        <v>0</v>
-      </c>
-      <c r="I302" t="inlineStr">
+      <c r="H304" t="b">
+        <v>0</v>
+      </c>
+      <c r="I304" t="inlineStr">
         <is>
           <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
-      <c r="J302" t="inlineStr">
+      <c r="J304" t="inlineStr">
         <is>
           <t>completed</t>
         </is>
       </c>
-      <c r="K302" t="inlineStr">
+      <c r="K304" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="L302" t="inlineStr">
-        <is>
-          <t>dataset</t>
-        </is>
-      </c>
-      <c r="M302" t="inlineStr">
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M304" t="inlineStr">
         <is>
           <t>Tula Foundation</t>
         </is>
       </c>
-      <c r="N302" t="n">
+      <c r="N304" t="n">
         <v>1</v>
       </c>
-      <c r="O302" t="inlineStr">
+      <c r="O304" t="inlineStr">
         <is>
           <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
-      <c r="P302" t="inlineStr">
+      <c r="P304" t="inlineStr">
         <is>
           <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
-      <c r="Q302" t="inlineStr">
+      <c r="Q304" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="R302" t="inlineStr">
+      <c r="R304" t="inlineStr">
         <is>
           <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
-      <c r="S302" t="inlineStr">
+      <c r="S304" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
         </is>
       </c>
-      <c r="T302" t="inlineStr"/>
-      <c r="U302" t="inlineStr">
+      <c r="T304" t="inlineStr"/>
+      <c r="U304" t="inlineStr">
         <is>
           <t>2025-04-02</t>
         </is>
       </c>
-      <c r="V302" t="n">
-        <v>0</v>
-      </c>
-      <c r="W302" t="inlineStr">
+      <c r="V304" t="n">
+        <v>0</v>
+      </c>
+      <c r="W304" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="X302" t="inlineStr"/>
+      <c r="X304" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deployed 0dfded112 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X304"/>
+  <dimension ref="A1:X305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2163,7 +2163,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr"/>
+      <c r="X16" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -13355,12 +13357,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
+          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
+          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -13370,7 +13372,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
+          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -13388,12 +13390,12 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -13412,16 +13414,16 @@
         </is>
       </c>
       <c r="N119" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
         </is>
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr">
@@ -13431,12 +13433,12 @@
       </c>
       <c r="R119" t="inlineStr">
         <is>
-          <t>10.21966/vavm-b152</t>
+          <t>10.21966/7nb6-zk37</t>
         </is>
       </c>
       <c r="S119" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
         </is>
       </c>
       <c r="T119" t="inlineStr">
@@ -13465,12 +13467,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>bfad4541-a06a-489e-bd95-a5e7c65e0dc1</t>
+          <t>e1b86825-d43b-47e1-bf45-ab791f44772d</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>ca-cioos_0e446321-34f3-4d5a-8c7d-79c89eb76373</t>
+          <t>ca-cioos_0e4f324c-6498-4c89-9e19-f2f9f474a1df</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -13480,7 +13482,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Stream temperature time-series – Calvert Island – 2013 - 2019</t>
+          <t>LiDAR-derived Drainage Network for Calvert Island - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -13498,12 +13500,12 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -13522,16 +13524,16 @@
         </is>
       </c>
       <c r="N120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.25940955, 51.55841821], [-127.87488807, 51.55841821], [-127.87488807, 51.75224257], [-128.25940955, 51.75224257], [-128.25940955, 51.55841821]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16, 51.41], [-127.88, 51.41], [-127.88, 51.73], [-128.16, 51.73], [-128.16, 51.41]]]}</t>
         </is>
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -13541,12 +13543,12 @@
       </c>
       <c r="R120" t="inlineStr">
         <is>
-          <t>10.21966/7nb6-zk37</t>
+          <t>10.21966/vavm-b152</t>
         </is>
       </c>
       <c r="S120" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFDT2lYSlBQZ0VNdDg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MW5MeGIydVA3U1VKdWo</t>
         </is>
       </c>
       <c r="T120" t="inlineStr">
@@ -14455,12 +14457,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -14470,7 +14472,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -14488,7 +14490,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -14508,7 +14510,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N129" t="n">
@@ -14516,27 +14518,27 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T129" t="inlineStr">
@@ -14546,7 +14548,7 @@
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V129" t="n">
@@ -14565,12 +14567,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -14580,7 +14582,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -14598,7 +14600,7 @@
       </c>
       <c r="I130" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J130" t="inlineStr">
@@ -14618,7 +14620,7 @@
       </c>
       <c r="M130" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N130" t="n">
@@ -14626,27 +14628,27 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R130" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S130" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T130" t="inlineStr">
@@ -14656,7 +14658,7 @@
       </c>
       <c r="U130" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V130" t="n">
@@ -19401,9 +19403,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X173" t="n">
-        <v>1</v>
-      </c>
+      <c r="X173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -20613,9 +20613,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X184" t="n">
-        <v>1</v>
-      </c>
+      <c r="X184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -22914,7 +22912,7 @@
       </c>
       <c r="U205" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="V205" t="n">
@@ -22925,9 +22923,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X205" t="n">
-        <v>1</v>
-      </c>
+      <c r="X205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -32045,12 +32041,12 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
+          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
+          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -32060,7 +32056,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -32106,7 +32102,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
         </is>
       </c>
       <c r="P289" t="inlineStr">
@@ -32121,12 +32117,12 @@
       </c>
       <c r="R289" t="inlineStr">
         <is>
-          <t>10.21966/kde9-8g12</t>
+          <t>10.21966/9a97-2j48</t>
         </is>
       </c>
       <c r="S289" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
         </is>
       </c>
       <c r="T289" t="inlineStr">
@@ -32155,12 +32151,12 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
+          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
+          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -32170,7 +32166,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -32216,7 +32212,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
         </is>
       </c>
       <c r="P290" t="inlineStr">
@@ -32231,12 +32227,12 @@
       </c>
       <c r="R290" t="inlineStr">
         <is>
-          <t>10.21966/9a97-2j48</t>
+          <t>10.21966/kde9-8g12</t>
         </is>
       </c>
       <c r="S290" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
         </is>
       </c>
       <c r="T290" t="inlineStr">
@@ -33578,7 +33574,7 @@
         </is>
       </c>
       <c r="X302" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="303">
@@ -33679,7 +33675,9 @@
       </c>
       <c r="V303" t="inlineStr"/>
       <c r="W303" t="inlineStr"/>
-      <c r="X303" t="inlineStr"/>
+      <c r="X303" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="n">
@@ -33687,12 +33685,12 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+          <t>1e13d2ee-580f-4785-838b-908a449781a3</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+          <t>ca-cioos_741bd412-6387-4dcd-8d61-7046b949f406</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
@@ -33702,7 +33700,7 @@
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+          <t>Global Eutrophication Monitoring Dataset of Trinidad and Tobago</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
@@ -33720,12 +33718,12 @@
       </c>
       <c r="I304" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J304" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K304" t="inlineStr">
@@ -33740,7 +33738,7 @@
       </c>
       <c r="M304" t="inlineStr">
         <is>
-          <t>Tula Foundation</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N304" t="n">
@@ -33748,44 +33746,156 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-61.59, 10.35], [-61.46, 10.35], [-61.46, 10.68], [-61.59, 10.68], [-61.59, 10.35]]]}</t>
+        </is>
+      </c>
+      <c r="P304" t="inlineStr">
+        <is>
+          <t>[{'max': '1.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>nutrients, particulateMatter, oxygen, phytoplanktonBiomassAndDiversity, zooplanktonBiomassAndDiversity, seaSurfaceTemperature, subSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity</t>
+        </is>
+      </c>
+      <c r="R304" t="inlineStr">
+        <is>
+          <t>10.21966/nrrn-rr63</t>
+        </is>
+      </c>
+      <c r="S304" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/P3VNaxsDaISmZcvgBvJIKlt634d2/-Op0_nycnfen8FFkS3Ti</t>
+        </is>
+      </c>
+      <c r="T304" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="U304" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="V304" t="n">
+        <v>0</v>
+      </c>
+      <c r="W304" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X304" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>303</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>0cef18ab-cea6-4522-baba-1bcd73a30646</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>ca-cioos_66fbb7f5-3644-471a-95ee-f8d3758e888b</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Hakai Institute</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Mount Robson Aerial Photo and LiDAR Survey</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="H305" t="b">
+        <v>0</v>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory, Geospatial</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>dataset</t>
+        </is>
+      </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>Tula Foundation</t>
+        </is>
+      </c>
+      <c r="N305" t="n">
+        <v>1</v>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
           <t>{'type': 'Polygon', 'coordinates': [[[-119.3, 53.03], [-118.8, 53.03], [-118.8, 53.26], [-119.3, 53.26], [-119.3, 53.03]]]}</t>
         </is>
       </c>
-      <c r="P304" t="inlineStr">
+      <c r="P305" t="inlineStr">
         <is>
           <t>[{'max': '3954.0', 'min': '800.0'}]</t>
         </is>
       </c>
-      <c r="Q304" t="inlineStr">
+      <c r="Q305" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="R304" t="inlineStr">
+      <c r="R305" t="inlineStr">
         <is>
           <t>10.21966/w9n0-kn30</t>
         </is>
       </c>
-      <c r="S304" t="inlineStr">
+      <c r="S305" t="inlineStr">
         <is>
           <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OICbtZXkj6anGvgB3Qi</t>
         </is>
       </c>
-      <c r="T304" t="inlineStr"/>
-      <c r="U304" t="inlineStr">
+      <c r="T305" t="inlineStr"/>
+      <c r="U305" t="inlineStr">
         <is>
           <t>2025-04-02</t>
         </is>
       </c>
-      <c r="V304" t="n">
-        <v>0</v>
-      </c>
-      <c r="W304" t="inlineStr">
+      <c r="V305" t="n">
+        <v>0</v>
+      </c>
+      <c r="W305" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="X304" t="inlineStr"/>
+      <c r="X305" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deployed 45a6a1935 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -6105,12 +6105,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6176,17 +6176,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -6215,12 +6215,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6286,17 +6286,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -8405,12 +8405,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8420,7 +8420,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -8462,16 +8462,16 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -8481,12 +8481,12 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T74" t="inlineStr">
@@ -8496,7 +8496,7 @@
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V74" t="n">
@@ -8515,12 +8515,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8530,7 +8530,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -8572,16 +8572,16 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -8591,12 +8591,12 @@
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T75" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="U75" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V75" t="n">
@@ -15005,12 +15005,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -15020,7 +15020,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -15038,7 +15038,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -15058,20 +15058,20 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N134" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -15081,12 +15081,12 @@
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -15096,7 +15096,7 @@
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V134" t="n">
@@ -15115,12 +15115,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -15130,7 +15130,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -15148,7 +15148,7 @@
       </c>
       <c r="I135" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J135" t="inlineStr">
@@ -15168,20 +15168,20 @@
       </c>
       <c r="M135" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N135" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -15191,12 +15191,12 @@
       </c>
       <c r="R135" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S135" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T135" t="inlineStr">
@@ -15206,7 +15206,7 @@
       </c>
       <c r="U135" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V135" t="n">
@@ -19399,7 +19399,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X173" t="inlineStr"/>
+      <c r="X173" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">

</xml_diff>

<commit_message>
Deployed d07856efe to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -6105,12 +6105,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6120,7 +6120,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6176,17 +6176,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6196,7 +6196,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -6215,12 +6215,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -6276,7 +6276,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P54" t="inlineStr">
@@ -6286,17 +6286,17 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T54" t="inlineStr">
@@ -6306,7 +6306,7 @@
       </c>
       <c r="U54" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V54" t="n">
@@ -8955,12 +8955,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>5b78f1a7-6adb-4610-9ebe-019c3da65ae8</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_bb59cb9e-887a-40a3-b41a-f4a5b2263ce6</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8970,7 +8970,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Fountain Valley LiDAR Data - 2019 &amp; 2020 - Hakai Airborne Coastal Observatory - British Columbia - Canada</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -9016,12 +9016,12 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-122.0, 50.56], [-121.7, 50.56], [-121.7, 50.8], [-122.0, 50.8], [-122.0, 50.56]]]}</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -9031,12 +9031,12 @@
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/8f0v-t572</t>
         </is>
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MmUnbGWVNvtiQAsYVPj</t>
         </is>
       </c>
       <c r="T79" t="inlineStr">
@@ -9046,7 +9046,7 @@
       </c>
       <c r="U79" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="V79" t="n">
@@ -9065,12 +9065,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -9080,7 +9080,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -9098,7 +9098,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -9126,12 +9126,12 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -9141,12 +9141,12 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T80" t="inlineStr">
@@ -9175,12 +9175,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>5b78f1a7-6adb-4610-9ebe-019c3da65ae8</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>ca-cioos_bb59cb9e-887a-40a3-b41a-f4a5b2263ce6</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -9190,7 +9190,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Fountain Valley LiDAR Data - 2019 &amp; 2020 - Hakai Airborne Coastal Observatory - British Columbia - Canada</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -9208,7 +9208,7 @@
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J81" t="inlineStr">
@@ -9236,12 +9236,12 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-122.0, 50.56], [-121.7, 50.56], [-121.7, 50.8], [-122.0, 50.8], [-122.0, 50.56]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>[{'max': '1500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -9251,12 +9251,12 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>10.21966/8f0v-t572</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MmUnbGWVNvtiQAsYVPj</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T81" t="inlineStr">
@@ -9266,7 +9266,7 @@
       </c>
       <c r="U81" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-10</t>
         </is>
       </c>
       <c r="V81" t="n">
@@ -9497,9 +9497,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X83" t="n">
-        <v>1</v>
-      </c>
+      <c r="X83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -14009,7 +14007,9 @@
           <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X124" t="inlineStr"/>
+      <c r="X124" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -18859,12 +18859,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
+          <t>75b60436-da51-4ccf-b14a-27f45f782b2b</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>ca-cioos_24f1c230-6c37-470c-907d-25b9b022f5c2</t>
+          <t>ca-cioos_476204a7-0714-4755-953d-61fa3c5df497</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -18874,7 +18874,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Differential infestation of juvenile Pacific salmon by parasitic sea lice in British Columbia, Canada</t>
+          <t>Hakai Institute Nutrients (Dosser et al., 2021)</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -18892,7 +18892,7 @@
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>Juvenile Salmon Program</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -18920,27 +18920,27 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.87477074, 49.80151064], [-124.30109865, 49.80151064], [-124.30109865, 50.66883255], [-126.87477074, 50.66883255], [-126.87477074, 49.80151064]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.6, 50.69], [-126.3, 50.8], [-124.8, 50.44], [-123.9, 49.65], [-125.1, 49.65], [-127.6, 50.69]]]}</t>
         </is>
       </c>
       <c r="P169" t="inlineStr">
         <is>
-          <t>[{'max': '9.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q169" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>nutrients</t>
         </is>
       </c>
       <c r="R169" t="inlineStr">
         <is>
-          <t>10.21966/54tw-kh93</t>
+          <t>10.21966/j3j5-wt70</t>
         </is>
       </c>
       <c r="S169" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZDeElXT3dpUFNlOGQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/oOseiEWez6TzqPUIisEXczg6G8y2/-MoZtzH-n9LBy9Bn29Hl</t>
         </is>
       </c>
       <c r="T169" t="inlineStr">
@@ -18950,7 +18950,7 @@
       </c>
       <c r="U169" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="V169" t="n">
@@ -18969,12 +18969,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>75b60436-da51-4ccf-b14a-27f45f782b2b</t>
+          <t>2709d7b1-22e1-4268-bcda-dc0c79f2878e</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>ca-cioos_476204a7-0714-4755-953d-61fa3c5df497</t>
+          <t>ca-cioos_24f1c230-6c37-470c-907d-25b9b022f5c2</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -18984,7 +18984,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Hakai Institute Nutrients (Dosser et al., 2021)</t>
+          <t>Differential infestation of juvenile Pacific salmon by parasitic sea lice in British Columbia, Canada</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -19002,7 +19002,7 @@
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Juvenile Salmon Program</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -19030,27 +19030,27 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.6, 50.69], [-126.3, 50.8], [-124.8, 50.44], [-123.9, 49.65], [-125.1, 49.65], [-127.6, 50.69]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.87477074, 49.80151064], [-124.30109865, 49.80151064], [-124.30109865, 50.66883255], [-126.87477074, 50.66883255], [-126.87477074, 49.80151064]]]}</t>
         </is>
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '9.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q170" t="inlineStr">
         <is>
-          <t>nutrients</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R170" t="inlineStr">
         <is>
-          <t>10.21966/j3j5-wt70</t>
+          <t>10.21966/54tw-kh93</t>
         </is>
       </c>
       <c r="S170" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/oOseiEWez6TzqPUIisEXczg6G8y2/-MoZtzH-n9LBy9Bn29Hl</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MTZDeElXT3dpUFNlOGQ</t>
         </is>
       </c>
       <c r="T170" t="inlineStr">
@@ -19060,7 +19060,7 @@
       </c>
       <c r="U170" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="V170" t="n">
@@ -19181,7 +19181,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X171" t="inlineStr"/>
+      <c r="X171" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -19401,9 +19403,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X173" t="n">
-        <v>1</v>
-      </c>
+      <c r="X173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -21823,9 +21823,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X195" t="n">
-        <v>1</v>
-      </c>
+      <c r="X195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -28311,7 +28309,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X254" t="inlineStr"/>
+      <c r="X254" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -28531,7 +28531,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X256" t="inlineStr"/>
+      <c r="X256" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -30399,12 +30401,12 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
+          <t>3988f8e8-36ea-4cda-9bd9-a03157116ef5</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>ca-cioos_53189107-9df5-426b-acb4-f903468554fe</t>
+          <t>ca-cioos_d43a79c1-a6ba-4e37-8dc2-6ced6312828e</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
@@ -30414,7 +30416,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Comparing invertebrate and seaweed diversity in kelp forests and urchin barrens in Owen Bay, British Columbia, using Autonomous Reef Monitoring Structures (ARMS)</t>
+          <t>Data from Manuscript: Parasites of the hermit crab Pagurus hirsutiusculus; distribution, prevalence, and thermal ecology</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
@@ -30432,7 +30434,7 @@
       </c>
       <c r="I274" t="inlineStr">
         <is>
-          <t>Sentinels of Change, Genomics</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J274" t="inlineStr">
@@ -30456,41 +30458,41 @@
         </is>
       </c>
       <c r="N274" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.2335, 50.2999], [-125.2163, 50.2999], [-125.2163, 50.313], [-125.2335, 50.313], [-125.2335, 50.2999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.4, 51.66], [-127.9, 51.81], [-122.2, 49.03], [-123.3, 49.01], [-123.0, 48.83], [-123.0, 48.78], [-123.3, 48.7], [-123.3, 48.53], [-123.6, 48.59], [-125.2, 48.73], [-125.6, 48.95], [-125.6, 50.11], [-128.4, 51.66]]]}</t>
         </is>
       </c>
       <c r="P274" t="inlineStr">
         <is>
-          <t>[{'max': '6.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q274" t="inlineStr">
         <is>
-          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
+          <t>invertebrateAbundanceAndDistribution, seaSurfaceSalinity</t>
         </is>
       </c>
       <c r="R274" t="inlineStr">
         <is>
-          <t>10.21966/e5mw-tr82</t>
+          <t>10.21966/xb3t-qb88</t>
         </is>
       </c>
       <c r="S274" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/5Jh4rsxoBsRd4mVFqZ0XJoMtMHI2/-P-tq8uNjGhWtk4rBny0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3eh7IMAvm8ZUtcMBeifFL0eJCIA3/-O5Kei32z9cfatfgKj5y</t>
         </is>
       </c>
       <c r="T274" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="U274" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="V274" t="n">
@@ -30501,9 +30503,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X274" t="n">
-        <v>1</v>
-      </c>
+      <c r="X274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -30511,12 +30511,12 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
+          <t>c4932b55-1dd8-4f2f-89da-5822056ecc37</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>ca-cioos_73abfecf-d35c-4f9c-a991-eee5cece08ea</t>
+          <t>ca-cioos_53189107-9df5-426b-acb4-f903468554fe</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
@@ -30526,7 +30526,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>Kelp Canopy Extent 2012 - NW Calvert Island</t>
+          <t>Comparing invertebrate and seaweed diversity in kelp forests and urchin barrens in Owen Bay, British Columbia, using Autonomous Reef Monitoring Structures (ARMS)</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
@@ -30544,7 +30544,7 @@
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>Geospatial</t>
+          <t>Sentinels of Change, Genomics</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
@@ -30568,41 +30568,41 @@
         </is>
       </c>
       <c r="N275" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.16959381103513, 51.63613234359897], [-128.11191558837888, 51.63613234359897], [-128.11191558837888, 51.681709494104325], [-128.16959381103513, 51.681709494104325], [-128.16959381103513, 51.63613234359897]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.2335, 50.2999], [-125.2163, 50.2999], [-125.2163, 50.313], [-125.2335, 50.313], [-125.2335, 50.2999]]]}</t>
         </is>
       </c>
       <c r="P275" t="inlineStr">
         <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
+          <t>[{'max': '6.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q275" t="inlineStr">
         <is>
-          <t>other, macroalgalCanopyCoverAndComposition</t>
+          <t>invertebrateAbundanceAndDistribution, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R275" t="inlineStr">
         <is>
-          <t>10.21966/63rs-yt91</t>
+          <t>10.21966/e5mw-tr82</t>
         </is>
       </c>
       <c r="S275" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxUM01laTFaREhKbWE</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/5Jh4rsxoBsRd4mVFqZ0XJoMtMHI2/-P-tq8uNjGhWtk4rBny0</t>
         </is>
       </c>
       <c r="T275" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="U275" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="V275" t="n">
@@ -30613,7 +30613,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X275" t="inlineStr"/>
+      <c r="X275" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -30621,12 +30623,12 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
+          <t>33bb67af-4d61-4b15-93a9-f3ab2498430b</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>ca-cioos_940218ef-d7f8-4f3f-9e69-52150ecdbec5</t>
+          <t>ca-cioos_73abfecf-d35c-4f9c-a991-eee5cece08ea</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
@@ -30636,7 +30638,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>North Vancouver Island Aerial Survey - 2024 - Airborne Coastal Observatory</t>
+          <t>Kelp Canopy Extent 2012 - NW Calvert Island</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -30654,7 +30656,7 @@
       </c>
       <c r="I276" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory, Geospatial</t>
+          <t>Geospatial</t>
         </is>
       </c>
       <c r="J276" t="inlineStr">
@@ -30678,31 +30680,31 @@
         </is>
       </c>
       <c r="N276" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.7, 50.35], [-125.4, 50.35], [-125.4, 50.63], [-126.7, 50.63], [-126.7, 50.35]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.16959381103513, 51.63613234359897], [-128.11191558837888, 51.63613234359897], [-128.11191558837888, 51.681709494104325], [-128.16959381103513, 51.681709494104325], [-128.16959381103513, 51.63613234359897]]]}</t>
         </is>
       </c>
       <c r="P276" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q276" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, macroalgalCanopyCoverAndComposition</t>
         </is>
       </c>
       <c r="R276" t="inlineStr">
         <is>
-          <t>10.21966/kdhe-hz07</t>
+          <t>10.21966/63rs-yt91</t>
         </is>
       </c>
       <c r="S276" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OCoHpqOwDbp834fqRY3</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUxUM01laTFaREhKbWE</t>
         </is>
       </c>
       <c r="T276" t="inlineStr">
@@ -30712,7 +30714,7 @@
       </c>
       <c r="U276" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="V276" t="n">
@@ -30731,12 +30733,12 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
+          <t>bc1133da-5601-4f92-bc53-41be547c936b</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>ca-cioos_c7466354-bacc-4781-acdc-543dd03d1eab</t>
+          <t>ca-cioos_940218ef-d7f8-4f3f-9e69-52150ecdbec5</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
@@ -30746,7 +30748,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Nanwakolas LiDAR Surveys - Airborne Coastal Observatory</t>
+          <t>North Vancouver Island Aerial Survey - 2024 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -30792,12 +30794,12 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.8, 49.26], [-124.5, 49.26], [-124.5, 50.83], [-126.8, 50.83], [-126.8, 49.26]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.7, 50.35], [-125.4, 50.35], [-125.4, 50.63], [-126.7, 50.63], [-126.7, 50.35]]]}</t>
         </is>
       </c>
       <c r="P277" t="inlineStr">
         <is>
-          <t>[{'max': '1700.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q277" t="inlineStr">
@@ -30807,12 +30809,12 @@
       </c>
       <c r="R277" t="inlineStr">
         <is>
-          <t>10.21966/e0r7-ge27</t>
+          <t>10.21966/kdhe-hz07</t>
         </is>
       </c>
       <c r="S277" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OjbuSE_uZcCs3Fit_mg</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OCoHpqOwDbp834fqRY3</t>
         </is>
       </c>
       <c r="T277" t="inlineStr">
@@ -30822,7 +30824,7 @@
       </c>
       <c r="U277" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="V277" t="n">
@@ -30841,12 +30843,12 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>f7433c1a-3aad-4761-81c4-c191a5e6ac92</t>
+          <t>39818579-9692-4256-9810-d8b80e9821aa</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>ca-cioos_52e97374-bee5-4b1a-9b85-7170a5df8d6b</t>
+          <t>ca-cioos_c7466354-bacc-4781-acdc-543dd03d1eab</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
@@ -30856,7 +30858,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Biomass and density of Pycnopodia helianthoides from the central coast of BC</t>
+          <t>Nanwakolas LiDAR Surveys - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
@@ -30874,7 +30876,7 @@
       </c>
       <c r="I278" t="inlineStr">
         <is>
-          <t>Oceanography, Nearshore</t>
+          <t>Airborne Coastal Observatory, Geospatial</t>
         </is>
       </c>
       <c r="J278" t="inlineStr">
@@ -30902,37 +30904,37 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.617, 51.3321], [-127.3509, 51.3321], [-127.3509, 52.3317], [-128.617, 52.3317], [-128.617, 51.3321]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.8, 49.26], [-124.5, 49.26], [-124.5, 50.83], [-126.8, 50.83], [-126.8, 49.26]]]}</t>
         </is>
       </c>
       <c r="P278" t="inlineStr">
         <is>
-          <t>[{'max': '10.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1700.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q278" t="inlineStr">
         <is>
-          <t>seaSurfaceSalinity, subSurfaceSalinity, seaSurfaceTemperature, subSurfaceTemperature, invertebrateAbundanceAndDistribution</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R278" t="inlineStr">
         <is>
-          <t>10.21966/xy6n-qz76</t>
+          <t>10.21966/e0r7-ge27</t>
         </is>
       </c>
       <c r="S278" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-OteEfuBSvhg-2RySC4a</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-OjbuSE_uZcCs3Fit_mg</t>
         </is>
       </c>
       <c r="T278" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="U278" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="V278" t="n">
@@ -30951,12 +30953,12 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
+          <t>f7433c1a-3aad-4761-81c4-c191a5e6ac92</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>ca-cioos_b4844ae2-d9c1-42f2-ae4d-a8f994c395a0</t>
+          <t>ca-cioos_52e97374-bee5-4b1a-9b85-7170a5df8d6b</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
@@ -30966,7 +30968,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Putting fjord biodiversity on the map for British Columbia conservation planning</t>
+          <t>Biomass and density of Pycnopodia helianthoides from the central coast of BC</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
@@ -30984,7 +30986,7 @@
       </c>
       <c r="I279" t="inlineStr">
         <is>
-          <t>Genomics, Oceanography</t>
+          <t>Oceanography, Nearshore</t>
         </is>
       </c>
       <c r="J279" t="inlineStr">
@@ -31004,45 +31006,45 @@
       </c>
       <c r="M279" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N279" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.0471, 52.2577], [-128.9141, 51.7033], [-127.6841, 50.7687], [-123.7744, 48.9864], [-122.764, 49.331], [-122.8299, 49.9706], [-127.0471, 52.2577]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.617, 51.3321], [-127.3509, 51.3321], [-127.3509, 52.3317], [-128.617, 52.3317], [-128.617, 51.3321]]]}</t>
         </is>
       </c>
       <c r="P279" t="inlineStr">
         <is>
-          <t>[{'max': '595.0', 'min': '0.0'}]</t>
+          <t>[{'max': '10.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q279" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution, subSurfaceTemperature, subSurfaceSalinity</t>
+          <t>seaSurfaceSalinity, subSurfaceSalinity, seaSurfaceTemperature, subSurfaceTemperature, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R279" t="inlineStr">
         <is>
-          <t>10.21966/n141-m959</t>
+          <t>10.21966/xy6n-qz76</t>
         </is>
       </c>
       <c r="S279" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-Ow-ZgW1jkC5-WyrtlLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/Q7WjoEJM1Sc9HrFLJCRgKAtMzTH2/-OteEfuBSvhg-2RySC4a</t>
         </is>
       </c>
       <c r="T279" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="U279" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="V279" t="n">
@@ -31053,9 +31055,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X279" t="n">
-        <v>1</v>
-      </c>
+      <c r="X279" t="inlineStr"/>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -31063,12 +31063,12 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
+          <t>c7a168e8-f15e-446f-a49d-0b4a1f043ac2</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
+          <t>ca-cioos_b4844ae2-d9c1-42f2-ae4d-a8f994c395a0</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
@@ -31078,7 +31078,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
+          <t>Putting fjord biodiversity on the map for British Columbia conservation planning</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
@@ -31096,7 +31096,7 @@
       </c>
       <c r="I280" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Genomics, Oceanography</t>
         </is>
       </c>
       <c r="J280" t="inlineStr">
@@ -31116,56 +31116,58 @@
       </c>
       <c r="M280" t="inlineStr">
         <is>
-          <t>Hakai Institute</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N280" t="n">
+        <v>2</v>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.0471, 52.2577], [-128.9141, 51.7033], [-127.6841, 50.7687], [-123.7744, 48.9864], [-122.764, 49.331], [-122.8299, 49.9706], [-127.0471, 52.2577]]]}</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>[{'max': '595.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>fishAbundanceAndDistribution, subSurfaceTemperature, subSurfaceSalinity</t>
+        </is>
+      </c>
+      <c r="R280" t="inlineStr">
+        <is>
+          <t>10.21966/n141-m959</t>
+        </is>
+      </c>
+      <c r="S280" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-Ow-ZgW1jkC5-WyrtlLV</t>
+        </is>
+      </c>
+      <c r="T280" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="U280" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="V280" t="n">
+        <v>0</v>
+      </c>
+      <c r="W280" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X280" t="n">
         <v>1</v>
       </c>
-      <c r="O280" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
-        </is>
-      </c>
-      <c r="P280" t="inlineStr">
-        <is>
-          <t>[{'max': '2.5', 'min': '2.5'}]</t>
-        </is>
-      </c>
-      <c r="Q280" t="inlineStr">
-        <is>
-          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R280" t="inlineStr">
-        <is>
-          <t>10.21966/rrzq-yw32</t>
-        </is>
-      </c>
-      <c r="S280" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
-        </is>
-      </c>
-      <c r="T280" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="U280" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="V280" t="n">
-        <v>0</v>
-      </c>
-      <c r="W280" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="X280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -31173,12 +31175,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
+          <t>58d56d16-6350-4b01-a062-6bdb2d9f89b4</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
+          <t>ca-cioos_1f1774ff-7398-4099-b89f-59df7ef0749e</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
@@ -31188,17 +31190,17 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
+          <t>Surface underway seawater and marine boundary layer observations of partial pressure of carbon dioxide (pCO2), water temperature, salinity and other parameters made during the M/V Seaspan Royal cruises in the coastal waters of British Columbia, Canada from 2022-07-01 to 2022-12-20</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>collection</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CC-BY-4.0</t>
         </is>
       </c>
       <c r="H281" t="b">
@@ -31211,7 +31213,7 @@
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K281" t="inlineStr">
@@ -31234,23 +31236,27 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-134.4, 48.0], [-122.6, 48.0], [-122.6, 56.0], [-134.4, 56.0], [-134.4, 48.0]]]}</t>
         </is>
       </c>
       <c r="P281" t="inlineStr">
         <is>
-          <t>[{'max': '600.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2.5', 'min': '2.5'}]</t>
         </is>
       </c>
       <c r="Q281" t="inlineStr">
         <is>
-          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
-        </is>
-      </c>
-      <c r="R281" t="inlineStr"/>
+          <t>oxygen, inorganicCarbon, subSurfaceSalinity, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R281" t="inlineStr">
+        <is>
+          <t>10.21966/rrzq-yw32</t>
+        </is>
+      </c>
       <c r="S281" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/64WELpDV0tXYqOqiWFYNzMJdW4k1/-P0d5bTNUbXdaZiFm9zI</t>
         </is>
       </c>
       <c r="T281" t="inlineStr">
@@ -31260,11 +31266,17 @@
       </c>
       <c r="U281" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="V281" t="inlineStr"/>
-      <c r="W281" t="inlineStr"/>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="V281" t="n">
+        <v>0</v>
+      </c>
+      <c r="W281" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
       <c r="X281" t="inlineStr"/>
     </row>
     <row r="282">
@@ -31273,12 +31285,12 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
+          <t>c1e0447b-a06c-44c8-abd0-3108b2f00b7a</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
+          <t>ca-cioos_a787372d-e6f0-4128-bd08-7e9f5e667e1d</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
@@ -31288,17 +31300,17 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
+          <t>Discrete water chemistry measurements of the carbon dioxide system, nutrients, and organic carbon in fresh and marine waters of the Northeast Pacific coast of North America</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>collection</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>CC-BY-4.0</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H282" t="b">
@@ -31306,12 +31318,12 @@
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>Estuary Resilience</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>tentative</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K282" t="inlineStr">
@@ -31334,47 +31346,37 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.5, 43.3], [-121.8, 43.3], [-121.8, 62.0], [-153.5, 62.0], [-153.5, 43.3]]]}</t>
         </is>
       </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>[{'max': '100.0', 'min': '0.2'}]</t>
+          <t>[{'max': '600.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q282" t="inlineStr">
         <is>
-          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
-        </is>
-      </c>
-      <c r="R282" t="inlineStr">
-        <is>
-          <t>10.21966/r9zr-xz33</t>
-        </is>
-      </c>
+          <t>dissolvedOrganicCarbon, nitrousOxide, oxygen, stableCarbonIsotopes, inorganicCarbon, nutrients, particulateMatter, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceCurrents, subSurfaceTemperature</t>
+        </is>
+      </c>
+      <c r="R282" t="inlineStr"/>
       <c r="S282" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/3LY8ezYsI9hglwZSsfkAdSBcoEG3/-P0d-gfRwatFu4gaeuhY</t>
         </is>
       </c>
       <c r="T282" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="U282" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="V282" t="n">
-        <v>0</v>
-      </c>
-      <c r="W282" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="V282" t="inlineStr"/>
+      <c r="W282" t="inlineStr"/>
       <c r="X282" t="inlineStr"/>
     </row>
     <row r="283">
@@ -31383,12 +31385,12 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
+          <t>97677e6b-1d06-4466-8849-043df22984c1</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
+          <t>ca-cioos_05c75bd9-1953-4ab9-8573-878845854662</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
@@ -31398,7 +31400,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Glendale River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F283" t="inlineStr">
@@ -31444,7 +31446,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.72874, 50.69623], [-125.7357, 50.67697], [-125.73637, 50.66065], [-125.72893, 50.65255], [-125.71434, 50.64835], [-125.71329, 50.65188], [-125.72626, 50.65827], [-125.72636, 50.66466], [-125.72865, 50.68116], [-125.72721, 50.69604], [-125.72855, 50.69614], [-125.72874, 50.69623]]]}</t>
         </is>
       </c>
       <c r="P283" t="inlineStr">
@@ -31459,12 +31461,12 @@
       </c>
       <c r="R283" t="inlineStr">
         <is>
-          <t>10.21966/9dbb-5d54</t>
+          <t>10.21966/r9zr-xz33</t>
         </is>
       </c>
       <c r="S283" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7FmsNQ6HChfyLfTcX</t>
         </is>
       </c>
       <c r="T283" t="inlineStr">
@@ -31493,12 +31495,12 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
+          <t>c428c9ff-19ed-40ec-82e0-40ab10960364</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
+          <t>ca-cioos_0e50f5a3-6100-4f1a-b184-ba327def9f3a</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
@@ -31508,7 +31510,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kaouk River estuary (Provisional)</t>
         </is>
       </c>
       <c r="F284" t="inlineStr">
@@ -31554,7 +31556,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.15825, 50.07693], [-127.15157, 50.07806], [-127.13204, 50.06944], [-127.11152, 50.06781], [-127.0959, 50.06667], [-127.04315, 50.06879], [-127.04168, 50.06455], [-127.0902, 50.05983], [-127.10062, 50.05658], [-127.11983, 50.05885], [-127.13887, 50.06423], [-127.15988, 50.0753], [-127.15874, 50.07693], [-127.15825, 50.07693]]]}</t>
         </is>
       </c>
       <c r="P284" t="inlineStr">
@@ -31569,12 +31571,12 @@
       </c>
       <c r="R284" t="inlineStr">
         <is>
-          <t>10.21966/vpz7-mm73</t>
+          <t>10.21966/9dbb-5d54</t>
         </is>
       </c>
       <c r="S284" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq6X1wQRkybrW6sac5D</t>
         </is>
       </c>
       <c r="T284" t="inlineStr">
@@ -31603,12 +31605,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>0ce3ee5b-425b-4eb0-a201-96bdfb795a3f</t>
+          <t>2de5b0d2-71b1-4041-bd01-118e9c529dac</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>ca-cioos_354b5b83-e752-4ffb-a740-d1cdc02ac8c6</t>
+          <t>ca-cioos_2ba57f02-c88b-42b8-8f8c-07cfdeab45d3</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
@@ -31618,7 +31620,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Dtlaxsiwè River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kw'a'luxw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F285" t="inlineStr">
@@ -31664,7 +31666,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.1721, 50.61011], [-127.17933, 50.612], [-127.1873, 50.6098], [-127.19703, 50.61072], [-127.20524, 50.61585], [-127.19007, 50.61844], [-127.18675, 50.61393], [-127.17744, 50.61359], [-127.17161, 50.61118], [-127.17203, 50.61011], [-127.1721, 50.61011]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.29886, 49.3576], [-124.30659, 49.32057], [-124.28624, 49.31332], [-124.26557, 49.29566], [-124.26427, 49.29899], [-124.28624, 49.3283], [-124.29878, 49.35744], [-124.29886, 49.3576]]]}</t>
         </is>
       </c>
       <c r="P285" t="inlineStr">
@@ -31679,12 +31681,12 @@
       </c>
       <c r="R285" t="inlineStr">
         <is>
-          <t>10.21966/ydm2-m238</t>
+          <t>10.21966/vpz7-mm73</t>
         </is>
       </c>
       <c r="S285" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7Dng-ZtRd05hnZCq1</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptH1k-7T2gjAKY814I</t>
         </is>
       </c>
       <c r="T285" t="inlineStr">
@@ -31713,12 +31715,12 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>1a2aa5c8-9a83-46f7-967d-1127436c2084</t>
+          <t>0ce3ee5b-425b-4eb0-a201-96bdfb795a3f</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>ca-cioos_58a5140a-0b2c-4186-a648-53d9f58e5226</t>
+          <t>ca-cioos_354b5b83-e752-4ffb-a740-d1cdc02ac8c6</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
@@ -31728,7 +31730,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Kvai River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Dtlaxsiwè River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F286" t="inlineStr">
@@ -31774,7 +31776,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.81882, 51.77547], [-127.83122, 51.77986], [-127.85192, 51.781], [-127.86785, 51.78358], [-127.8958, 51.77366], [-127.89418, 51.77118], [-127.87834, 51.77309], [-127.86508, 51.77748], [-127.84009, 51.77519], [-127.82731, 51.77452], [-127.82025, 51.77309], [-127.81853, 51.77566], [-127.81882, 51.77547]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.1721, 50.61011], [-127.17933, 50.612], [-127.1873, 50.6098], [-127.19703, 50.61072], [-127.20524, 50.61585], [-127.19007, 50.61844], [-127.18675, 50.61393], [-127.17744, 50.61359], [-127.17161, 50.61118], [-127.17203, 50.61011], [-127.1721, 50.61011]]]}</t>
         </is>
       </c>
       <c r="P286" t="inlineStr">
@@ -31789,12 +31791,12 @@
       </c>
       <c r="R286" t="inlineStr">
         <is>
-          <t>10.21966/pm9m-h431</t>
+          <t>10.21966/ydm2-m238</t>
         </is>
       </c>
       <c r="S286" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7QQE3ifLCAPcu3Jih</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7Dng-ZtRd05hnZCq1</t>
         </is>
       </c>
       <c r="T286" t="inlineStr">
@@ -31823,12 +31825,12 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>c035b81c-0fc3-446e-bec5-8b8933ae874b</t>
+          <t>1a2aa5c8-9a83-46f7-967d-1127436c2084</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>ca-cioos_7fbc28f7-ee87-4361-bbee-0ed8ce24522d</t>
+          <t>ca-cioos_58a5140a-0b2c-4186-a648-53d9f58e5226</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
@@ -31838,7 +31840,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Gwa'dzi River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Kvai River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F287" t="inlineStr">
@@ -31884,7 +31886,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.46176, 50.74217], [-127.49022, 50.72165], [-127.49167, 50.71188], [-127.4832, 50.70356], [-127.4874, 50.69181], [-127.46443, 50.6928], [-127.47282, 50.70776], [-127.47992, 50.71424], [-127.48305, 50.72058], [-127.45901, 50.74011], [-127.46153, 50.74217], [-127.46176, 50.74217]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.81882, 51.77547], [-127.83122, 51.77986], [-127.85192, 51.781], [-127.86785, 51.78358], [-127.8958, 51.77366], [-127.89418, 51.77118], [-127.87834, 51.77309], [-127.86508, 51.77748], [-127.84009, 51.77519], [-127.82731, 51.77452], [-127.82025, 51.77309], [-127.81853, 51.77566], [-127.81882, 51.77547]]]}</t>
         </is>
       </c>
       <c r="P287" t="inlineStr">
@@ -31899,12 +31901,12 @@
       </c>
       <c r="R287" t="inlineStr">
         <is>
-          <t>10.21966/xq99-x273</t>
+          <t>10.21966/pm9m-h431</t>
         </is>
       </c>
       <c r="S287" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7BCRnF2C30YPkxIyd</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7QQE3ifLCAPcu3Jih</t>
         </is>
       </c>
       <c r="T287" t="inlineStr">
@@ -31933,12 +31935,12 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
+          <t>c035b81c-0fc3-446e-bec5-8b8933ae874b</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
+          <t>ca-cioos_7fbc28f7-ee87-4361-bbee-0ed8ce24522d</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
@@ -31948,7 +31950,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Gwa'dzi River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F288" t="inlineStr">
@@ -31994,7 +31996,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.46176, 50.74217], [-127.49022, 50.72165], [-127.49167, 50.71188], [-127.4832, 50.70356], [-127.4874, 50.69181], [-127.46443, 50.6928], [-127.47282, 50.70776], [-127.47992, 50.71424], [-127.48305, 50.72058], [-127.45901, 50.74011], [-127.46153, 50.74217], [-127.46176, 50.74217]]]}</t>
         </is>
       </c>
       <c r="P288" t="inlineStr">
@@ -32009,12 +32011,12 @@
       </c>
       <c r="R288" t="inlineStr">
         <is>
-          <t>10.21966/kde9-8g12</t>
+          <t>10.21966/xq99-x273</t>
         </is>
       </c>
       <c r="S288" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7BCRnF2C30YPkxIyd</t>
         </is>
       </c>
       <c r="T288" t="inlineStr">
@@ -32043,12 +32045,12 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
+          <t>ddf1f914-89b7-41fe-8e72-e5217476fc09</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
+          <t>ca-cioos_81883927-2334-45eb-b1c5-f6deb7add791</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
@@ -32058,7 +32060,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Conuma River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -32104,7 +32106,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.40799, 49.80074], [-126.43876, 49.78731], [-126.46497, 49.7786], [-126.46147, 49.79048], [-126.41255, 49.80261], [-126.40758, 49.80074], [-126.40799, 49.80074]]]}</t>
         </is>
       </c>
       <c r="P289" t="inlineStr">
@@ -32119,12 +32121,12 @@
       </c>
       <c r="R289" t="inlineStr">
         <is>
-          <t>10.21966/9a97-2j48</t>
+          <t>10.21966/kde9-8g12</t>
         </is>
       </c>
       <c r="S289" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpteQ8r8Ydn0LR9h4VG</t>
         </is>
       </c>
       <c r="T289" t="inlineStr">
@@ -32153,12 +32155,12 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
+          <t>5216f7f5-a569-4f76-9cab-171f1e847498</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
+          <t>ca-cioos_83a949b4-99be-4a36-a910-0c81946a9bf6</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
@@ -32168,7 +32170,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Muuyaḥi River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
@@ -32214,7 +32216,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.90617, 49.43155], [-125.91545, 49.42581], [-125.92033, 49.41507], [-125.9511, 49.38039], [-125.93437, 49.37197], [-125.89701, 49.41092], [-125.8986, 49.42679], [-125.90617, 49.43168], [-125.90617, 49.43155]]]}</t>
         </is>
       </c>
       <c r="P290" t="inlineStr">
@@ -32229,12 +32231,12 @@
       </c>
       <c r="R290" t="inlineStr">
         <is>
-          <t>10.21966/ed9w-2653</t>
+          <t>10.21966/9a97-2j48</t>
         </is>
       </c>
       <c r="S290" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptLdNw6_h2xTcYUjkS</t>
         </is>
       </c>
       <c r="T290" t="inlineStr">
@@ -32263,12 +32265,12 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>1af6a43a-e73b-4774-8e10-b9f2928ab133</t>
+          <t>1f4b5991-bbcb-416b-807c-ed8ca5f4d9f4</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>ca-cioos_ae7e017c-9211-4f98-b56e-90a4bbac161c</t>
+          <t>ca-cioos_86f1dd95-27a0-4c52-97e4-15be649ce73a</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
@@ -32278,7 +32280,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Snuneymuxw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Xwésam River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
@@ -32324,7 +32326,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.88685, 49.19332], [-123.92494, 49.1612], [-123.92581, 49.13841], [-123.91159, 49.123], [-123.88023, 49.11117], [-123.85971, 49.12766], [-123.89792, 49.16196], [-123.88099, 49.18866], [-123.88685, 49.19332]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.92043, 50.31848], [-125.94107, 50.31848], [-125.94046, 50.36243], [-125.9639, 50.38185], [-125.95731, 50.39906], [-125.94094, 50.38954], [-125.93716, 50.37831], [-125.91445, 50.37257], [-125.91994, 50.31835], [-125.92043, 50.31848]]]}</t>
         </is>
       </c>
       <c r="P291" t="inlineStr">
@@ -32339,12 +32341,12 @@
       </c>
       <c r="R291" t="inlineStr">
         <is>
-          <t>10.21966/k01q-wb27</t>
+          <t>10.21966/ed9w-2653</t>
         </is>
       </c>
       <c r="S291" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt459vxCIH7YPRN9fp</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptUCw9y_sktWpuppc0</t>
         </is>
       </c>
       <c r="T291" t="inlineStr">
@@ -32373,12 +32375,12 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
+          <t>1af6a43a-e73b-4774-8e10-b9f2928ab133</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
+          <t>ca-cioos_ae7e017c-9211-4f98-b56e-90a4bbac161c</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
@@ -32388,7 +32390,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Snuneymuxw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
@@ -32434,7 +32436,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635], [-123.66843, 48.91641]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.88685, 49.19332], [-123.92494, 49.1612], [-123.92581, 49.13841], [-123.91159, 49.123], [-123.88023, 49.11117], [-123.85971, 49.12766], [-123.89792, 49.16196], [-123.88099, 49.18866], [-123.88685, 49.19332]]]}</t>
         </is>
       </c>
       <c r="P292" t="inlineStr">
@@ -32449,12 +32451,12 @@
       </c>
       <c r="R292" t="inlineStr">
         <is>
-          <t>10.21966/q2e0-j004</t>
+          <t>10.21966/k01q-wb27</t>
         </is>
       </c>
       <c r="S292" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt459vxCIH7YPRN9fp</t>
         </is>
       </c>
       <c r="T292" t="inlineStr">
@@ -32483,12 +32485,12 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
+          <t>b7638e0b-e734-4a96-97af-9e7729b61831</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
+          <t>ca-cioos_bea3da72-dafe-4e25-b5b2-0176e0ffba44</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
@@ -32498,7 +32500,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Chemainus River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
@@ -32544,7 +32546,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.66843, 48.91641], [-123.6484, 48.90105], [-123.6554, 48.88016], [-123.6751, 48.87641], [-123.68894, 48.88178], [-123.68329, 48.89633], [-123.67928, 48.90316], [-123.67136, 48.91722], [-123.66848, 48.91635], [-123.66843, 48.91641]]]}</t>
         </is>
       </c>
       <c r="P293" t="inlineStr">
@@ -32559,12 +32561,12 @@
       </c>
       <c r="R293" t="inlineStr">
         <is>
-          <t>10.21966/hjkj-6611</t>
+          <t>10.21966/q2e0-j004</t>
         </is>
       </c>
       <c r="S293" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpszvIrt9OF8-BLQW2N</t>
         </is>
       </c>
       <c r="T293" t="inlineStr">
@@ -32593,12 +32595,12 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
+          <t>879a98f9-7e86-46dc-9449-e05cbf720b1e</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>ca-cioos_dce15b7b-3772-4106-ab20-c3979c4c3f57</t>
+          <t>ca-cioos_d6e2bb44-2cad-4008-8af8-268054f5dfc6</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
@@ -32608,7 +32610,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Fulmore River - Shoal Creek Estuary Complex (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Asiixw River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -32654,7 +32656,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.08798, 50.4777], [-126.09599, 50.48418], [-126.09046, 50.50918], [-126.0647, 50.52425], [-125.99698, 50.53569], [-125.93459, 50.56717], [-125.93173, 50.56202], [-125.93764, 50.55458], [-125.91055, 50.55134], [-125.89853, 50.54943], [-125.90063, 50.54466], [-125.96416, 50.53989], [-125.98973, 50.52043], [-126.06566, 50.5067], [-126.08779, 50.47789], [-126.08798, 50.4777]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.67758, 51.98241], [-126.67797, 51.9818], [-126.67794, 51.97239], [-126.67998, 51.96699], [-126.68252, 51.95773], [-126.67601, 51.95751], [-126.67021, 51.95869], [-126.66832, 51.96062], [-126.67093, 51.96366], [-126.67565, 51.96617], [-126.67379, 51.97286], [-126.67744, 51.98251], [-126.67758, 51.98241]]]}</t>
         </is>
       </c>
       <c r="P294" t="inlineStr">
@@ -32669,12 +32671,12 @@
       </c>
       <c r="R294" t="inlineStr">
         <is>
-          <t>10.21966/g1cn-xs92</t>
+          <t>10.21966/hjkj-6611</t>
         </is>
       </c>
       <c r="S294" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptdJ8iUmLeOrdmqzrQ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq7XYdY4GReTVYPK2zz</t>
         </is>
       </c>
       <c r="T294" t="inlineStr">
@@ -32703,12 +32705,12 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
+          <t>4c7b7347-767d-45e4-b3ad-7e0133b31e1c</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
+          <t>ca-cioos_dce15b7b-3772-4106-ab20-c3979c4c3f57</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
@@ -32718,7 +32720,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Fulmore River - Shoal Creek Estuary Complex (Provisional)</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
@@ -32764,7 +32766,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.08798, 50.4777], [-126.09599, 50.48418], [-126.09046, 50.50918], [-126.0647, 50.52425], [-125.99698, 50.53569], [-125.93459, 50.56717], [-125.93173, 50.56202], [-125.93764, 50.55458], [-125.91055, 50.55134], [-125.89853, 50.54943], [-125.90063, 50.54466], [-125.96416, 50.53989], [-125.98973, 50.52043], [-126.06566, 50.5067], [-126.08779, 50.47789], [-126.08798, 50.4777]]]}</t>
         </is>
       </c>
       <c r="P295" t="inlineStr">
@@ -32779,12 +32781,12 @@
       </c>
       <c r="R295" t="inlineStr">
         <is>
-          <t>10.21966/npe4-3036</t>
+          <t>10.21966/g1cn-xs92</t>
         </is>
       </c>
       <c r="S295" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptdJ8iUmLeOrdmqzrQ</t>
         </is>
       </c>
       <c r="T295" t="inlineStr">
@@ -32813,12 +32815,12 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
+          <t>8dadb6a8-8eb2-44ea-9d2d-c4332e4c544b</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>ca-cioos_e9b72149-8cf1-4000-ae3e-6b29ad60b078</t>
+          <t>ca-cioos_dfb93c87-300e-4843-91f9-7c51bc59422e</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
@@ -32828,7 +32830,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Malksope River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Little Qualicum River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -32874,7 +32876,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.46569, 50.12556], [-127.45723, 50.13142], [-127.43281, 50.13338], [-127.42845, 50.13765], [-127.41181, 50.14408], [-127.40973, 50.14233], [-127.41999, 50.13627], [-127.41803, 50.13195], [-127.43106, 50.12796], [-127.46545, 50.12446], [-127.46569, 50.12548], [-127.46569, 50.12556]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-124.50281, 49.36977], [-124.50159, 49.36509], [-124.49039, 49.36183], [-124.484, 49.35439], [-124.48233, 49.35536], [-124.49153, 49.36749], [-124.50289, 49.36977], [-124.50281, 49.36977]]]}</t>
         </is>
       </c>
       <c r="P296" t="inlineStr">
@@ -32889,12 +32891,12 @@
       </c>
       <c r="R296" t="inlineStr">
         <is>
-          <t>10.21966/21sf-ey03</t>
+          <t>10.21966/npe4-3036</t>
         </is>
       </c>
       <c r="S296" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq77iyWJfPg4z-FvOSb</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Opt2a41JCjjQCuqrK6m</t>
         </is>
       </c>
       <c r="T296" t="inlineStr">
@@ -32923,12 +32925,12 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>5177d019-598e-4415-b778-9688403652c8</t>
+          <t>35245eae-e508-47da-bcf7-54346cda086a</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>ca-cioos_ed84df74-5a2d-4a7d-87c8-a7b93f11088e</t>
+          <t>ca-cioos_e9b72149-8cf1-4000-ae3e-6b29ad60b078</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
@@ -32938,7 +32940,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Nalaxdlala River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Malksope River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -32984,7 +32986,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-125.9489, 50.70902], [-125.9696, 50.70291], [-126.00938, 50.69118], [-126.00108, 50.66848], [-125.98257, 50.68374], [-125.98152, 50.69271], [-125.95462, 50.70263], [-125.94785, 50.70768], [-125.9489, 50.70911], [-125.9489, 50.70902]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.46569, 50.12556], [-127.45723, 50.13142], [-127.43281, 50.13338], [-127.42845, 50.13765], [-127.41181, 50.14408], [-127.40973, 50.14233], [-127.41999, 50.13627], [-127.41803, 50.13195], [-127.43106, 50.12796], [-127.46545, 50.12446], [-127.46569, 50.12548], [-127.46569, 50.12556]]]}</t>
         </is>
       </c>
       <c r="P297" t="inlineStr">
@@ -32999,12 +33001,12 @@
       </c>
       <c r="R297" t="inlineStr">
         <is>
-          <t>10.21966/4krv-aw23</t>
+          <t>10.21966/21sf-ey03</t>
         </is>
       </c>
       <c r="S297" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptbxmpkBsfyWWfSxOJ</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-Oq77iyWJfPg4z-FvOSb</t>
         </is>
       </c>
       <c r="T297" t="inlineStr">
@@ -33033,12 +33035,12 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
+          <t>5177d019-598e-4415-b778-9688403652c8</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>ca-cioos_b922699f-69b6-4d63-b538-7c290086a408</t>
+          <t>ca-cioos_ed84df74-5a2d-4a7d-87c8-a7b93f11088e</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
@@ -33048,7 +33050,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>BC Estuary Water Quality Monitoring Data - Quw'utsun/Xwulqw'selu River Estuary (Provisional)</t>
+          <t>BC Estuary Water Quality Monitoring Data - Nalaxdlala River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
@@ -33094,7 +33096,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-123.56201, 48.73508], [-123.59772, 48.75559], [-123.62127, 48.76514], [-123.63885, 48.77426], [-123.66935, 48.78033], [-123.67901, 48.75472], [-123.65155, 48.74322], [-123.63017, 48.7405], [-123.60792, 48.74289], [-123.56494, 48.72987], [-123.56179, 48.73529], [-123.56201, 48.73508]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-125.9489, 50.70902], [-125.9696, 50.70291], [-126.00938, 50.69118], [-126.00108, 50.66848], [-125.98257, 50.68374], [-125.98152, 50.69271], [-125.95462, 50.70263], [-125.94785, 50.70768], [-125.9489, 50.70911], [-125.9489, 50.70902]]]}</t>
         </is>
       </c>
       <c r="P298" t="inlineStr">
@@ -33109,17 +33111,17 @@
       </c>
       <c r="R298" t="inlineStr">
         <is>
-          <t>10.21966/2ha7-9p26</t>
+          <t>10.21966/4krv-aw23</t>
         </is>
       </c>
       <c r="S298" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpsCA3ycwZ7bFTDIQxh</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OptbxmpkBsfyWWfSxOJ</t>
         </is>
       </c>
       <c r="T298" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="U298" t="inlineStr">
@@ -33143,12 +33145,12 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>dd471e82-a6b8-4f32-891c-bbea26e9998e</t>
+          <t>d320d90e-96bf-4993-81c5-f1f57886b0e6</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>ca-cioos_aeb30028-a7eb-462e-ac0f-6c5fe101d4a2</t>
+          <t>ca-cioos_b922699f-69b6-4d63-b538-7c290086a408</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
@@ -33158,7 +33160,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>DNA Metabarcoding Captures Temporal and Vertical Dynamics of Mesozooplankton Communities</t>
+          <t>BC Estuary Water Quality Monitoring Data - Quw'utsun/Xwulqw'selu River Estuary (Provisional)</t>
         </is>
       </c>
       <c r="F299" t="inlineStr">
@@ -33176,12 +33178,12 @@
       </c>
       <c r="I299" t="inlineStr">
         <is>
-          <t>Genomics, Oceanography</t>
+          <t>Estuary Resilience</t>
         </is>
       </c>
       <c r="J299" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>tentative</t>
         </is>
       </c>
       <c r="K299" t="inlineStr">
@@ -33196,45 +33198,45 @@
       </c>
       <c r="M299" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Hakai Institute</t>
         </is>
       </c>
       <c r="N299" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>{'type': 'Point', 'coordinates': [-125.0992, 50.0307]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-123.56201, 48.73508], [-123.59772, 48.75559], [-123.62127, 48.76514], [-123.63885, 48.77426], [-123.66935, 48.78033], [-123.67901, 48.75472], [-123.65155, 48.74322], [-123.63017, 48.7405], [-123.60792, 48.74289], [-123.56494, 48.72987], [-123.56179, 48.73529], [-123.56201, 48.73508]]]}</t>
         </is>
       </c>
       <c r="P299" t="inlineStr">
         <is>
-          <t>[{'max': '260.0', 'min': '0.0'}]</t>
+          <t>[{'max': '100.0', 'min': '0.2'}]</t>
         </is>
       </c>
       <c r="Q299" t="inlineStr">
         <is>
-          <t>zooplanktonBiomassAndDiversity</t>
+          <t>other, seaSurfaceTemperature, subSurfaceSalinity, seaSurfaceSalinity, subSurfaceTemperature, oxygen</t>
         </is>
       </c>
       <c r="R299" t="inlineStr">
         <is>
-          <t>10.21966/6b20-7r76</t>
+          <t>10.21966/2ha7-9p26</t>
         </is>
       </c>
       <c r="S299" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-OvzbmseH_syBXg1RXKd</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/mALzxHvoyRXof5FCVKOlOJC585n1/-OpsCA3ycwZ7bFTDIQxh</t>
         </is>
       </c>
       <c r="T299" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="U299" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="V299" t="n">
@@ -33363,12 +33365,12 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>d269f354-8527-4e94-bb32-9de4fe3fabdf</t>
+          <t>098c52a1-6dde-4e64-8b27-5a34e40870e6</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>ca-cioos_da232383-781d-4852-8542-cf0cb8aa5f26</t>
+          <t>ca-cioos_e5e61f93-db9b-48d0-b779-45e73fabfd0a</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
@@ -33378,17 +33380,17 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Data for Paper: Detection differences between eDNA and mid-water trawls are driven by fish biomass and habitat preferences</t>
+          <t>High Resolution Coastal Carbon Monitoring in the Northeast Pacific</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>dataset</t>
+          <t>collection</t>
         </is>
       </c>
       <c r="G301" t="inlineStr">
         <is>
-          <t>CC-BY-NC-ND-4.0</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H301" t="b">
@@ -33396,12 +33398,12 @@
       </c>
       <c r="I301" t="inlineStr">
         <is>
-          <t>Genomics</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
@@ -33420,31 +33422,27 @@
         </is>
       </c>
       <c r="N301" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-126.6289, 50.7424], [-127.321, 50.6868], [-124.8052, 48.3262], [-123.2452, 48.1432], [-122.9596, 49.0945], [-126.6289, 50.7424]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-160.4964, 46.7847], [-118.6667, 46.7847], [-118.6667, 62.7421], [-160.4964, 62.7421], [-160.4964, 46.7847]]]}</t>
         </is>
       </c>
       <c r="P301" t="inlineStr">
         <is>
-          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0', 'min': '0'}]</t>
         </is>
       </c>
       <c r="Q301" t="inlineStr">
         <is>
-          <t>fishAbundanceAndDistribution</t>
-        </is>
-      </c>
-      <c r="R301" t="inlineStr">
-        <is>
-          <t>10.21966/hky6-1022</t>
-        </is>
-      </c>
+          <t>inorganicCarbon</t>
+        </is>
+      </c>
+      <c r="R301" t="inlineStr"/>
       <c r="S301" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-P1l_Wv09HnWD1is-Yik</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-P0csr75piiewsICpJu8</t>
         </is>
       </c>
       <c r="T301" t="inlineStr">
@@ -33454,17 +33452,11 @@
       </c>
       <c r="U301" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="V301" t="n">
-        <v>0</v>
-      </c>
-      <c r="W301" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="V301" t="inlineStr"/>
+      <c r="W301" t="inlineStr"/>
       <c r="X301" t="inlineStr"/>
     </row>
     <row r="302">
@@ -33473,12 +33465,12 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>098c52a1-6dde-4e64-8b27-5a34e40870e6</t>
+          <t>d269f354-8527-4e94-bb32-9de4fe3fabdf</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>ca-cioos_e5e61f93-db9b-48d0-b779-45e73fabfd0a</t>
+          <t>ca-cioos_da232383-781d-4852-8542-cf0cb8aa5f26</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
@@ -33488,17 +33480,17 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>High Resolution Coastal Carbon Monitoring in the Northeast Pacific</t>
+          <t>Data for Paper: Detection differences between eDNA and mid-water trawls are driven by fish biomass and habitat preferences</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>collection</t>
+          <t>dataset</t>
         </is>
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>CC-BY-NC-ND-4.0</t>
         </is>
       </c>
       <c r="H302" t="b">
@@ -33506,12 +33498,12 @@
       </c>
       <c r="I302" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Genomics</t>
         </is>
       </c>
       <c r="J302" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K302" t="inlineStr">
@@ -33530,42 +33522,54 @@
         </is>
       </c>
       <c r="N302" t="n">
+        <v>3</v>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>{'type': 'Polygon', 'coordinates': [[[-126.6289, 50.7424], [-127.321, 50.6868], [-124.8052, 48.3262], [-123.2452, 48.1432], [-122.9596, 49.0945], [-126.6289, 50.7424]]]}</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>[{'max': '20.0', 'min': '0.0'}]</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>fishAbundanceAndDistribution</t>
+        </is>
+      </c>
+      <c r="R302" t="inlineStr">
+        <is>
+          <t>10.21966/hky6-1022</t>
+        </is>
+      </c>
+      <c r="S302" t="inlineStr">
+        <is>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/jnK2pbrIzbMBHpSiUOi8XDUeev93/-P1l_Wv09HnWD1is-Yik</t>
+        </is>
+      </c>
+      <c r="T302" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="U302" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="V302" t="n">
+        <v>0</v>
+      </c>
+      <c r="W302" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="X302" t="n">
         <v>1</v>
       </c>
-      <c r="O302" t="inlineStr">
-        <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-160.4964, 46.7847], [-118.6667, 46.7847], [-118.6667, 62.7421], [-160.4964, 62.7421], [-160.4964, 46.7847]]]}</t>
-        </is>
-      </c>
-      <c r="P302" t="inlineStr">
-        <is>
-          <t>[{'max': '0', 'min': '0'}]</t>
-        </is>
-      </c>
-      <c r="Q302" t="inlineStr">
-        <is>
-          <t>inorganicCarbon</t>
-        </is>
-      </c>
-      <c r="R302" t="inlineStr"/>
-      <c r="S302" t="inlineStr">
-        <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RLSJmX44tkZoh8ncSpZECUoikBt1/-P0csr75piiewsICpJu8</t>
-        </is>
-      </c>
-      <c r="T302" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="U302" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="V302" t="inlineStr"/>
-      <c r="W302" t="inlineStr"/>
-      <c r="X302" t="inlineStr"/>
     </row>
     <row r="303">
       <c r="A303" t="n">
@@ -33787,7 +33791,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X304" t="inlineStr"/>
+      <c r="X304" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="n">
@@ -33997,7 +34003,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X306" t="inlineStr"/>
+      <c r="X306" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="n">

</xml_diff>

<commit_message>
Deployed d2600fcbc to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -3685,9 +3685,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X30" t="n">
-        <v>1</v>
-      </c>
+      <c r="X30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -6005,12 +6003,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6020,7 +6018,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6066,7 +6064,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -6076,17 +6074,17 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
@@ -6096,7 +6094,7 @@
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V52" t="n">
@@ -6115,12 +6113,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6130,7 +6128,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6176,7 +6174,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6186,17 +6184,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6206,7 +6204,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -8965,12 +8963,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
+          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
+          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8980,7 +8978,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
+          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -8998,7 +8996,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>Geospatial, Airborne Coastal Observatory</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -9026,12 +9024,12 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
         </is>
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>[{'max': '500.0', 'min': '0.0'}]</t>
+          <t>[{'max': '150.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr">
@@ -9041,12 +9039,12 @@
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>10.21966/eysg-7a26</t>
+          <t>10.21966/wfcv-n753</t>
         </is>
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
         </is>
       </c>
       <c r="T79" t="inlineStr">
@@ -9075,12 +9073,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>281d7444-efa6-4b18-ac0a-55c8f8b484be</t>
+          <t>a8d40002-d393-40da-882c-73c0ad8ca7e6</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ca-cioos_c3958106-fc49-44bd-8227-bfc3e8bcb58c</t>
+          <t>ca-cioos_c3eff62f-bcee-4faa-a7e1-7b9380d94e74</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -9090,7 +9088,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Moore Island Archaeology Survey - 2019 - Airborne Coastal Observatory</t>
+          <t>Ancient Forest Wetlands, BC - Upper Fraser River - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -9108,7 +9106,7 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Geospatial, Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J80" t="inlineStr">
@@ -9136,12 +9134,12 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-129.5, 52.65], [-129.4, 52.65], [-129.4, 52.7], [-129.5, 52.7], [-129.5, 52.65]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-121.3, 53.79], [-121.2, 53.79], [-121.2, 53.84], [-121.3, 53.84], [-121.3, 53.79]]]}</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>[{'max': '150.0', 'min': '0.0'}]</t>
+          <t>[{'max': '500.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -9151,12 +9149,12 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>10.21966/wfcv-n753</t>
+          <t>10.21966/eysg-7a26</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6MBp3WwVTVbFK-0kv</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-Mj6RrLonwFgP-TX9bPv</t>
         </is>
       </c>
       <c r="T80" t="inlineStr">
@@ -12925,12 +12923,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -12940,7 +12938,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -12963,7 +12961,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -12982,11 +12980,11 @@
         </is>
       </c>
       <c r="N115" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
@@ -13001,12 +12999,12 @@
       </c>
       <c r="R115" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S115" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T115" t="inlineStr">
@@ -13016,7 +13014,7 @@
       </c>
       <c r="U115" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V115" t="n">
@@ -13024,7 +13022,7 @@
       </c>
       <c r="W115" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X115" t="inlineStr"/>
@@ -13035,12 +13033,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -13050,7 +13048,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -13073,7 +13071,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -13092,11 +13090,11 @@
         </is>
       </c>
       <c r="N116" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -13111,12 +13109,12 @@
       </c>
       <c r="R116" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T116" t="inlineStr">
@@ -13126,7 +13124,7 @@
       </c>
       <c r="U116" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V116" t="n">
@@ -13134,7 +13132,7 @@
       </c>
       <c r="W116" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X116" t="inlineStr"/>
@@ -15007,9 +15005,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X133" t="n">
-        <v>1</v>
-      </c>
+      <c r="X133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -16331,9 +16327,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X145" t="n">
-        <v>1</v>
-      </c>
+      <c r="X145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -18533,9 +18527,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X165" t="n">
-        <v>1</v>
-      </c>
+      <c r="X165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -19305,7 +19297,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X172" t="inlineStr"/>
+      <c r="X172" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -20515,9 +20509,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X183" t="n">
-        <v>1</v>
-      </c>
+      <c r="X183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -23149,9 +23141,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X207" t="n">
-        <v>1</v>
-      </c>
+      <c r="X207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="n">

</xml_diff>

<commit_message>
Deployed 4ab8a8ed2 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5775,7 +5775,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X49" t="inlineStr"/>
+      <c r="X49" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -6003,12 +6005,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6018,7 +6020,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6064,7 +6066,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -6074,17 +6076,17 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
@@ -6094,7 +6096,7 @@
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V52" t="n">
@@ -6113,12 +6115,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6128,7 +6130,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6174,7 +6176,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6184,17 +6186,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6204,7 +6206,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -13905,7 +13907,9 @@
           <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X123" t="inlineStr"/>
+      <c r="X123" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -14903,12 +14907,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -14918,7 +14922,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14936,7 +14940,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -14956,20 +14960,20 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
@@ -14979,12 +14983,12 @@
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -14994,7 +14998,7 @@
       </c>
       <c r="U133" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V133" t="n">
@@ -15005,9 +15009,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X133" t="n">
-        <v>1</v>
-      </c>
+      <c r="X133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -15015,12 +15017,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -15030,7 +15032,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -15048,7 +15050,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -15068,20 +15070,20 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N134" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -15091,12 +15093,12 @@
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -15106,7 +15108,7 @@
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V134" t="n">
@@ -16329,9 +16331,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X145" t="n">
-        <v>1</v>
-      </c>
+      <c r="X145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -24801,7 +24801,9 @@
           <t>[{'year': '2026', 'total': 2}]</t>
         </is>
       </c>
-      <c r="X222" t="inlineStr"/>
+      <c r="X222" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -25791,9 +25793,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X231" t="n">
-        <v>1</v>
-      </c>
+      <c r="X231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -34221,9 +34221,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X308" t="n">
-        <v>1</v>
-      </c>
+      <c r="X308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="n">

</xml_diff>

<commit_message>
Deployed bc0b32fac to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -6003,12 +6003,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6018,7 +6018,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -6074,17 +6074,17 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V52" t="n">
@@ -6113,12 +6113,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6128,7 +6128,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6184,17 +6184,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6204,7 +6204,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -14353,12 +14353,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
+          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
+          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -14368,7 +14368,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
+          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -14386,7 +14386,7 @@
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t>Genomics, Watersheds</t>
+          <t>Watersheds, Oceanography</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
@@ -14406,7 +14406,7 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>University of British Columbia</t>
+          <t>Skeena Fisheries Commission</t>
         </is>
       </c>
       <c r="N128" t="n">
@@ -14414,27 +14414,27 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>[{'max': '0.0', 'min': '0.0'}]</t>
+          <t>[{'max': '5.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R128" t="inlineStr">
         <is>
-          <t>10.21966/1.715630</t>
+          <t>10.21966/66x5-a210</t>
         </is>
       </c>
       <c r="S128" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
         </is>
       </c>
       <c r="T128" t="inlineStr">
@@ -14444,7 +14444,7 @@
       </c>
       <c r="U128" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="V128" t="n">
@@ -14463,12 +14463,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>41e0fbeb-9e27-429c-84ea-7bb1be3f2a0d</t>
+          <t>9a930f50-82e2-4d7c-9686-6b551b9a458e</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ca-cioos_74f47ab6-a1ca-4aef-9115-cf2baaf87bef</t>
+          <t>ca-cioos_765d00bb-beec-486c-bd00-e27f972b7324</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -14478,7 +14478,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Dissolved and particulate organic carbon chemistry for freshwater and marine stations from 2014 through 2016 on Calvert and Hecate Islands, British Columbia, Canada</t>
+          <t>Microbial activity and carbon fluxes in rainforest soil – Tsunami Hill, Calvert Island – June 2015 - April 2016</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -14496,7 +14496,7 @@
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t>Watersheds, Oceanography</t>
+          <t>Genomics, Watersheds</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -14516,7 +14516,7 @@
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t>Skeena Fisheries Commission</t>
+          <t>University of British Columbia</t>
         </is>
       </c>
       <c r="N129" t="n">
@@ -14524,27 +14524,27 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.23772561, 51.55090182], [-127.87151456, 51.55090182], [-127.87151456, 51.75810598], [-128.23772561, 51.75810598], [-128.23772561, 51.55090182]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13650264, 51.64966999], [-128.12495841, 51.64966999], [-128.12495841, 51.65523482], [-128.13650264, 51.65523482], [-128.13650264, 51.64966999]]]}</t>
         </is>
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>[{'max': '5.0', 'min': '0.0'}]</t>
+          <t>[{'max': '0.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other</t>
         </is>
       </c>
       <c r="R129" t="inlineStr">
         <is>
-          <t>10.21966/66x5-a210</t>
+          <t>10.21966/1.715630</t>
         </is>
       </c>
       <c r="S129" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWFXb1lySHV6ZnY5ck0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUE0SHdBOUNiWjU5bFY</t>
         </is>
       </c>
       <c r="T129" t="inlineStr">
@@ -14554,7 +14554,7 @@
       </c>
       <c r="U129" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="V129" t="n">
@@ -15005,7 +15005,9 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X133" t="inlineStr"/>
+      <c r="X133" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">

</xml_diff>

<commit_message>
Deployed f5fd62e72 to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5343,12 +5343,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -5414,17 +5414,17 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V46" t="n">
@@ -5453,12 +5453,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5468,7 +5468,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -5529,12 +5529,12 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
@@ -5563,12 +5563,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5578,7 +5578,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5624,7 +5624,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5634,17 +5634,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5654,7 +5654,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -6003,12 +6003,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6018,7 +6018,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -6074,17 +6074,17 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V52" t="n">
@@ -6113,12 +6113,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6128,7 +6128,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6184,17 +6184,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6204,7 +6204,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -8303,12 +8303,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -8318,7 +8318,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -8360,16 +8360,16 @@
         </is>
       </c>
       <c r="N73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
@@ -8379,12 +8379,12 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T73" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="U73" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V73" t="n">
@@ -8413,12 +8413,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8428,7 +8428,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -8470,16 +8470,16 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -8489,12 +8489,12 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T74" t="inlineStr">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V74" t="n">
@@ -13905,7 +13905,9 @@
           <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X123" t="inlineStr"/>
+      <c r="X123" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -15005,9 +15007,7 @@
           <t>[]</t>
         </is>
       </c>
-      <c r="X133" t="n">
-        <v>1</v>
-      </c>
+      <c r="X133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -31269,7 +31269,9 @@
       </c>
       <c r="V281" t="inlineStr"/>
       <c r="W281" t="inlineStr"/>
-      <c r="X281" t="inlineStr"/>
+      <c r="X281" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="n">

</xml_diff>

<commit_message>
Deployed 2df2cbc8b to main with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/main/catalog_summary.xlsx
+++ b/main/catalog_summary.xlsx
@@ -5343,12 +5343,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
+          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
+          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
+          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -5376,7 +5376,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Nearshore</t>
+          <t>Oceanography</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
@@ -5404,7 +5404,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -5414,17 +5414,17 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>other, invertebrateAbundanceAndDistribution</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>10.21966/6zp4-ye07</t>
+          <t>10.21966/1.715784</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
         </is>
       </c>
       <c r="T46" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="V46" t="n">
@@ -5453,12 +5453,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
+          <t>f8f299be-a37e-43bf-9416-5ff59e664f65</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
+          <t>ca-cioos_1c9b7bcd-d3cc-4856-9428-df7abb2149f0</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -5468,7 +5468,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
+          <t>Mobile Invertebrate Rocky Intertidal Surveys - BC Central Coast - 2016-2018</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -5514,7 +5514,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.24596616, 51.41449798], [-127.75115224, 51.41449798], [-127.75115224, 51.74287494], [-128.24596616, 51.74287494], [-128.24596616, 51.41449798]]]}</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -5529,12 +5529,12 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>10.21966/zs6a-j496</t>
+          <t>10.21966/6zp4-ye07</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MURNVGtYRFppYzB6YWI</t>
         </is>
       </c>
       <c r="T47" t="inlineStr">
@@ -5563,12 +5563,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>1bba6c8a-b99c-4fbd-8eae-7c8b771a841d</t>
+          <t>f2f9c9d6-0385-4732-b7d5-acc6bbb2e83a</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ca-cioos_17396d02-88ff-4240-837b-5d3a45e70ea0</t>
+          <t>ca-cioos_2738ef2b-0c74-422d-a140-082e5f7b3793</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -5578,7 +5578,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Water column CO2 system measurements collected during the 2016 National Oceanic and Atmospheric Administration West Coast Ocean Acidification survey (NOAA WCOA2016) from California to British Columbia</t>
+          <t>Surfgrass Communities - Motile Invertebrate Surveys - BC Central Coast - 2018-2019</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -5596,7 +5596,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Oceanography</t>
+          <t>Nearshore</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -5624,7 +5624,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-131.40081275, 43.38978964], [-121.83893073, 43.38978964], [-121.83893073, 53.31525434], [-131.40081275, 53.31525434], [-131.40081275, 43.38978964]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.17701209, 51.62693395], [-128.1138407, 51.62693395], [-128.1138407, 51.67805576], [-128.17701209, 51.67805576], [-128.17701209, 51.62693395]]]}</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
@@ -5634,17 +5634,17 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, invertebrateAbundanceAndDistribution</t>
         </is>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>10.21966/1.715784</t>
+          <t>10.21966/zs6a-j496</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXM3TWYzcWNJZ2p1Nk0</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXd4OWhCMU42TmhvaFY</t>
         </is>
       </c>
       <c r="T48" t="inlineStr">
@@ -5654,7 +5654,7 @@
       </c>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -6003,12 +6003,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
+          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
+          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -6018,7 +6018,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
+          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -6064,7 +6064,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
@@ -6074,17 +6074,17 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>other, dissolvedOrganicCarbon</t>
+          <t>other, inorganicCarbon</t>
         </is>
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>10.21966/1.715793</t>
+          <t>10.21966/zxzr-e472</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
         </is>
       </c>
       <c r="T52" t="inlineStr">
@@ -6094,7 +6094,7 @@
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="V52" t="n">
@@ -6113,12 +6113,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2abe9ff4-76de-4221-9ca6-ec3403a56efa</t>
+          <t>6083b388-4d24-4ac3-9464-dfea94468203</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ca-cioos_6d779012-e236-4a03-b11a-a5915f0f4342</t>
+          <t>ca-cioos_6c0697e9-7776-4d36-8219-b21ce72fbcc9</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -6128,7 +6128,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Underway surface seawater and marine boundary layer observations made from the Alaska Marine Highway System M/V Columbia from October 2017 to October 2018</t>
+          <t>Surface water CO2 parameters collected by Alaskan citizens around the northern Gulf of Alaska from April 2015 to August 2017. Version 1.0.</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -6174,7 +6174,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-140.68082679, 46.98536693], [-119.96438849, 46.98536693], [-119.96438849, 59.31669647], [-140.68082679, 59.31669647], [-140.68082679, 46.98536693]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-153.45020164, 58.42955383], [-145.36907065, 58.42955383], [-145.36907065, 61.89059635], [-153.45020164, 61.89059635], [-153.45020164, 58.42955383]]]}</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
@@ -6184,17 +6184,17 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>other, inorganicCarbon</t>
+          <t>other, dissolvedOrganicCarbon</t>
         </is>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>10.21966/zxzr-e472</t>
+          <t>10.21966/1.715793</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MWdoaWlmcWF6VWhJWTk</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MXhoOWQwcFE2aUY3Q1M</t>
         </is>
       </c>
       <c r="T53" t="inlineStr">
@@ -6204,7 +6204,7 @@
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="V53" t="n">
@@ -8303,12 +8303,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -8318,7 +8318,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -8360,16 +8360,16 @@
         </is>
       </c>
       <c r="N73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
@@ -8379,12 +8379,12 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>10.21966/5rp3-3207</t>
+          <t>10.21966/awsk-my87</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T73" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="U73" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="V73" t="n">
@@ -8413,12 +8413,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8428,7 +8428,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -8470,16 +8470,16 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -8489,12 +8489,12 @@
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>10.21966/awsk-my87</t>
+          <t>10.21966/5rp3-3207</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T74" t="inlineStr">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="U74" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V74" t="n">
@@ -12923,12 +12923,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
+          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
+          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -12938,7 +12938,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
+          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -12961,7 +12961,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>completed</t>
+          <t>onGoing</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -12980,11 +12980,11 @@
         </is>
       </c>
       <c r="N115" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
         </is>
       </c>
       <c r="P115" t="inlineStr">
@@ -12999,12 +12999,12 @@
       </c>
       <c r="R115" t="inlineStr">
         <is>
-          <t>10.21966/zvwf-qn04</t>
+          <t>10.21966/XNH1-TP28</t>
         </is>
       </c>
       <c r="S115" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
         </is>
       </c>
       <c r="T115" t="inlineStr">
@@ -13014,7 +13014,7 @@
       </c>
       <c r="U115" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V115" t="n">
@@ -13022,7 +13022,7 @@
       </c>
       <c r="W115" t="inlineStr">
         <is>
-          <t>[{'year': '2025', 'total': 1}]</t>
+          <t>[{'year': '2022', 'total': 1}]</t>
         </is>
       </c>
       <c r="X115" t="inlineStr"/>
@@ -13033,12 +13033,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>55826c6b-772a-45b4-a869-b97a4774e232</t>
+          <t>67871f51-9f69-44f6-9206-747e4d2a1553</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ca-cioos_ef59cc12-5031-4c65-b379-7ca03ad76d34</t>
+          <t>ca-cioos_ed3c5cb4-e6b0-4c8a-808e-3583a9a6cfde</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -13048,7 +13048,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Precipitation time-series – Central Coast and Quadra Island – 2013 - 2019 Version 1.0</t>
+          <t>Observed stream flow from seven small coastal watersheds in British Columbia, Canada, Sept 2013 – April 2019</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -13071,7 +13071,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>onGoing</t>
+          <t>completed</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -13090,11 +13090,11 @@
         </is>
       </c>
       <c r="N116" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.35114344, 51.37506462], [-127.65170145, 51.37506462], [-127.65170145, 51.8069493], [-128.35114344, 51.8069493], [-128.35114344, 51.37506462]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13265424, 51.60936247], [-127.95907025, 51.60936247], [-127.95907025, 51.69558793], [-128.13265424, 51.69558793], [-128.13265424, 51.60936247]]]}</t>
         </is>
       </c>
       <c r="P116" t="inlineStr">
@@ -13109,12 +13109,12 @@
       </c>
       <c r="R116" t="inlineStr">
         <is>
-          <t>10.21966/XNH1-TP28</t>
+          <t>10.21966/zvwf-qn04</t>
         </is>
       </c>
       <c r="S116" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUh2UDc1YkRVdUxzOVc</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MU1zSkI4S24ySE1rMGI</t>
         </is>
       </c>
       <c r="T116" t="inlineStr">
@@ -13124,7 +13124,7 @@
       </c>
       <c r="U116" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V116" t="n">
@@ -13132,7 +13132,7 @@
       </c>
       <c r="W116" t="inlineStr">
         <is>
-          <t>[{'year': '2022', 'total': 1}]</t>
+          <t>[{'year': '2025', 'total': 1}]</t>
         </is>
       </c>
       <c r="X116" t="inlineStr"/>
@@ -13905,9 +13905,7 @@
           <t>[{'year': '2022', 'total': 2}, {'year': '2023', 'total': 1}]</t>
         </is>
       </c>
-      <c r="X123" t="n">
-        <v>1</v>
-      </c>
+      <c r="X123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -14905,12 +14903,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -14920,7 +14918,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -14938,7 +14936,7 @@
       </c>
       <c r="I133" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J133" t="inlineStr">
@@ -14958,20 +14956,20 @@
       </c>
       <c r="M133" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr">
@@ -14981,12 +14979,12 @@
       </c>
       <c r="R133" t="inlineStr">
         <is>
-          <t>10.21966/1.135248</t>
+          <t>10.21966/x6q2-me90</t>
         </is>
       </c>
       <c r="S133" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T133" t="inlineStr">
@@ -14996,7 +14994,7 @@
       </c>
       <c r="U133" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="V133" t="n">
@@ -15015,12 +15013,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -15030,7 +15028,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -15048,7 +15046,7 @@
       </c>
       <c r="I134" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J134" t="inlineStr">
@@ -15068,20 +15066,20 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N134" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -15091,12 +15089,12 @@
       </c>
       <c r="R134" t="inlineStr">
         <is>
-          <t>10.21966/x6q2-me90</t>
+          <t>10.21966/1.135248</t>
         </is>
       </c>
       <c r="S134" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T134" t="inlineStr">
@@ -15106,7 +15104,7 @@
       </c>
       <c r="U134" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="V134" t="n">
@@ -31269,9 +31267,7 @@
       </c>
       <c r="V281" t="inlineStr"/>
       <c r="W281" t="inlineStr"/>
-      <c r="X281" t="n">
-        <v>1</v>
-      </c>
+      <c r="X281" t="inlineStr"/>
     </row>
     <row r="282">
       <c r="A282" t="n">

</xml_diff>